<commit_message>
Site, schema, and narrative updates
- Drop Uganda columns from data/timeseries.csv (now 7 cols, global only)
- Per-country detail (DRC, Uganda) lives in country_breakdown.csv
- Add data/story.md narrative (Story so far + Latest update)
- Add data/declarations.csv with CDC + WHO declaration links per country
- Site: render story.md (inline markdown), declarations table, last-updated
  timestamp from Last-Modified header; remove Uganda-specific stat cards
  and table columns
- Pull doubling-time chart from publication path (data too provisional);
  render code retained for future re-enabling
- Update build_xlsx.py to new 7-column schema
- Update README and METHODOLOGY to match
</commit_message>
<xml_diff>
--- a/outputs/ebola_timeseries.xlsx
+++ b/outputs/ebola_timeseries.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I47"/>
+  <dimension ref="A1:G47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -487,10 +487,8 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
     <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="48" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -503,7 +501,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Global outbreak totals (all reporting countries). Compiled from WHO AFRO Sitrep, WHO DON, CDC, Africa CDC, BNO News. Uganda breakout in columns F-G.</t>
+          <t>Global outbreak totals (all reporting countries). Compiled from WHO AFRO Sitrep, WHO DON, CDC, Africa CDC, BNO News. Per-country detail in the Country Breakdown sheet.</t>
         </is>
       </c>
     </row>
@@ -539,20 +537,10 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Uganda Confirmed</t>
+          <t>Primary Source</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Uganda Deaths</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>Primary Source</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Source Timestamp</t>
         </is>
@@ -576,18 +564,12 @@
       <c r="E5" s="4" t="n">
         <v>80</v>
       </c>
-      <c r="F5" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" s="5" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>BNO / WHO DON / DRC MoH declaration</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>2026-05-15</t>
         </is>
@@ -611,18 +593,12 @@
       <c r="E6" s="6" t="n">
         <v>87</v>
       </c>
-      <c r="F6" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="G6" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H6" s="7" t="inlineStr">
+      <c r="F6" s="7" t="inlineStr">
         <is>
           <t>BNO News (May 16) / Africa CDC</t>
         </is>
       </c>
-      <c r="I6" s="7" t="inlineStr">
+      <c r="G6" s="7" t="inlineStr">
         <is>
           <t>2026-05-16</t>
         </is>
@@ -646,18 +622,12 @@
       <c r="E7" s="4" t="n">
         <v>87</v>
       </c>
-      <c r="F7" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G7" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H7" s="5" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>BNO News (May 17) / WHO PHEIC declaration</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>2026-05-17</t>
         </is>
@@ -681,18 +651,12 @@
       <c r="E8" s="6" t="n">
         <v>132</v>
       </c>
-      <c r="F8" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="G8" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H8" s="7" t="inlineStr">
+      <c r="F8" s="7" t="inlineStr">
         <is>
           <t>WHO AFRO Weekly Sitrep 01 (as of 18 May) + BNO News for confirmed</t>
         </is>
       </c>
-      <c r="I8" s="7" t="inlineStr">
+      <c r="G8" s="7" t="inlineStr">
         <is>
           <t>2026-05-18</t>
         </is>
@@ -716,18 +680,12 @@
       <c r="E9" s="4" t="n">
         <v>131</v>
       </c>
-      <c r="F9" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G9" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>WHO / Wikipedia summary of WHO data</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>2026-05-19</t>
         </is>
@@ -751,18 +709,12 @@
       <c r="E10" s="6" t="n">
         <v>139</v>
       </c>
-      <c r="F10" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="G10" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H10" s="7" t="inlineStr">
+      <c r="F10" s="7" t="inlineStr">
         <is>
           <t>BNO News (May 20) / WHO Director-General briefing</t>
         </is>
       </c>
-      <c r="I10" s="7" t="inlineStr">
+      <c r="G10" s="7" t="inlineStr">
         <is>
           <t>2026-05-20</t>
         </is>
@@ -786,18 +738,12 @@
       <c r="E11" s="4" t="n">
         <v>176</v>
       </c>
-      <c r="F11" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G11" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>WHO DON603 (data as of 21 May, pub. 22 May)</t>
         </is>
       </c>
-      <c r="I11" s="5" t="inlineStr">
+      <c r="G11" s="5" t="inlineStr">
         <is>
           <t>2026-05-21</t>
         </is>
@@ -821,18 +767,12 @@
       <c r="E12" s="6" t="n">
         <v>176</v>
       </c>
-      <c r="F12" s="6" t="n">
-        <v>2</v>
-      </c>
-      <c r="G12" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H12" s="7" t="inlineStr">
+      <c r="F12" s="7" t="inlineStr">
         <is>
           <t>CDC Situation Summary (May 22)</t>
         </is>
       </c>
-      <c r="I12" s="7" t="inlineStr">
+      <c r="G12" s="7" t="inlineStr">
         <is>
           <t>2026-05-22</t>
         </is>
@@ -856,18 +796,12 @@
       <c r="E13" s="4" t="n">
         <v>177</v>
       </c>
-      <c r="F13" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="G13" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="F13" s="5" t="inlineStr">
         <is>
           <t>WHO Tedros briefing (May 22, via CIDRAP/ABC) + Uganda MoH (May 23, +3 cases)</t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr">
+      <c r="G13" s="5" t="inlineStr">
         <is>
           <t>2026-05-23</t>
         </is>
@@ -891,18 +825,12 @@
       <c r="E14" s="6" t="n">
         <v>220</v>
       </c>
-      <c r="F14" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="G14" s="6" t="n">
-        <v>1</v>
-      </c>
-      <c r="H14" s="7" t="inlineStr">
+      <c r="F14" s="7" t="inlineStr">
         <is>
           <t>DRC govt figures (Sunday May 24, via Reuters/AP/UN News/CNN) for cases; WHO DG Tedros (May 25 remarks) for suspected deaths ('at least 220'); no-dip rule applied</t>
         </is>
       </c>
-      <c r="I14" s="7" t="inlineStr">
+      <c r="G14" s="7" t="inlineStr">
         <is>
           <t>2026-05-24</t>
         </is>
@@ -926,18 +854,12 @@
       <c r="E15" s="4" t="n">
         <v>220</v>
       </c>
-      <c r="F15" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="G15" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="F15" s="5" t="inlineStr">
         <is>
           <t>Uganda MoH (May 25): +2 confirmed (Kampala health workers); DRC cases carry Sunday May 24 govt figures (Reuters/AP); WHO DG Tedros (May 25 remarks) for suspected deaths ('at least 220'); no-dip rule applied</t>
         </is>
       </c>
-      <c r="I15" s="5" t="inlineStr">
+      <c r="G15" s="5" t="inlineStr">
         <is>
           <t>2026-05-25</t>
         </is>
@@ -1162,38 +1084,38 @@
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="A25:I25"/>
-    <mergeCell ref="A41:I41"/>
-    <mergeCell ref="A37:I37"/>
-    <mergeCell ref="A46:I46"/>
-    <mergeCell ref="A18:I18"/>
-    <mergeCell ref="A27:I27"/>
-    <mergeCell ref="A26:I26"/>
-    <mergeCell ref="A21:I21"/>
-    <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A33:I33"/>
-    <mergeCell ref="A47:I47"/>
-    <mergeCell ref="A42:I42"/>
-    <mergeCell ref="A32:I32"/>
-    <mergeCell ref="A23:I23"/>
-    <mergeCell ref="A22:I22"/>
-    <mergeCell ref="A35:I35"/>
-    <mergeCell ref="A20:I20"/>
-    <mergeCell ref="A38:I38"/>
-    <mergeCell ref="A29:I29"/>
-    <mergeCell ref="A43:I43"/>
-    <mergeCell ref="A19:I19"/>
-    <mergeCell ref="A28:I28"/>
-    <mergeCell ref="A44:I44"/>
-    <mergeCell ref="A40:I40"/>
-    <mergeCell ref="A31:I31"/>
-    <mergeCell ref="A39:I39"/>
-    <mergeCell ref="A34:I34"/>
-    <mergeCell ref="A24:I24"/>
-    <mergeCell ref="A30:I30"/>
-    <mergeCell ref="A36:I36"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A45:I45"/>
+    <mergeCell ref="A32:G32"/>
+    <mergeCell ref="A22:G22"/>
+    <mergeCell ref="A35:G35"/>
+    <mergeCell ref="A20:G20"/>
+    <mergeCell ref="A38:G38"/>
+    <mergeCell ref="A29:G29"/>
+    <mergeCell ref="A43:G43"/>
+    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="A28:G28"/>
+    <mergeCell ref="A44:G44"/>
+    <mergeCell ref="A40:G40"/>
+    <mergeCell ref="A31:G31"/>
+    <mergeCell ref="A39:G39"/>
+    <mergeCell ref="A34:G34"/>
+    <mergeCell ref="A24:G24"/>
+    <mergeCell ref="A30:G30"/>
+    <mergeCell ref="A45:G45"/>
+    <mergeCell ref="A36:G36"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A25:G25"/>
+    <mergeCell ref="A41:G41"/>
+    <mergeCell ref="A37:G37"/>
+    <mergeCell ref="A46:G46"/>
+    <mergeCell ref="A18:G18"/>
+    <mergeCell ref="A27:G27"/>
+    <mergeCell ref="A21:G21"/>
+    <mergeCell ref="A26:G26"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A33:G33"/>
+    <mergeCell ref="A47:G47"/>
+    <mergeCell ref="A42:G42"/>
+    <mergeCell ref="A23:G23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add CDC Travel Notice columns to declarations.csv; pin browser for unattended xcancel runs
</commit_message>
<xml_diff>
--- a/outputs/ebola_timeseries.xlsx
+++ b/outputs/ebola_timeseries.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G48"/>
+  <dimension ref="A1:G49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1089,8 +1089,15 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" s="9" t="inlineStr">
+        <is>
+          <t>• 2026-05-25 (schema change, declarations.csv): Added two columns to distinguish CDC's clinician-facing HAN advisory from its traveler-facing Travel Health Notice. New schema: `country, first_report_date, case_status, cdc_advisory, cdc_url, cdc_travel_notice_level, cdc_travel_notice_url, who_status, who_url, notes`. Backfilled both rows: DRC at Level 3 (Reconsider Nonessential Travel, https://wwwnc.cdc.gov/travel/notices/level3/ebola-democratic-republic-of-the-congo), Uganda at Level 1 (Practice Usual Precautions, https://wwwnc.cdc.gov/travel/notices/level1/ebola-uganda). Note: CDC has escalated DRC from Level 2 to Level 3 since the 2026-05-16 CDC Situation Summary publication, which still links to the Level 2 page. METHODOLOGY.md updated to document the new schema and the two-system distinction. Daily-task SKILL.md updated to instruct future runs to check the per-country travel-notice URLs each pass.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="33">
+  <mergeCells count="34">
     <mergeCell ref="A32:G32"/>
     <mergeCell ref="A22:G22"/>
     <mergeCell ref="A35:G35"/>
@@ -1108,6 +1115,7 @@
     <mergeCell ref="A48:G48"/>
     <mergeCell ref="A24:G24"/>
     <mergeCell ref="A30:G30"/>
+    <mergeCell ref="A49:G49"/>
     <mergeCell ref="A45:G45"/>
     <mergeCell ref="A36:G36"/>
     <mergeCell ref="A1:G1"/>

</xml_diff>

<commit_message>
Add src/validate.py pre-commit gate; apply no-dip rule retroactively to May 19, May 22, May 23 rows
</commit_message>
<xml_diff>
--- a/outputs/ebola_timeseries.xlsx
+++ b/outputs/ebola_timeseries.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G49"/>
+  <dimension ref="A1:G51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -669,20 +669,20 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>516</v>
+        <v>528</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>33</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>549</v>
+        <v>561</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>WHO / Wikipedia summary of WHO data</t>
+          <t>WHO Sitrep 01 figures carried forward (no-dip rule); May 19 Wikipedia summary reported 516/33/131</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
@@ -756,20 +756,20 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D12" s="6" t="n">
-        <v>827</v>
+        <v>831</v>
       </c>
       <c r="E12" s="6" t="n">
         <v>176</v>
       </c>
       <c r="F12" s="7" t="inlineStr">
         <is>
-          <t>CDC Situation Summary (May 22)</t>
+          <t>WHO DON603 figures carried forward (no-dip rule); May 22 CDC Situation Summary reported 744/83/176</t>
         </is>
       </c>
       <c r="G12" s="7" t="inlineStr">
@@ -788,17 +788,17 @@
         <v>750</v>
       </c>
       <c r="C13" s="4" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>837</v>
+        <v>838</v>
       </c>
       <c r="E13" s="4" t="n">
         <v>177</v>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>WHO Tedros briefing (May 22, via CIDRAP/ABC) + Uganda MoH (May 23, +3 cases)</t>
+          <t>WHO Tedros briefing (May 22, via CIDRAP/ABC) + Uganda MoH (May 23); DRC confirmed carried forward from revised May 22 (no-dip cascade); briefing-source globals: 750/87/837</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
@@ -1096,8 +1096,22 @@
         </is>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" s="9" t="inlineStr">
+        <is>
+          <t>• 2026-05-25 (index.html render): Added a "CDC travel notice" column to the public declarations table on index.html, positioned between "CDC advisory" (HAN) and "WHO status" so the two CDC systems read left to right. Cell shows the level + meaning (e.g., "Level 3 (Reconsider Nonessential Travel)") and links to the matching wwwnc.cdc.gov page. Empty `cdc_travel_notice_level` cells fall back to a blank cell. Colspan on the loading and empty-state rows bumped from 6 to 7.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="9" t="inlineStr">
+        <is>
+          <t>• 2026-05-25 (validator + retroactive no-dip cleanup): Added src/validate.py as a pre-commit gate that enforces schema, monotonic cumulative columns, total = sus + conf, country-sum-equals-global on the latest date, date format/uniqueness. First run caught four legacy no-dip violations from partial revision reconciliation. Applied retroactive cleanup per the rule as written in METHODOLOGY.md: May 19 row carried forward from revised May 18 (WHO Sitrep 01): suspected 516→528, total 549→561, suspected_deaths 131→132. May 22 row carried forward from revised May 21 (WHO DON603): suspected 744→746, confirmed 83→85, total 827→831. The May 22 lift cascaded into May 23: DRC confirmed bumped 82→83 to stay non-decreasing, lifting global confirmed 87→88 and total 837→838. country_breakdown.csv DRC rows updated to match: May 19 DRC suspected 516→528, suspected_deaths 131→132; May 22 DRC suspected 744→746, confirmed 81→83; May 23 DRC confirmed 82→83. All primary_source fields amended to flag the carry-forward and record the same-day source's original figures for audit. May 24 and May 25 rows unaffected. Validator now passes clean.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="34">
+  <mergeCells count="36">
     <mergeCell ref="A32:G32"/>
     <mergeCell ref="A22:G22"/>
     <mergeCell ref="A35:G35"/>
@@ -1116,6 +1130,7 @@
     <mergeCell ref="A24:G24"/>
     <mergeCell ref="A30:G30"/>
     <mergeCell ref="A49:G49"/>
+    <mergeCell ref="A51:G51"/>
     <mergeCell ref="A45:G45"/>
     <mergeCell ref="A36:G36"/>
     <mergeCell ref="A1:G1"/>
@@ -1126,6 +1141,7 @@
     <mergeCell ref="A18:G18"/>
     <mergeCell ref="A27:G27"/>
     <mergeCell ref="A21:G21"/>
+    <mergeCell ref="A50:G50"/>
     <mergeCell ref="A26:G26"/>
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A33:G33"/>
@@ -1331,22 +1347,22 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>-12</v>
+        <v>0</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>0</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>516</v>
+        <v>528</v>
       </c>
       <c r="F9" s="4" t="n">
         <v>33</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H9" s="4" t="n">
         <v>5</v>
@@ -1359,13 +1375,13 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>84</v>
+        <v>72</v>
       </c>
       <c r="C10" s="6" t="n">
         <v>18</v>
       </c>
       <c r="D10" s="6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E10" s="6" t="n">
         <v>600</v>
@@ -1415,19 +1431,19 @@
         </is>
       </c>
       <c r="B12" s="6" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="C12" s="6" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="D12" s="6" t="n">
         <v>0</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="G12" s="6" t="n">
         <v>96</v>
@@ -1443,10 +1459,10 @@
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="C13" s="4" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D13" s="4" t="n">
         <v>1</v>
@@ -1455,7 +1471,7 @@
         <v>414</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G13" s="4" t="n">
         <v>90</v>
@@ -1474,7 +1490,7 @@
         <v>154</v>
       </c>
       <c r="C14" s="6" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="D14" s="6" t="n">
         <v>43</v>
@@ -1864,18 +1880,18 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>516</v>
+        <v>528</v>
       </c>
       <c r="D13" s="4" t="n">
         <v>31</v>
       </c>
       <c r="E13" s="4" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="F13" s="4" t="n"/>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>WHO / Wikipedia summary of WHO data</t>
+          <t>WHO Sitrep 01 figures carried forward (no-dip rule); May 19 Wikipedia summary reported 516 sus / 131 deaths</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -2050,10 +2066,10 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>744</v>
+        <v>746</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="E19" s="4" t="n">
         <v>176</v>
@@ -2061,7 +2077,7 @@
       <c r="F19" s="4" t="n"/>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>CDC Situation Summary (May 22)</t>
+          <t>WHO DON603 figures carried forward (no-dip rule); May 22 CDC reported 744/81/176</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
@@ -2115,7 +2131,7 @@
         <v>750</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>177</v>
@@ -2123,7 +2139,7 @@
       <c r="F21" s="4" t="n"/>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>WHO Tedros briefing (May 22, via CIDRAP/ABC) + Uganda MoH (May 23, +3 cases)</t>
+          <t>WHO Tedros briefing (May 22, via CIDRAP/ABC) + Uganda MoH (May 23); DRC confirmed carried forward from revised May 22 (no-dip cascade); briefing reported 82</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">

</xml_diff>

<commit_message>
README: document src/validate.py pre-commit gate
</commit_message>
<xml_diff>
--- a/outputs/ebola_timeseries.xlsx
+++ b/outputs/ebola_timeseries.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G51"/>
+  <dimension ref="A1:G52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -827,7 +827,7 @@
       </c>
       <c r="F14" s="7" t="inlineStr">
         <is>
-          <t>DRC govt figures (Sunday May 24, via Reuters/AP/UN News/CNN) for cases; WHO DG Tedros (May 25 remarks) for suspected deaths ('at least 220'); no-dip rule applied</t>
+          <t>DRC govt figures (Sunday May 24, via Reuters/AP/UN News/CNN) for cases; WHO DG Tedros (May 25 Virtual Ministerial Briefing on Bundibugyo) reaffirms 220 suspected deaths and 10 confirmed deaths in DRC; no-dip rule applied</t>
         </is>
       </c>
       <c r="G14" s="7" t="inlineStr">
@@ -856,7 +856,7 @@
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Uganda MoH (May 25): +2 confirmed (Kampala health workers); DRC cases carry Sunday May 24 govt figures (Reuters/AP); WHO DG Tedros (May 25 remarks) for suspected deaths ('at least 220'); no-dip rule applied</t>
+          <t>WHO DG Tedros (May 25 Virtual Ministerial Briefing on Bundibugyo): 904 sus / 101 conf / 220 sus deaths / 10 conf deaths in DRC; Uganda MoH (May 25 press release): +2 confirmed (Kampala health workers), Uganda 7 conf / 1 death; no-dip rule applied</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
@@ -1110,14 +1110,22 @@
         </is>
       </c>
     </row>
+    <row r="52">
+      <c r="A52" s="9" t="inlineStr">
+        <is>
+          <t>• 2026-05-25 (late-evening run): No new numerical figures since the evening run. Citation upgrade applied to May 24 and May 25 rows: WHO DG Tedros's [remarks at the Virtual Ministerial Briefing on the Bundibugyo Ebola Outbreak](https://www.who.int/news-room/speeches/item/who-director-general-s-remarks-at-the-virtual-ministerial-briefing-on-the-bundibugyo-ebola-outbreak-25-may-2026) (25 May 2026) now serve as the primary source for the DRC figures (904 sus / 101 conf / 220 sus deaths / 10 conf deaths). This is a WHO-DG-attributed primary source, higher-tier than the Reuters/AP wires previously cited; corroborated by [UN News (25 May)](https://news.un.org/en/story/2026/05/1167584) and Xinhua. Uganda figures still cite Uganda MoH May 25 press release (+2 health workers in Kampala, total 7 conf / 1 death). The Tedros briefing gave 5 confirmed for Uganda; that figure predates the Uganda MoH same-day +2 release. Per source-preference, the Uganda national MoH remains the authoritative source for Uganda's count. WHO Sitrep 02 and WHO DON604 still not published. CDC Situation Summary still dated 16 May with stale figures; DRC travel notice remains Level 3 (Reconsider Nonessential Travel). 7-day lookback against May 19–25: no numerical revisions required. story.md "Latest update" refreshed to incorporate the WHO DG quote ("the epidemic is outpacing us"), DRC national risk upgraded from "high" to "very high", two treatment centers set alight in eastern DRC, 100,000+ displaced by fighting, $3.9M WHO Contingency Fund release, and WHO clinical-trial prioritization of two monoclonal antibodies + obeldesivir. No declarations.csv change (national risk upgrade is a WHO statement, not a formal declaration change; PHEIC level unchanged). Charts and XLSX regenerated; output filenames unchanged (most-recent Report Date still 2026-05-25).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="36">
+  <mergeCells count="37">
     <mergeCell ref="A32:G32"/>
     <mergeCell ref="A22:G22"/>
     <mergeCell ref="A35:G35"/>
     <mergeCell ref="A20:G20"/>
     <mergeCell ref="A38:G38"/>
     <mergeCell ref="A29:G29"/>
+    <mergeCell ref="A52:G52"/>
     <mergeCell ref="A43:G43"/>
     <mergeCell ref="A19:G19"/>
     <mergeCell ref="A28:G28"/>
@@ -2203,7 +2211,7 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>Cases per DRC govt Sunday update (Reuters/AP); suspected deaths per WHO DG Tedros remarks (May 25); no-dip rule</t>
+          <t>DRC govt Sunday update (Reuters/AP) for cases; WHO DG Tedros (May 25 Virtual Ministerial Briefing) reaffirms 220 sus deaths / 10 conf deaths; no-dip rule</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
@@ -2267,12 +2275,12 @@
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>DRC cases carry Sunday May 24 figures; suspected deaths per WHO DG Tedros (May 25); no-dip rule</t>
+          <t>WHO DG Tedros (May 25 Virtual Ministerial Briefing on Bundibugyo): 904 sus / 101 conf / 220 sus deaths / 10 conf deaths; no-dip rule</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>2026-05-24</t>
+          <t>2026-05-25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Methodology: add MoH carve-out; apply DRC May 30 cleaned baseline
Adds the MoH methodology-change carve-out to the no-dip rule and applies it
to the 2026-05-30 DRC MoH ~700-case removal (lab capacity ramp-up; remaining
suspected cases tested negative for Ebola). May 30 and May 31 rows revised
to the DRC MoH cleaned baseline. OBSERVED_REVISION_RANGE split into upward
and downward bands. Validator gets NO_DIP_EXEMPTIONS dicts so the dip is
explicit and auditable.
</commit_message>
<xml_diff>
--- a/outputs/ebola_timeseries.xlsx
+++ b/outputs/ebola_timeseries.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G128"/>
+  <dimension ref="A1:G135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -988,20 +988,20 @@
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>906</v>
+        <v>349</v>
       </c>
       <c r="C20" s="6" t="n">
-        <v>134</v>
+        <v>234</v>
       </c>
       <c r="D20" s="6" t="n">
-        <v>1040</v>
+        <v>583</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>223</v>
+        <v>0</v>
       </c>
       <c r="F20" s="7" t="inlineStr">
         <is>
-          <t>[WHO DON605](https://www.who.int/emergencies/disease-outbreak-news/item/2026-DON605) figures carried forward (no-dip rule). [WHO DG Tedros press briefing in Bunia, 30 May 2026](https://www.who.int/news-room/speeches/item/who-director-general-s-remarks-at-the-press-briefing-on-the-on-the-bundibugyo-ebola-outbreak---30-may-2026) is qualitative (community ownership, safe burials, dignified care, urges countries to reconsider border closures): no new global case/death figures cited. BNO @BNOFeed Daily Ebola Update May 30 graphic reports DRC MoH cleaned-baseline figures: DR Congo 574 cases / 17 deaths (N/A deltas; "Today, Congo removed nearly 700 suspected cases after they tested negative for Ebola. This follows an increase in testing capabilities. As a result, it's unknown how many new cases were added today"); Uganda 9 conf / 1 death (unchanged); TOTAL 583 cases / 18 deaths. The DRC MoH ~700-case removal is a DRC-MoH-attributed single-source dip; per the no-dip rule it is held pending WHO corroboration. Cumulative TOTAL would drop from 1,040 → 583 (-43.94%) and TOTAL DEATHS from 224 (223 sus + 1 Uganda conf) → 18 (-91.96%) if applied; WHO Sitrep 03 expected Tue 2 Jun will likely reconcile a partial catch-up reflecting both the +100 DRC lab confirmations from 29 May and the ~700 sus-case removal from 30 May. WHO DON605 reconciled figures remain authoritative for this row.</t>
+          <t>REVISED 2026-05-31 (PM): MoH methodology-change carve-out applied per METHODOLOGY.md. BNO @BNOFeed Daily Ebola Update May 30 graphic carries DRC MoH's formally-announced cleaned baseline: "Today, Congo removed nearly 700 suspected cases after they tested negative for Ebola. This follows an increase in testing capabilities." DRC totals on the cleaned baseline: 574 cases / 17 deaths. Per the carve-out, DRC MoH is the single high-value source needed because the dip IS the definitional reclassification (lab capacity ramp-up; remaining cases tested negative). Sus/conf split: DRC confirmed carries forward at DRC MoH's running 225 (BNO @BNOFeed May 29 graphic, +100 lab catch-up); DRC suspected = 574 - 225 = 349. DRC suspected_deaths column zeroed by DRC MoH (17 deaths = pre-cleanup conf_deaths only); DRC conf_deaths = 17 unchanged. Uganda 9 conf / 1 death unchanged. Global: sus 906→349 (-61.48%), conf 134→234 (+74.63%), total 1040→583 (-43.94%), sus_deaths 223→0 (-100%). Prior values were the WHO DON605 carry-forward held under the no-dip rule pending WHO corroboration; the rule's MoH carve-out (added 2026-05-31 PM) now exempts this row's downward revisions. [WHO DG Tedros press briefing in Bunia, 30 May 2026](https://www.who.int/news-room/speeches/item/who-director-general-s-remarks-at-the-press-briefing-on-the-on-the-bundibugyo-ebola-outbreak---30-may-2026) remains qualitative (community ownership, safe burials, border-closure pushback); WHO Sitrep 03 expected Tue 2 Jun will reconcile DRC MoH's cleaned baseline against WHO surveillance. Original WHO DON605 figures: 906/134/1040/223. NO_DIP_EXEMPTIONS entry: 2026-05-30 → {suspected_global, total_global, suspected_deaths_global}.</t>
         </is>
       </c>
       <c r="G20" s="7" t="inlineStr">
@@ -1017,20 +1017,20 @@
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>906</v>
+        <v>447</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>134</v>
+        <v>234</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>1040</v>
+        <v>681</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>223</v>
+        <v>0</v>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>[WHO DON605](https://www.who.int/emergencies/disease-outbreak-news/item/2026-DON605) figures carried forward (no-dip rule). Citation upgrade this pass: [Joint statement by the Government of the DRC and WHO, 31 May 2026](https://www.who.int/news/item/31-05-2026-joint-statement-by-the-government-of-the-democratic-republic-of-the-congo-and-who-concerning-the-outbreak-of-ebola-disease-caused-by-the-bundibugyo-virus) issued at the conclusion of the Tedros / Kamba / Muyaya Bunia mission. Statement is qualitative (no global case/death figures): reaffirms "rapidly evolving situation, with cases and deaths notified in several health zones of Ituri, North Kivu and South Kivu"; commits to "rapidly undertake randomized control trials on candidate vaccines and treatments"; explicit call that "borders remain open, and that entry controls do not obstruct the flow of desperately needed medical supplies and personnel" (reinforces Tedros's 30 May press-briefing border-closure pushback). BNO @BNOFeed Daily Ebola Update May 31 graphic (posted ~14h before this pass) reports DRC MoH-attributed running figures on the cleaned baseline: DR Congo 672 cases (+98) / 55 deaths (+38); Uganda 9 conf / 1 death (unchanged); TOTAL 681 (+98) / 56 (+38). Implied DRC MoH cleaned baseline still materially below WHO DON605's 1,040 reconciled total; DRC MoH single-source dip remains held pending WHO Sitrep 03 / DON606. WHO DG Tedros 31 May tweet thread documents the opening of a new 42-bed Ebola treatment center in Bunia (converted from a pediatric building entrusted to WHO by Centre Évangélique Médical) — operational milestone, no figures. Per source-preference order, WHO DON605 wins for the row's cumulative attribution.</t>
+          <t>REVISED 2026-05-31 (PM): MoH methodology-change carve-out applied per METHODOLOGY.md; new baseline rolls forward from the revised May 30 row. BNO @BNOFeed Daily Ebola Update May 31 graphic (sourced to DRC MoH + Uganda MoH + WHO) reports DRC running on the cleaned baseline: DR Congo 672 cases (+98 from May 30) / 55 deaths (+38 from May 30); Uganda 9 conf / 1 death (unchanged); TOTAL 681 (+98) / 56 (+38). Sus/conf split inference: DRC confirmed carries forward at DRC MoH's running 225 (no fresh May 31 lab figure published; +38 deaths attributed to conf_deaths as DRC MoH continues to lab-confirm previously-probable deaths); DRC suspected = 672 - 225 = 447; DRC sus_deaths stays at 0 (column zeroed May 30 carries forward); DRC conf_deaths 17 + 38 = 55. Uganda unchanged. Global vs May 30: sus 349→447 (+98), conf 234 (unchanged), total 583→681 (+98), sus_deaths 0 (unchanged). Global vs prior WHO DON605 carry-forward (906/134/1040/223): sus -50.66%, conf +74.63%, total -34.52%, sus_deaths -100%. Citation upgrade this pass: [Joint statement by the Government of the DRC and WHO, 31 May 2026](https://www.who.int/news/item/31-05-2026-joint-statement-by-the-government-of-the-democratic-republic-of-the-congo-and-who-concerning-the-outbreak-of-ebola-disease-caused-by-the-bundibugyo-virus) closing the Tedros / Kamba / Muyaya Bunia mission. Statement qualitative (no global figures): commits to "rapidly undertake randomized control trials on candidate vaccines and treatments"; explicit call that "borders remain open." WHO DG Tedros 31 May tweets document opening of a new 42-bed Ebola treatment center in Bunia (converted from a pediatric building entrusted to WHO by Centre Évangélique Médical). WHO Sitrep 03 expected Tue 2 Jun will reconcile DRC MoH's cleaned baseline against WHO surveillance.</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
@@ -1781,8 +1781,57 @@
         </is>
       </c>
     </row>
+    <row r="129">
+      <c r="A129" s="9" t="inlineStr">
+        <is>
+          <t>• 2026-05-31 (PM2 run, methodology refinement per Web): Added "MoH methodology-change carve-out" to the no-dip rule in METHODOLOGY.md. Rationale: the no-dip rule as originally written required two high-value sources to apply a downward revision. The DRC MoH 30 May ~700-case cleanup (lab capacity ramp-up; suspected cases that subsequently tested negative for Ebola are removed) is a formally-announced definitional reclassification by the official surveillance authority. A definitional cleanup announced by the surveillance source IS the reclassification, by definition; waiting for WHO Sitrep reconciliation in that case is a delay, not a correction. The carve-out waives the two-source threshold when the dip is a MoH (DRC or Uganda) formal announcement and the wire is faithfully carrying it. The standard no-dip rule still applies to wire-only paraphrases of unreconciled recounts. Operationally: exemptions are recorded in `src/validate.py`'s NO_DIP_EXEMPTIONS_TIMESERIES (date → columns) and NO_DIP_EXEMPTIONS_BREAKDOWN ((date, country) → columns) so the no-dip validator skips the named columns on the named row(s). Every exemption gets a NOTES bullet citing the MoH announcement and the figures applied. This was the prototypical case; future MoH cleanups will follow the same pattern.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="9" t="inlineStr">
+        <is>
+          <t>• 2026-05-31 (PM2 run, carve-out applied to May 30 row): timeseries.csv May 30 row revised per DRC MoH cleaned baseline via BNO @BNOFeed May 30 graphic: suspected_global 906→349 (-61.48%), confirmed_global 134→234 (+74.63%), total_global 1040→583 (-43.94%), suspected_deaths_global 223→0 (-100%). Sus/conf split: DRC confirmed accepts DRC MoH's running 225 (BNO @BNOFeed May 29 +100 lab catch-up); DRC suspected = 574 - 225 = 349. DRC sus_deaths column zeroed by DRC MoH in the same cleanup (the 17 deaths on BNO's May 30 graphic = pre-cleanup conf_deaths only). DRC conf_deaths = 17 unchanged. Uganda 9 / 1 unchanged. NO_DIP_EXEMPTIONS_TIMESERIES entry: "2026-05-30" → {suspected_global, total_global, suspected_deaths_global}. The confirmed_global column is NOT exempt because the revision is upward (134 → 234); the dip exemption applies only to the columns going downward. NO_DIP_EXEMPTIONS_BREAKDOWN entry: ("2026-05-30", "DRC") → {suspected, suspected_deaths}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="9" t="inlineStr">
+        <is>
+          <t>• 2026-05-31 (PM2 run, carve-out propagated to May 31 row): timeseries.csv May 31 row revised: suspected_global 906→447 (-50.66%), confirmed_global 134→234 (+74.63%), total_global 1040→681 (-34.52%), suspected_deaths_global 223→0 (-100%). Split: DRC conf carries the May 30 DRC MoH running 225 forward (no fresh May 31 lab figure published); DRC sus = 672 - 225 = 447. DRC sus_deaths stays at 0 (column zeroed May 30); +38 deaths in BNO's May 31 graphic attributed to conf_deaths as DRC MoH continues to lab-confirm previously-probable deaths, so DRC conf_deaths = 17 + 38 = 55. No exemption needed for the May 31 row in the validator: cumulative globals against the May 30 baseline are non-decreasing (sus 349→447, conf 234→234, total 583→681, sus_deaths 0→0). Per-country DRC also non-decreasing against May 30 baseline (sus 349→447, conf 225→225, sus_deaths 0→0, conf_deaths 17→55).</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="9" t="inlineStr">
+        <is>
+          <t>• 2026-05-31 (PM2 run, chart constants): Split OBSERVED_REVISION_RANGE into OBSERVED_UPWARD_REVISION_RANGE (still "&lt;1-35%", reflecting WHO Sitrep / DON reconciliation history) and OBSERVED_DOWNWARD_REVISION_RANGE ("up to 100%", reflecting the May 30 MoH carve-out: sus -61.48%, sus_deaths -100%). Chart-footnote string updated to surface both directions: "Bars after {LAST_SITREP_STABLE_DATE} are provisional; revisions have run +{up} (Sitrep reconciliation) and {down} downward (MoH definitional cleanups)." Generate_charts.py constants comment updated to document both ranges and the mechanisms behind each.</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="9" t="inlineStr">
+        <is>
+          <t>• 2026-05-31 (PM2 run, validator): Added NO_DIP_EXEMPTIONS_TIMESERIES and NO_DIP_EXEMPTIONS_BREAKDOWN dicts at the top of src/validate.py with named exemptions per the carve-out. The cumulative non-decreasing checks now skip exempt (date, column) and (date, country, column) tuples. Validator passes clean after revisions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="9" t="inlineStr">
+        <is>
+          <t>• 2026-05-31 (PM2 run, story.md): "Latest update" rewritten to lead with the DRC MoH cleanup and the new lower figures, explicitly explaining that the visual drop on the chart is the surveillance signal working as intended (suspected-cases bar deliberately wide → lab capacity catches up → negatives get removed → tighter denominator). The WHO/DRC Joint Statement section retained as the second paragraph. "Story so far" unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="9" t="inlineStr">
+        <is>
+          <t>• 2026-05-31 (PM2 run, declarations.csv): No change. CDC HAN, CDC Travel Health Notice levels, WHO PHEIC, Uganda border closure all unchanged. The carve-out is a tracker methodology refinement, not a declaration change.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="107">
+  <mergeCells count="114">
     <mergeCell ref="A126:G126"/>
     <mergeCell ref="A53:G53"/>
     <mergeCell ref="A109:G109"/>
@@ -1807,8 +1856,10 @@
     <mergeCell ref="A105:G105"/>
     <mergeCell ref="A26:G26"/>
     <mergeCell ref="A71:G71"/>
+    <mergeCell ref="A129:G129"/>
     <mergeCell ref="A116:G116"/>
     <mergeCell ref="A91:G91"/>
+    <mergeCell ref="A131:G131"/>
     <mergeCell ref="A100:G100"/>
     <mergeCell ref="A52:G52"/>
     <mergeCell ref="A63:G63"/>
@@ -1828,6 +1879,7 @@
     <mergeCell ref="A78:G78"/>
     <mergeCell ref="A65:G65"/>
     <mergeCell ref="A75:G75"/>
+    <mergeCell ref="A133:G133"/>
     <mergeCell ref="A80:G80"/>
     <mergeCell ref="A120:G120"/>
     <mergeCell ref="A55:G55"/>
@@ -1844,10 +1896,12 @@
     <mergeCell ref="A58:G58"/>
     <mergeCell ref="A40:G40"/>
     <mergeCell ref="A67:G67"/>
+    <mergeCell ref="A130:G130"/>
     <mergeCell ref="A24:G24"/>
     <mergeCell ref="A82:G82"/>
     <mergeCell ref="A60:G60"/>
     <mergeCell ref="A123:G123"/>
+    <mergeCell ref="A132:G132"/>
     <mergeCell ref="A110:G110"/>
     <mergeCell ref="A124:G124"/>
     <mergeCell ref="A25:G25"/>
@@ -1859,10 +1913,12 @@
     <mergeCell ref="A2:G2"/>
     <mergeCell ref="A86:G86"/>
     <mergeCell ref="A47:G47"/>
+    <mergeCell ref="A135:G135"/>
     <mergeCell ref="A122:G122"/>
     <mergeCell ref="A125:G125"/>
     <mergeCell ref="A72:G72"/>
     <mergeCell ref="A29:G29"/>
+    <mergeCell ref="A134:G134"/>
     <mergeCell ref="A81:G81"/>
     <mergeCell ref="A112:G112"/>
     <mergeCell ref="A121:G121"/>
@@ -2397,22 +2453,22 @@
         </is>
       </c>
       <c r="B20" s="6" t="n">
-        <v>0</v>
+        <v>-557</v>
       </c>
       <c r="C20" s="6" t="n">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="D20" s="6" t="n">
-        <v>0</v>
+        <v>-223</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>156</v>
+        <v>-401</v>
       </c>
       <c r="F20" s="6" t="n">
-        <v>46</v>
+        <v>146</v>
       </c>
       <c r="G20" s="6" t="n">
-        <v>46</v>
+        <v>-177</v>
       </c>
       <c r="H20" s="6" t="n">
         <v>7</v>
@@ -2425,7 +2481,7 @@
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>0</v>
+        <v>98</v>
       </c>
       <c r="C21" s="4" t="n">
         <v>0</v>
@@ -2434,13 +2490,13 @@
         <v>0</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>0</v>
+        <v>-459</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>22</v>
+        <v>122</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>0</v>
+        <v>-223</v>
       </c>
       <c r="H21" s="4" t="n">
         <v>7</v>
@@ -3484,20 +3540,20 @@
         </is>
       </c>
       <c r="C35" s="4" t="n">
-        <v>906</v>
+        <v>349</v>
       </c>
       <c r="D35" s="4" t="n">
-        <v>125</v>
+        <v>225</v>
       </c>
       <c r="E35" s="4" t="n">
-        <v>223</v>
+        <v>0</v>
       </c>
       <c r="F35" s="4" t="n">
         <v>17</v>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>[WHO DON605](https://www.who.int/emergencies/disease-outbreak-news/item/2026-DON605) figures carried forward (no-dip rule). BNO @BNOFeed Daily Ebola Update May 30 graphic shows DRC MoH cleaned-baseline running count: 574 cases / 17 deaths (N/A deltas). DRC MoH note via BNO "Today, Congo removed nearly 700 suspected cases after they tested negative for Ebola. This follows an increase in testing capabilities. As a result, it's unknown how many new cases were added today." The DRC MoH ~700-case removal would imply: from BNO's May 29 pre-removal DRC ~1,028 sus / 225 conf / 240 deaths → May 30 cleaned-baseline ~574 / 225 / 17 (DRC MoH consolidating sus + conf into 574 total cases; deaths drop reflects reclassification of non-Ebola deaths). Held pending WHO corroboration. WHO Sitrep 03 expected Tue 2 Jun. WHO DG Tedros in Bunia 30 May; qualitative press briefing, no new figures.</t>
+          <t>REVISED 2026-05-31 (PM): MoH methodology-change carve-out applied per METHODOLOGY.md. BNO @BNOFeed Daily Ebola Update May 30 graphic carries DRC MoH cleaned-baseline figures: 574 cases / 17 deaths. DRC MoH note via BNO: "Today, Congo removed nearly 700 suspected cases after they tested negative for Ebola. This follows an increase in testing capabilities. As a result, it's unknown how many new cases were added today." Per the carve-out, DRC MoH is the single high-value source needed (definitional reclassification by the surveillance authority itself). Split: DRC conf carries DRC MoH's running 225 (BNO @BNOFeed May 29 graphic, +100 lab catch-up from WHO DON605's 125); DRC sus = 574 - 225 = 349; DRC sus_deaths zeroed by DRC MoH (17 deaths line = pre-cleanup conf_deaths only); DRC conf_deaths = 17 unchanged. Revisions vs prior WHO DON605 carry-forward (906/125/223/17): sus -61.48%, conf +80.00%, sus_deaths -100%, conf_deaths unchanged. NO_DIP_EXEMPTIONS_BREAKDOWN entry: (2026-05-30, DRC) → {suspected, suspected_deaths}. WHO Sitrep 03 expected Tue 2 Jun will reconcile.</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr">
@@ -3548,20 +3604,20 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>906</v>
+        <v>447</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>125</v>
+        <v>225</v>
       </c>
       <c r="E37" s="4" t="n">
-        <v>223</v>
+        <v>0</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>17</v>
+        <v>55</v>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>[WHO DON605](https://www.who.int/emergencies/disease-outbreak-news/item/2026-DON605) figures carried forward (no-dip rule). BNO @BNOFeed Daily Ebola Update May 31 graphic (posted ~6h before this pass): DR Congo 672 cases (+98) / 55 deaths (+38), on the May 30 DRC MoH cleaned baseline. New confirmations and deaths added to the cleaned baseline. Still materially below WHO DON605's reconciled DRC 906 sus + 125 conf = 1,031 total per WHO methodology; DRC MoH single-source dip remains held pending WHO Sitrep 03 / DON606.</t>
+          <t>REVISED 2026-05-31 (PM): MoH methodology-change carve-out propagated from revised May 30 row. BNO @BNOFeed Daily Ebola Update May 31 graphic (sourced to DRC MoH + Uganda MoH + WHO): DR Congo 672 cases (+98) / 55 deaths (+38), on the May 30 DRC MoH cleaned baseline. Split inference: DRC conf carries the May 30 DRC MoH running 225 forward (no fresh May 31 lab figure published); DRC sus = 672 - 225 = 447; DRC sus_deaths stays at 0 (column zeroed May 30); +38 deaths attributed to conf_deaths as DRC MoH continues lab-confirming previously-probable deaths, so DRC conf_deaths = 17 + 38 = 55. Revisions vs prior WHO DON605 carry-forward (906/125/223/17): sus -50.66%, conf +80.00%, sus_deaths -100%, conf_deaths +223.53%. Revisions vs revised May 30 row: sus +98 (+28.08%), conf 0, sus_deaths 0, conf_deaths +38 (+223.53%). WHO Sitrep 03 expected Tue 2 Jun will reconcile.</t>
         </is>
       </c>
       <c r="H37" s="5" t="inlineStr">

</xml_diff>

<commit_message>
declarations: Uganda CDC notice Level 1->2 (May 27); add State Dept L4, Title 42, Africa CDC PHECS
Surfaced by Web audit: declarations.csv had drifted out of sync with live
CDC and US government sources across six consecutive runs. Refresh applies
the missed events between May 18 and May 31.

- Uganda cdc_travel_notice_level: Level 1 -> Level 2 (CDC raised it on
  2026-05-27; confirmed by US Embassy Kampala 28 May health alert)
- Uganda cdc_travel_notice_url: /level1/ebola-uganda -> /level2/ebola-uganda
- DRC cdc_travel_notice_level unchanged at Level 3 (re-verified)
- DRC + Uganda notes expanded: US State Department Level 4 (Do Not Travel)
  advisory, US entry restrictions on non-US passport holders, CDC Title 42
  Order, Africa CDC PHECS declaration of 2026-05-18, US arrivals screening
  funnel (IAD/ATL/IAH), WHO+DRC Joint Statement 2026-05-31 borders-open ask
- DRC notes: 12 -> 13 health zones; Sud-Kivu first lab-confirmed 2026-05-25
</commit_message>
<xml_diff>
--- a/outputs/ebola_timeseries.xlsx
+++ b/outputs/ebola_timeseries.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H135"/>
+  <dimension ref="A1:H139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1888,12 +1888,41 @@
         </is>
       </c>
     </row>
+    <row r="136">
+      <c r="A136" s="9" t="inlineStr">
+        <is>
+          <t>• 2026-05-31 (PM3 run, schema change per Web): Added `confirmed_deaths_global` column to data/timeseries.csv schema, between `suspected_deaths_global` and `primary_source`. Rationale: after the DRC MoH cleanup zeroed the suspected-deaths column on 2026-05-30, "suspected deaths" stopped being a useful headline metric. Real deaths are still accumulating; they're just on the confirmed side now (DRC ran +38 lab confirmations on 31 May for a DRC conf_deaths total of 55). The deaths chart was showing 0 new deaths in the 7-day rolling window on May 31, which was technically true for the suspected column but materially misleading. Schema is now: report_date, suspected_global, confirmed_global, total_global, suspected_deaths_global, confirmed_deaths_global, primary_source, source_timestamp. Backfilled historical values from country_breakdown.csv DRC + Uganda sums: May 15-23 = 1 (Uganda only); May 24-26 = 11 (DRC 10 + Uganda 1); May 27-30 = 18 (DRC 17 + Uganda 1); May 31 = 56 (DRC 55 + Uganda 1). Cumulative monotonically non-decreasing throughout; no NO_DIP_EXEMPTIONS entry needed for the new column. src/validate.py updated to include confirmed_deaths_global in EXPECTED_TIMESERIES_COLS and CUMULATIVE_TIMESERIES_COLS, plus the parse loop. src/build_xlsx.py updated to add the new column to the main sheet header and the Charts sheet's daily-delta + rolling-sum derivation. Validator passes clean.</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="9" t="inlineStr">
+        <is>
+          <t>• 2026-05-31 (PM3 run, deaths chart restructure): Reworked render_deaths_chart in src/generate_charts.py to mirror render_cases_chart structurally. Bars now stacked: confirmed deaths (COLOR_CONFIRMED, bottom) + suspected deaths (COLOR_SUSPECTED, top); hatched on provisional dates. Cumulative-line overlay now carries two lines: total deaths (sus + conf, COLOR_CUMULATIVE bronze) and confirmed-only deaths (COLOR_CUMULATIVE_CONF deep red), matching the cases chart's two-line treatment. The gap between the lines is the share of the running death count still in clinical-suspicion-only status. Chart suptitle changed from "7-day rolling sum of suspected deaths" to "7-day rolling sum of new deaths"; axis label and inline title updated to match. Legend rebuilt: confirmed deaths Patch + suspected deaths Patch + provisional swatch + cumulative-total Line2D + cumulative-confirmed Line2D. The MoH-baseline-reset marker (vertical dashed line + "MoH baseline reset" label) carries over from the prior commit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="9" t="inlineStr">
+        <is>
+          <t>• 2026-05-31 (PM3 run, captions): Refreshed YYYY-MM-DD_caption-x.txt and YYYY-MM-DD_caption-linkedin.txt in the project folder root to reflect the cleaned-baseline cumulative figures (447 sus / 234 conf / 681 total cases; 0 sus deaths / 56 conf deaths) and the 7-day rolling sums under the new schema (+120 cases, +45 deaths). X caption at 251 chars (under 270 limit).</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="9" t="inlineStr">
+        <is>
+          <t>• 2026-05-31 (PM4 run, declarations.csv refresh — surfaced by Web): Audit of declarations.csv against live CDC/WHO sources surfaced several missed events between 2026-05-18 and 2026-05-31. Updates applied: (1) **Uganda CDC Travel Health Notice escalated from Level 1 to Level 2 on 2026-05-27** — explicitly confirmed by the [US Embassy Kampala 28 May health alert](https://ug.usembassy.gov/health-alert-u-s-embassy-kampala-uganda-may-28-2026/) ("On May 27, the U.S. Centers for Disease Control and Prevention (CDC) increased its Travel Health Notice for Ebola Bundibugyo Virus Disease from a Level 1 to Level 2"). cdc_travel_notice_level changed from "Level 1 (Practice Usual Precautions)" to "Level 2 (Practice Enhanced Precautions)"; cdc_travel_notice_url changed from /level1/ebola-uganda to /level2/ebola-uganda. This was missed in the 2026-05-27 PM run, the 2026-05-28 scheduled run, the 2026-05-30 scheduled run, and the 2026-05-31 AM/PM/PM2/PM3 runs — six consecutive runs that recorded "declarations.csv: no change" without re-verifying the live travel-notice index. Procedural lesson: the daily run's declarations check needs to actually fetch the per-country travel-notice URL and verify the level, not just confirm the URL still resolves. The /level1/ebola-uganda URL still resolves but now serves stale content from a prior SVD outbreak. (2) **DRC CDC Travel Notice remains at Level 3** — re-verified via search-result page title ("Ebola Bundibugyo Virus Disease in the Democratic Republic of the Congo - Level 3 - Reconsider Nonessential Travel") and the US Embassy Kampala alert linking the /level3/ DRC URL. No change to DRC's cdc_travel_notice_level / URL. (3) **Africa CDC PHECS declaration on 2026-05-18** (Public Health Emergency of Continental Security) — added to both DRC and Uganda notes fields, sourced to the [Africa CDC statement on US travel restrictions](https://africacdc.org/news-item/u-s-travel-restrictions-related-to-the-bundibugyo-ebola-outbreak/). Schema doesn't have an Africa CDC column; the PHECS is documented in notes for now. (4) **US State Department Travel Advisory at Level 4 (Do Not Travel)** for both DRC and Uganda — distinct from the CDC Travel Health Notice (which is at Level 3 / Level 2 respectively); the State Department advisory is a separate US government advisory at the country level. Added to notes for both rows. (5) **US entry restrictions** on non-US passport holders who travelled to DRC, Uganda, or South Sudan in the previous 21 days, in effect from 2026-05-22 and extended to green-card holders the same week — added to notes for both rows. (6) **CDC Title 42 Order** for arrivals from affected countries — added to notes for both rows with the [CDC media release URL](https://www.cdc.gov/media/releases/2026/statement-update-on-title-42-order.html). (7) **US arrivals from affected countries funneled through IAD (from 2026-05-21), ATL (from 2026-05-22), IAH Houston (from 2026-05-26)** for enhanced screening — added to DRC notes. (8) **WHO/DRC Joint Statement of 2026-05-31** linked in DRC notes for the explicit "borders remain open" ask. (9) **Cases now span 13 health zones** (up from 12 noted in original DRC entry) — updated DRC notes. (10) **Sud-Kivu first lab-confirmed case 2026-05-25** — added to DRC notes (this was logged in the timeseries.csv May 25 primary_source but not surfaced in declarations.csv). Validator passes; no schema change. Note: declarations.csv's current schema does not have columns for US State Department Travel Advisory or Africa CDC PHECS. If these become recurring fields worth tracking with structured cells, the schema should be expanded; for now the notes field carries them.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="114">
+  <mergeCells count="118">
     <mergeCell ref="A130:H130"/>
     <mergeCell ref="A77:H77"/>
     <mergeCell ref="A83:H83"/>
     <mergeCell ref="A49:H49"/>
+    <mergeCell ref="A138:H138"/>
     <mergeCell ref="A132:H132"/>
     <mergeCell ref="A110:H110"/>
     <mergeCell ref="A119:H119"/>
@@ -1959,11 +1988,13 @@
     <mergeCell ref="A88:H88"/>
     <mergeCell ref="A70:H70"/>
     <mergeCell ref="A54:H54"/>
+    <mergeCell ref="A137:H137"/>
     <mergeCell ref="A41:H41"/>
     <mergeCell ref="A90:H90"/>
     <mergeCell ref="A74:H74"/>
     <mergeCell ref="A56:H56"/>
     <mergeCell ref="A26:H26"/>
+    <mergeCell ref="A139:H139"/>
     <mergeCell ref="A71:H71"/>
     <mergeCell ref="A129:H129"/>
     <mergeCell ref="A76:H76"/>
@@ -1997,6 +2028,7 @@
     <mergeCell ref="A46:H46"/>
     <mergeCell ref="A89:H89"/>
     <mergeCell ref="A120:H120"/>
+    <mergeCell ref="A136:H136"/>
     <mergeCell ref="A105:H105"/>
     <mergeCell ref="A57:H57"/>
     <mergeCell ref="A113:H113"/>

</xml_diff>

<commit_message>
Docs/UI: country-add rule in METHODOLOGY; confirmed-deaths column on index.html
Two refresh items surfaced by Web.

1) METHODOLOGY.md: added an explicit 'Adding a country to declarations.csv'
   section with the rule for when a new country gets its own row, plus a
   verification protocol so 'declarations.csv: no change' on a daily run
   means the per-country travel-notice URL was actually fetched and the
   level verified on the page (URL-resolves != level-unchanged; Uganda's
   /level1/ URL kept serving stale SVD content after CDC moved BVD to
   /level2/). Audit on current candidates (South Sudan etc): not in scope
   without their own CDC HAN / Travel Notice / WHO advisory.

2) index.html: added 'Confirmed deaths' headline stat card and 'Conf.
   Deaths' column to the Recent reporting table so the public page reflects
   the new confirmed_deaths_global schema column the charts use. Updated
   colspans (6 -> 7), wired up the render() function, refreshed deaths
   chart alt text.
</commit_message>
<xml_diff>
--- a/outputs/ebola_timeseries.xlsx
+++ b/outputs/ebola_timeseries.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H139"/>
+  <dimension ref="A1:H140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1916,8 +1916,15 @@
         </is>
       </c>
     </row>
+    <row r="140">
+      <c r="A140" s="9" t="inlineStr">
+        <is>
+          <t>• 2026-05-31 (PM5 run, METHODOLOGY.md country-add rule + index.html confirmed-deaths column — surfaced by Web): Two structural updates. (a) Added "Adding a country to declarations.csv" section to METHODOLOGY.md with explicit criteria for when a new country row gets added: own confirmed/suspected cases, OR own country-specific CDC Travel Health Notice, OR own country-specific CDC HAN entry (or multi-country HAN that names the country), OR own WHO country-specific declaration, OR non-US national health authority outbreak-specific advisory with stable primary-source URL. Explicitly clarified that a country appearing in another country's advisory (e.g., South Sudan in the US entry restrictions) does NOT warrant its own row; cross-country effects are captured in the affected countries' notes fields. Also documented the verification protocol on each daily run: a "declarations.csv: no change" report must mean the agent actually fetched the per-country CDC Travel Notice URL and verified the level on the page, plus scanned the CDC Travel Notices index. URL-resolves != level-unchanged (the Uganda /level1/ URL kept serving stale Sudan-virus content after CDC moved BVD to /level2/). Audit of currently-named-in-other-countries' advisories: South Sudan (in US entry restrictions and US State Dept Do Not Travel) does not have its own CDC HAN, CDC Travel Health Notice, or WHO country-specific advisory for this outbreak as of 2026-05-31; no row added. Other countries imposing their own measures (Canada, Bahamas) have their own national-level travel advisories but those are not in scope under the current schema (CDC/WHO only); if Web wants to track non-US national advisories, schema extension is warranted. (b) Updated index.html to surface the new confirmed_deaths_global column: added "Confirmed deaths" headline stat card (5th card; uses the "confirmed" red accent), added "Conf. Deaths" column to the Recent reporting table (between Susp. Deaths and Source), bumped table colspans from 6 to 7 (including the renderError fallback), wired up the new column in the render() function (slug "conf-deaths" → column "confirmed_deaths_global"). Also updated the deaths chart alt text to describe the new stacked structure. The public-facing index.html now reflects the same schema the charts and CSVs use.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="118">
+  <mergeCells count="119">
     <mergeCell ref="A130:H130"/>
     <mergeCell ref="A77:H77"/>
     <mergeCell ref="A83:H83"/>
@@ -2002,6 +2009,7 @@
     <mergeCell ref="A116:H116"/>
     <mergeCell ref="A131:H131"/>
     <mergeCell ref="A100:H100"/>
+    <mergeCell ref="A140:H140"/>
     <mergeCell ref="A53:H53"/>
     <mergeCell ref="A109:H109"/>
     <mergeCell ref="A35:H35"/>

</xml_diff>

<commit_message>
Backfill June 4 (397/65) + June 6 (507/88) rows from BNO daily graphics; add daily-row backfill policy to METHODOLOGY
</commit_message>
<xml_diff>
--- a/outputs/ebola_timeseries.xlsx
+++ b/outputs/ebola_timeseries.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H191"/>
+  <dimension ref="A1:H197"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1196,1217 +1196,1309 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B25" s="4" t="n">
         <v>116</v>
       </c>
       <c r="C25" s="4" t="n">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>516</v>
+        <v>513</v>
       </c>
       <c r="E25" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F25" s="4" t="n">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>[WHO Disease Outbreak News, data as of 5 June 2026] reconciled snapshot: DRC 381 confirmed / 64 confirmed deaths (DRC MoH figures published 4 June, as of 3 June; 233 hospitalised in isolation), across Ituri (359 conf / 17 health zones), North Kivu (19 conf / 7 health zones) and South Kivu (3 conf / 1 health zone). Uganda 19 confirmed / 2 deaths as of 5 June (3 new cases reported 5 June were contacts of confirmed cases; 8 of 9 geolocated cases in Kampala, 1 in Wakiso). Global: suspected 116 (carried forward from 3 June - no updated official suspected figure published in the 5 June WHO DON / Xinhua / CDC sources, all of which led with confirmed; DRC now testing nearly all samples with results within 24h per Health Minister Kamba, draining the suspected backlog), confirmed 400 (DRC 381 + Uganda 19), total 516, suspected_deaths 0 (column zeroed 30 May), confirmed_deaths 66 (DRC 64 + Uganda 2). DRC Health Minister Roger Kamba press briefing 4 June via Xinhua (https://english.news.cn/africa/20260605/75381cda9c1642f7acfdaac060a5bf0f/c.html) cited DRC 381 conf / 63 deaths / 233 hospitalised, contact tracing improved from ~9% to 55% (target 90%), 4,000+ Africa CDC test kits arrived enabling 24h results; WHO DON's 64 DRC conf_deaths used per source-preference (WHO DON &gt; MoH-via-wire, which said 63). vs June 3 (116/359/475/0/61): suspected unchanged, confirmed +41, total +41, conf_deaths +5; cumulative non-decreasing on all columns, no exemption needed. SOURCE-VIEW DIVERGENCE FLAG: BNO @BNOFeed Daily Ebola Update June 5 graphic shows TOTAL 471 confirmed (+74) / 84 deaths (+19) / 12 recovered (+3), a DRC MoH-attributed running wire count ~71 cases / 18 deaths above the WHO-reconciled total (BNO June 4 graphic = 397 conf / 65 deaths matched the official DRC 381 + Uganda 16 sum exactly; BNO June 3 = 378/63). Per source-preference order (WHO DON &gt; BNO News), WHO figures win for the row; BNO running count noted for transparency (same forward-lead pattern as June 1 and June 3). CDC June 5 release (https://www.cdc.gov/media/releases/2026/update-on-ebola-outbreak-in-the-democratic-republic-of-the-congo-and-uganda-6-5-2026.html): three MMWRs - Notes from the Field (largest Bundibugyo outbreak on record; first detected among healthcare-worker clusters), a US risk assessment (risk to general US public low), and CFA modeling (without strong interventions the outbreak could rival or exceed the 2014-2016 West Africa outbreak; &gt;20,000 cases in 2 of 3 simulations at 20% case isolation within 2 days). No WHO Weekly Sitrep 03 yet; DON + briefings remain the reconciliation channel. Catch-up run after June 3 (no June 4 row): the WHO 'as of 5 June' DON is the single reconciled data point and June 4 is not separately rowed (its DRC figure is the same as-of-3-June 381 count, Uganda's increment folds into the 5 June total).</t>
+          <t>BACKFILL (added 2026-06-08 run, daily-row policy): [BNO News @BNOFeed Daily Ebola Update June 4, 2026 graphic](https://x.com/BNOFeed) (MoH DR Congo + MoH Uganda + WHO): DR Congo 381 confirmed (+18) / 64 deaths (+2) / 7 recovered; Uganda 16 confirmed (+1) / 1 death / 2 recovered; TOTAL 397 confirmed (+19) / 65 deaths / 9 recovered. DRC 381/64 matches the WHO DON 'as of 5 June' reconciled DRC figure (published 4 June, as of 3 June), so the DRC component on this date is WHO-corroborated; Uganda 16/1 per Uganda MoH via Xinhua (one new confirmed Thursday 4 June). Global: suspected 116 (carried from 3 June cleaned baseline), confirmed 397 (DRC 381 + Uganda 16), total 513, suspected_deaths 0 (column zeroed 30 May), confirmed_deaths 65 (DRC 64 + Uganda 1). vs 3 June (116/359/475/0/61): confirmed +38, total +38, conf_deaths +4. Cumulative non-decreasing. Row backfilled after the fact: the 4 June scheduled run did not fire (laptop offline) and the 6 June run folded 4 June into the 5 June row. See METHODOLOGY.md 'Backfilling missed days.'</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B26" s="6" t="n">
         <v>116</v>
       </c>
       <c r="C26" s="6" t="n">
+        <v>400</v>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>516</v>
+      </c>
+      <c r="E26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>66</v>
+      </c>
+      <c r="G26" s="7" t="inlineStr">
+        <is>
+          <t>[WHO Disease Outbreak News, data as of 5 June 2026] reconciled snapshot: DRC 381 confirmed / 64 confirmed deaths (DRC MoH figures published 4 June, as of 3 June; 233 hospitalised in isolation), across Ituri (359 conf / 17 health zones), North Kivu (19 conf / 7 health zones) and South Kivu (3 conf / 1 health zone). Uganda 19 confirmed / 2 deaths as of 5 June (3 new cases reported 5 June were contacts of confirmed cases; 8 of 9 geolocated cases in Kampala, 1 in Wakiso). Global: suspected 116 (carried forward from 3 June - no updated official suspected figure published in the 5 June WHO DON / Xinhua / CDC sources, all of which led with confirmed; DRC now testing nearly all samples with results within 24h per Health Minister Kamba, draining the suspected backlog), confirmed 400 (DRC 381 + Uganda 19), total 516, suspected_deaths 0 (column zeroed 30 May), confirmed_deaths 66 (DRC 64 + Uganda 2). DRC Health Minister Roger Kamba press briefing 4 June via Xinhua (https://english.news.cn/africa/20260605/75381cda9c1642f7acfdaac060a5bf0f/c.html) cited DRC 381 conf / 63 deaths / 233 hospitalised, contact tracing improved from ~9% to 55% (target 90%), 4,000+ Africa CDC test kits arrived enabling 24h results; WHO DON's 64 DRC conf_deaths used per source-preference (WHO DON &gt; MoH-via-wire, which said 63). vs June 3 (116/359/475/0/61): suspected unchanged, confirmed +41, total +41, conf_deaths +5; cumulative non-decreasing on all columns, no exemption needed. SOURCE-VIEW DIVERGENCE FLAG: BNO @BNOFeed Daily Ebola Update June 5 graphic shows TOTAL 471 confirmed (+74) / 84 deaths (+19) / 12 recovered (+3), a DRC MoH-attributed running wire count ~71 cases / 18 deaths above the WHO-reconciled total (BNO June 4 graphic = 397 conf / 65 deaths matched the official DRC 381 + Uganda 16 sum exactly; BNO June 3 = 378/63). Per source-preference order (WHO DON &gt; BNO News), WHO figures win for the row; BNO running count noted for transparency (same forward-lead pattern as June 1 and June 3). CDC June 5 release (https://www.cdc.gov/media/releases/2026/update-on-ebola-outbreak-in-the-democratic-republic-of-the-congo-and-uganda-6-5-2026.html): three MMWRs - Notes from the Field (largest Bundibugyo outbreak on record; first detected among healthcare-worker clusters), a US risk assessment (risk to general US public low), and CFA modeling (without strong interventions the outbreak could rival or exceed the 2014-2016 West Africa outbreak; &gt;20,000 cases in 2 of 3 simulations at 20% case isolation within 2 days). No WHO Weekly Sitrep 03 yet; DON + briefings remain the reconciliation channel. Catch-up run after June 3 (no June 4 row): the WHO 'as of 5 June' DON is the single reconciled data point and June 4 is not separately rowed (its DRC figure is the same as-of-3-June 381 count, Uganda's increment folds into the 5 June total).</t>
+        </is>
+      </c>
+      <c r="H26" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="n">
+        <v>116</v>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>507</v>
+      </c>
+      <c r="D27" s="4" t="n">
+        <v>623</v>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="4" t="n">
+        <v>88</v>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>BACKFILL (added 2026-06-08 run, daily-row policy): [BNO News @BNOFeed Daily Ebola Update June 6, 2026 graphic](https://x.com/BNOFeed) (MoH DR Congo + MoH Uganda + WHO): DR Congo 488 confirmed (+36) / 86 deaths (+4) / 9 recovered; Uganda 19 confirmed / 2 deaths / 4 recovered; TOTAL 507 confirmed (+36) / 88 deaths (+4) / 13 recovered. Global: suspected 116 (carried from cleaned baseline), confirmed 507 (DRC 488 + Uganda 19), total 623, suspected_deaths 0 (column zeroed 30 May), confirmed_deaths 88 (DRC 86 + Uganda 2). vs 5 June (116/400/516/0/66): confirmed +107, total +107, conf_deaths +22. SOURCE-VIEW / TIER FLAG: DRC MoH-attributed running wire count; the +107 confirmed vs 5 June is mostly the BNO-vs-WHO instrument gap (5 June is WHO-reconciled DRC 381; 6 June is BNO running DRC 488), not one day of true incidence. WHO has not reconciled the post-5-June DRC count; the BNO running count historically overshoots WHO by ~15-18%, so 488 DRC is provisional and likely revised DOWN at the next WHO reconciliation. Cumulative non-decreasing. Row backfilled because the 6 June scheduled run folded 6 June into the 7 June row. See METHODOLOGY.md 'Backfilling missed days.'</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="n">
+        <v>116</v>
+      </c>
+      <c r="C28" s="6" t="n">
         <v>534</v>
       </c>
-      <c r="D26" s="6" t="n">
+      <c r="D28" s="6" t="n">
         <v>650</v>
       </c>
-      <c r="E26" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F26" s="6" t="n">
+      <c r="E28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F28" s="6" t="n">
         <v>93</v>
       </c>
-      <c r="G26" s="7" t="inlineStr">
+      <c r="G28" s="7" t="inlineStr">
         <is>
           <t>[BNO News @BNOFeed Daily Ebola Update June 7, 2026 graphic](https://x.com/BNOFeed) (sourced to MoH DR Congo + MoH Uganda + WHO): DR Congo 515 confirmed (+27) / 91 confirmed deaths (+5) / 12 recovered; Uganda 19 confirmed / 2 deaths / 4 recovered; TOTAL 534 confirmed (+27) / 93 deaths (+5) / 16 recovered. Global: suspected 116 (carried forward from 5 June WHO DON cleaned baseline; BNO tracks confirmed only, no fresh official suspected figure published 6-8 June), confirmed 534 (DRC 515 + Uganda 19), total 650, suspected_deaths 0 (column zeroed 30 May), confirmed_deaths 93 (DRC 91 + Uganda 2). vs 5 June (116/400/516/0/66): suspected unchanged, confirmed +134, total +134, conf_deaths +27; cumulative non-decreasing on all columns. CATCH-UP: folds in the 6 June BNO graphic (DRC 488 conf / 86 deaths; Uganda 19/2; TOTAL 507 conf / 88 deaths / 13 recovered) as the intermediate cumulative point; the single 7 June row carries the latest cumulative snapshot. SOURCE-VIEW / TIER FLAG: DRC MoH + Uganda MoH attributed running wire count carried by BNO; no WHO Weekly Sitrep 03 / DON606 / CDC reconciliation has published for 6-8 June (last WHO-reconciled point is the 5 June DON at DRC 381 / 64). Per METHODOLOGY.md source-preference order, BNO News is the designated fallback when nothing higher-tier is fresher (precedent: the 30-31 May BNO-sourced rows). The BNO running count has historically overshot the later WHO reconciliation by ~15-18% (1 Jun BNO 352 conf -&gt; WHO 330; 5 Jun BNO 471 -&gt; WHO 400), so the 7 June confirmed figure is provisional and likely to be revised DOWN when WHO/CDC next reconcile; under the no-dip rule that future dip would need the WHO+CDC two-source threshold (typically met). Bars provisional on charts (post-24-May hatching).</t>
         </is>
       </c>
-      <c r="H26" s="7" t="inlineStr">
+      <c r="H28" s="7" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="8" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="8" t="inlineStr">
         <is>
           <t>NOTES</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="9" t="inlineStr">
-        <is>
-          <t>• "Suspected Cases" includes all clinically suspected cases reported by DRC MoH; many are unconfirmed by lab testing.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="9" t="inlineStr">
-        <is>
-          <t>• "Confirmed Cases" = laboratory-confirmed Bundibugyo virus by PCR at INRB or partner labs.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="9" t="inlineStr">
         <is>
-          <t>• Death counts are "suspected deaths" — most have not been lab-confirmed. True CFR is uncertain.</t>
+          <t>• "Suspected Cases" includes all clinically suspected cases reported by DRC MoH; many are unconfirmed by lab testing.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="9" t="inlineStr">
         <is>
-          <t>• Uganda confirmed cases stood at 2 (both imported from DRC) through May 22; on May 23 Uganda MoH confirmed 3 additional cases (a health worker, a driver linked to the index patient, and a returning Congolese traveler), bringing the total to 5. The health-worker case indicates probable secondary local transmission in Uganda.</t>
+          <t>• "Confirmed Cases" = laboratory-confirmed Bundibugyo virus by PCR at INRB or partner labs.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="9" t="inlineStr">
         <is>
-          <t>• On May 21, CDC revised the May 20 total down from 675 to 626 as suspected cases were reclassified.</t>
+          <t>• Death counts are "suspected deaths" — most have not been lab-confirmed. True CFR is uncertain.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="9" t="inlineStr">
         <is>
-          <t>• Figures may differ slightly between sources due to reporting lag and retroactive reclassification.</t>
+          <t>• Uganda confirmed cases stood at 2 (both imported from DRC) through May 22; on May 23 Uganda MoH confirmed 3 additional cases (a health worker, a driver linked to the index patient, and a returning Congolese traveler), bringing the total to 5. The health-worker case indicates probable secondary local transmission in Uganda.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>• The outbreak was officially declared May 15; earliest known symptom onset was April 24, 2026.</t>
+          <t>• On May 21, CDC revised the May 20 total down from 675 to 626 as suspected cases were reclassified.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>• Sources: BNO News (bnonews.com), WHO Disease Outbreak News, CDC Ebola Situation Summary, Africa CDC, DRC MoH.</t>
+          <t>• Figures may differ slightly between sources due to reporting lag and retroactive reclassification.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-23: May 21 row revised per WHO DON603 (data as of 21 May): suspected 671→746, confirmed 64→85, deaths 166→176. WHO's reconciled figures published the next day exceeded BNO News's same-day reporting.</t>
+          <t>• The outbreak was officially declared May 15; earliest known symptom onset was April 24, 2026.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>• Column I 'Source Timestamp' shows the source's 'as of' date for each row. Each daily run re-checks the last 7 rows against the latest WHO/CDC/Africa CDC/BNO reports and applies revisions in place; revisions are logged here.</t>
+          <t>• Sources: BNO News (bnonews.com), WHO Disease Outbreak News, CDC Ebola Situation Summary, Africa CDC, DRC MoH.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-23: May 18 row revised to WHO AFRO Weekly Sitrep 01 (data as of 18 May): suspected 395→528, deaths 106→132. Confirmed left at 33 (BNO); Sitrep didn't publish a confirmed-cases breakdown for that date.</t>
+          <t>• 2026-05-23: May 21 row revised per WHO DON603 (data as of 21 May): suspected 671→746, confirmed 64→85, deaths 166→176. WHO's reconciled figures published the next day exceeded BNO News's same-day reporting.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>• Source preference order, in effect 2026-05-23: WHO Sitrep &gt; WHO DON &gt; CDC Situation Summary &gt; Africa CDC &gt; BNO News. WHO can revise downward; the daily-delta chart will sometimes show negative bars.</t>
+          <t>• Column I 'Source Timestamp' shows the source's 'as of' date for each row. Each daily run re-checks the last 7 rows against the latest WHO/CDC/Africa CDC/BNO reports and applies revisions in place; revisions are logged here.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-23: Updated the Uganda-note (originally written as-of May 22) to reflect Uganda MoH's May 23 confirmation of 3 additional cases, including likely local secondary transmission. Old text: 'Uganda confirmed cases (2) are imported from DRC; no onward transmission reported in Uganda as of May 22.'</t>
+          <t>• 2026-05-23: May 18 row revised to WHO AFRO Weekly Sitrep 01 (data as of 18 May): suspected 395→528, deaths 106→132. Confirmed left at 33 (BNO); Sitrep didn't publish a confirmed-cases breakdown for that date.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-23 (PM run): No new figures published since the morning row; sources unchanged (CIDRAP citing WHO/ABC + Uganda MoH still latest). Cumulative observed upward revisions across NOTES history span ~+6% to ~+34% (computed: May 18 sus +33.7%, May 18 deaths +24.5%, May 21 sus +11.2%, May 21 conf +32.8%, May 21 deaths +6.0%). Updated OBSERVED_REVISION_RANGE in generate_charts.py from '10-30%' to '5-35%' to bracket the observed values with small margin.</t>
+          <t>• Source preference order, in effect 2026-05-23: WHO Sitrep &gt; WHO DON &gt; CDC Situation Summary &gt; Africa CDC &gt; BNO News. WHO can revise downward; the daily-delta chart will sometimes show negative bars.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-23 (evening run): No material change since morning. Al Jazeera report (publ. May 23, last updated 16:48 UTC) confirms 'Nearly 750 suspected cases and 177 suspected deaths' in DRC and Uganda's total at 5 confirmed. WHO DON603 (May 21) and CIDRAP coverage of the May 22 Tedros briefing remain the latest reconciled figures. No WHO Sitrep 02 published yet. Cumulative totals unchanged.</t>
+          <t>• 2026-05-23: Updated the Uganda-note (originally written as-of May 22) to reflect Uganda MoH's May 23 confirmation of 3 additional cases, including likely local secondary transmission. Old text: 'Uganda confirmed cases (2) are imported from DRC; no onward transmission reported in Uganda as of May 22.'</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-24 (AM run): No new figures published since the 2026-05-23 PM run. Primary sources unchanged: WHO AFRO Sitrep 01 (data as of 18 May), WHO DON603 (data as of 21 May), CDC Situation Summary (last revised 16 May), and the 22 May Tedros media briefing remain the latest reconciled snapshots. Al Jazeera (23 May) and CIDRAP coverage of the 22 May Tedros briefing both continue to cite ~750 suspected cases / 177 suspected deaths in DRC + Uganda's 5 confirmed cases. Wikipedia currently lists '836 suspected, 186 deaths as of 22 May,' but no primary WHO/CDC/Africa CDC source publishes that figure with that timestamp; per source preference order, no revision applied pending higher-confidence confirmation. Cumulative totals unchanged. 7-day lookback against last 7 rows: no revisions required.</t>
+          <t>• 2026-05-23 (PM run): No new figures published since the morning row; sources unchanged (CIDRAP citing WHO/ABC + Uganda MoH still latest). Cumulative observed upward revisions across NOTES history span ~+6% to ~+34% (computed: May 18 sus +33.7%, May 18 deaths +24.5%, May 21 sus +11.2%, May 21 conf +32.8%, May 21 deaths +6.0%). Updated OBSERVED_REVISION_RANGE in generate_charts.py from '10-30%' to '5-35%' to bracket the observed values with small margin.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-24 (PM run): New row appended for 2026-05-24 based on DRC Ministry of Health statement released late Saturday 23 May (via AFP wire, carried by Citizen Digital and NPR/GPB on 24 May): 867 suspected cases and 204 suspected deaths across Ituri, Nord-Kivu, and Sud-Kivu provinces. Compared with the prior WHO toll (Friday: 750 sus / 177 deaths), this is +117 sus cases (+15.6%) and +27 sus deaths (+15.3%). Uganda unchanged at 5 confirmed / 1 death. Confirmed-case figure (87) carried forward from May 23; no higher-tier source has published a fresh DRC+Uganda confirmed breakdown since DON603 (data as of 21 May, confirmed=85) and the May 22 Tedros briefing. No new WHO Sitrep 02 yet. 7-day lookback against last 7 rows: no revisions required from higher-tier sources.</t>
+          <t>• 2026-05-23 (evening run): No material change since morning. Al Jazeera report (publ. May 23, last updated 16:48 UTC) confirms 'Nearly 750 suspected cases and 177 suspected deaths' in DRC and Uganda's total at 5 confirmed. WHO DON603 (May 21) and CIDRAP coverage of the May 22 Tedros briefing remain the latest reconciled figures. No WHO Sitrep 02 published yet. Cumulative totals unchanged.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-24 (scope change): Renamed main-sheet column headers from "(DRC+Uganda)" to "(Global)" to make the tracker country-agnostic. Historical values unchanged. Uganda-specific columns (F, G) preserved as the operationally salient cross-border detail. Added a "Country Breakdown" sheet (long format: Date x Country x counts) pre-populated with derived DRC + Uganda rows. When a new country reports cases, add them to the global totals on the main sheet AND add per-country rows on the Country Breakdown sheet. NOTE: The American citizen who tested positive in DRC on May 17 and was medevaced to Germany is presumed counted in the DRC tally per WHO convention (country of exposure). If WHO begins splitting "in-country" vs "exported" cases, the breakdown sheet should track this explicitly.</t>
+          <t>• 2026-05-24 (AM run): No new figures published since the 2026-05-23 PM run. Primary sources unchanged: WHO AFRO Sitrep 01 (data as of 18 May), WHO DON603 (data as of 21 May), CDC Situation Summary (last revised 16 May), and the 22 May Tedros media briefing remain the latest reconciled snapshots. Al Jazeera (23 May) and CIDRAP coverage of the 22 May Tedros briefing both continue to cite ~750 suspected cases / 177 suspected deaths in DRC + Uganda's 5 confirmed cases. Wikipedia currently lists '836 suspected, 186 deaths as of 22 May,' but no primary WHO/CDC/Africa CDC source publishes that figure with that timestamp; per source preference order, no revision applied pending higher-confidence confirmation. Cumulative totals unchanged. 7-day lookback against last 7 rows: no revisions required.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-25 (AM run): New row appended for 2026-05-25 based on BNO News (May 25) summary of the DRC Ministry of Health update. DRC reports 867 suspected cases (unchanged from May 23 MoH statement) and 91 lab-confirmed cases (up from 82 carried-forward in the country breakdown), bringing global confirmed to 96 (91 DRC + 5 Uganda). Global confirmed: 87 → 96 (+10.3%). Suspected deaths held at 204 per DRC MoH; BNO additionally reports 10 confirmed deaths in DRC, kept out of col E to preserve the historical 'suspected deaths' definition and flagged here for transparency. Country Breakdown sheet records the 10 confirmed DRC deaths in col F. Uganda unchanged at 5 confirmed / 1 death. Outbreak now spans 12 health zones across Ituri, Nord-Kivu, Sud-Kivu provinces. BNO's headline 'more than 960 cases / 216 deaths' implies a +1 Uganda death not corroborated by Uganda MoH or CDC; treating as a BNO summary rounding pending confirmation. 7-day lookback against last 7 rows: no revisions required from higher-tier sources (no WHO Sitrep 02 published; latest WHO DON603 is data as of 21 May).</t>
+          <t>• 2026-05-24 (PM run): New row appended for 2026-05-24 based on DRC Ministry of Health statement released late Saturday 23 May (via AFP wire, carried by Citizen Digital and NPR/GPB on 24 May): 867 suspected cases and 204 suspected deaths across Ituri, Nord-Kivu, and Sud-Kivu provinces. Compared with the prior WHO toll (Friday: 750 sus / 177 deaths), this is +117 sus cases (+15.6%) and +27 sus deaths (+15.3%). Uganda unchanged at 5 confirmed / 1 death. Confirmed-case figure (87) carried forward from May 23; no higher-tier source has published a fresh DRC+Uganda confirmed breakdown since DON603 (data as of 21 May, confirmed=85) and the May 22 Tedros briefing. No new WHO Sitrep 02 yet. 7-day lookback against last 7 rows: no revisions required from higher-tier sources.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-25 (PM run): Material updates since AM run. (1) Uganda MoH (Dr Olaro Charles, Director General of Health Services) press release confirmed 2 new EVD cases in Kampala (both health workers at a private healthcare facility, currently in isolation/treatment). Uganda confirmed: 5 → 7. No new deaths; Uganda total stands at 7 confirmed / 1 death. (2) DRC government figures released Sunday May 24 (per Reuters/AP wires, corroborated by CNN, UN News, NPR): 904 suspected cases, 101 confirmed, 119 suspected deaths, 10 confirmed deaths. These DRC numbers supersede the BNO News (May 25) figures (867 sus / 91 conf / 204 sus deaths) used in the AM run, per source-preference order (wire reports citing DRC government attribution &gt; BNO News).</t>
+          <t>• 2026-05-24 (scope change): Renamed main-sheet column headers from "(DRC+Uganda)" to "(Global)" to make the tracker country-agnostic. Historical values unchanged. Uganda-specific columns (F, G) preserved as the operationally salient cross-border detail. Added a "Country Breakdown" sheet (long format: Date x Country x counts) pre-populated with derived DRC + Uganda rows. When a new country reports cases, add them to the global totals on the main sheet AND add per-country rows on the Country Breakdown sheet. NOTE: The American citizen who tested positive in DRC on May 17 and was medevaced to Germany is presumed counted in the DRC tally per WHO convention (country of exposure). If WHO begins splitting "in-country" vs "exported" cases, the breakdown sheet should track this explicitly.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-25 (PM run) — May 24 row revised per Reuters/AP wires citing DRC govt Sunday update: suspected 867→904 (+4.3%), confirmed 87→101 (+16.1%), suspected deaths 204→119 (-41.7%, reclassification removing non-Ebola deaths). Uganda unchanged at 5 confirmed / 1 death. Total cases 954→1010.</t>
+          <t>• 2026-05-25 (AM run): New row appended for 2026-05-25 based on BNO News (May 25) summary of the DRC Ministry of Health update. DRC reports 867 suspected cases (unchanged from May 23 MoH statement) and 91 lab-confirmed cases (up from 82 carried-forward in the country breakdown), bringing global confirmed to 96 (91 DRC + 5 Uganda). Global confirmed: 87 → 96 (+10.3%). Suspected deaths held at 204 per DRC MoH; BNO additionally reports 10 confirmed deaths in DRC, kept out of col E to preserve the historical 'suspected deaths' definition and flagged here for transparency. Country Breakdown sheet records the 10 confirmed DRC deaths in col F. Uganda unchanged at 5 confirmed / 1 death. Outbreak now spans 12 health zones across Ituri, Nord-Kivu, Sud-Kivu provinces. BNO's headline 'more than 960 cases / 216 deaths' implies a +1 Uganda death not corroborated by Uganda MoH or CDC; treating as a BNO summary rounding pending confirmation. 7-day lookback against last 7 rows: no revisions required from higher-tier sources (no WHO Sitrep 02 published; latest WHO DON603 is data as of 21 May).</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-25 (PM run) — May 25 row revised: DRC carries Sunday May 24 figures forward (no newer DRC MoH statement): suspected 867→904, confirmed (DRC component) 91→101, suspected deaths 204→119. Uganda confirmed 5→7 per Uganda MoH May 25 press release. Global confirmed 96→108, total cases 963→1012.</t>
+          <t>• 2026-05-25 (PM run): Material updates since AM run. (1) Uganda MoH (Dr Olaro Charles, Director General of Health Services) press release confirmed 2 new EVD cases in Kampala (both health workers at a private healthcare facility, currently in isolation/treatment). Uganda confirmed: 5 → 7. No new deaths; Uganda total stands at 7 confirmed / 1 death. (2) DRC government figures released Sunday May 24 (per Reuters/AP wires, corroborated by CNN, UN News, NPR): 904 suspected cases, 101 confirmed, 119 suspected deaths, 10 confirmed deaths. These DRC numbers supersede the BNO News (May 25) figures (867 sus / 91 conf / 204 sus deaths) used in the AM run, per source-preference order (wire reports citing DRC government attribution &gt; BNO News).</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-25 (PM run) — Downward reclassification observed: DRC suspected deaths fell from 204 to 119 in the Sunday May 24 government update (-41.7%). This is the first material downward revision in the cumulative history and reflects DRC MoH/WHO reclassification of non-Ebola deaths out of the 'suspected deaths' category. The 10 confirmed deaths figure remains separate and is tracked in the Country Breakdown sheet. The OBSERVED_REVISION_RANGE in generate_charts.py was widened from '5-35%' to '4-35%' to bracket the new +4.3% lower bound (May 24 suspected); the chart-footnote text continues to describe upward revisions only, which is the historical pattern except for this single reclassification event.</t>
+          <t>• 2026-05-25 (PM run) — May 24 row revised per Reuters/AP wires citing DRC govt Sunday update: suspected 867→904 (+4.3%), confirmed 87→101 (+16.1%), suspected deaths 204→119 (-41.7%, reclassification removing non-Ebola deaths). Uganda unchanged at 5 confirmed / 1 death. Total cases 954→1010.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-25 (PM run, xcancel pass): Per Helen Branswell (STAT) and Krutika Kuppalli, MD FIDSA on X: the two new Uganda health-worker cases reportedly have uncertain exposure histories. They may not have cared for previously-known Uganda cases, which would imply undetected community transmission in Kampala. Not yet confirmed by Uganda MoH press materials, but worth tracking. No numerical change applied.</t>
+          <t>• 2026-05-25 (PM run) — May 25 row revised: DRC carries Sunday May 24 figures forward (no newer DRC MoH statement): suspected 867→904, confirmed (DRC component) 91→101, suspected deaths 204→119. Uganda confirmed 5→7 per Uganda MoH May 25 press release. Global confirmed 96→108, total cases 963→1012.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-25 (PM run, xcancel pass): BNO News @BNOFeed (citing RFI), corroborated by another wire-style account, reports that 7 Ebola patients escaped from a hospital in Mongbwalu (Ituri Province, DRC) after the facility was attacked by angry relatives. BNO calls it the 3rd such incident in recent days. Direct operational impact: these patients are now in the community and untraced. No primary WHO/DRC MoH confirmation yet; logged for transparency. Worth checking for in next run.</t>
+          <t>• 2026-05-25 (PM run) — Downward reclassification observed: DRC suspected deaths fell from 204 to 119 in the Sunday May 24 government update (-41.7%). This is the first material downward revision in the cumulative history and reflects DRC MoH/WHO reclassification of non-Ebola deaths out of the 'suspected deaths' category. The 10 confirmed deaths figure remains separate and is tracked in the Country Breakdown sheet. The OBSERVED_REVISION_RANGE in generate_charts.py was widened from '5-35%' to '4-35%' to bracket the new +4.3% lower bound (May 24 suspected); the chart-footnote text continues to describe upward revisions only, which is the historical pattern except for this single reclassification event.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-25 (PM run, xcancel pass): WHO Director-General Tedros, per a French wire (Cerfia citing OMS chief), reportedly said 'l'épidémie nous dépasse' ('the epidemic is overwhelming us') in remarks today, alongside a figure of 'at least 220 suspected Ebola deaths' across DRC and Uganda combined. The 220 figure is materially higher than the 119 suspected deaths in our May 24/25 rows (post-Sunday DRC reclassification) and aligns with the earlier CNN figure of '220 deaths thought to be linked'. Possible interpretations: (a) pre-reclassification gross count, (b) different inclusion criteria, (c) post-Sunday upward trend. No WHO primary source has published the 220 figure with a dated 'as of' attribution. NOT applying as a revision; flagging for next-run reconciliation when WHO Sitrep 02 or DON604 publishes.</t>
+          <t>• 2026-05-25 (PM run, xcancel pass): Per Helen Branswell (STAT) and Krutika Kuppalli, MD FIDSA on X: the two new Uganda health-worker cases reportedly have uncertain exposure histories. They may not have cared for previously-known Uganda cases, which would imply undetected community transmission in Kampala. Not yet confirmed by Uganda MoH press materials, but worth tracking. No numerical change applied.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-25 (PM run, xcancel pass): India's Directorate General of Civil Aviation (DGCA) issued an SOP for travelers arriving from DRC and Uganda, per @jagritichandra (The Hindu). Includes mandatory passenger declarations and segregated seating for suspected cases on Indian carriers. New cross-border preparedness signal; informational, no impact on case counts.</t>
+          <t>• 2026-05-25 (PM run, xcancel pass): BNO News @BNOFeed (citing RFI), corroborated by another wire-style account, reports that 7 Ebola patients escaped from a hospital in Mongbwalu (Ituri Province, DRC) after the facility was attacked by angry relatives. BNO calls it the 3rd such incident in recent days. Direct operational impact: these patients are now in the community and untraced. No primary WHO/DRC MoH confirmation yet; logged for transparency. Worth checking for in next run.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-25 (PM run, methodology change per Web): Adopted a 'no-dip' rule for cumulative figures. Cumulative metrics (suspected cases, confirmed cases, total cases, suspected deaths) are monotonically non-decreasing. When a source proposes a downward revision, the previous higher value is carried forward UNLESS multiple independent high-value sources confirm the dip. High-value sources: WHO official publications (Sitrep, DON); WHO Director-General statements (briefings, press conferences) even when not yet in a WHO document; DRC MoH official press releases; Uganda MoH official press releases; CDC publications. Single-source dips (e.g., a DRC MoH reclassification carried only by one wire) are held in NOTES pending corroboration. Upward revisions follow normal source-preference rules. Rationale: cumulative drops confuse general readers and almost always reflect definitional changes rather than actual recoveries.</t>
+          <t>• 2026-05-25 (PM run, xcancel pass): WHO Director-General Tedros, per a French wire (Cerfia citing OMS chief), reportedly said 'l'épidémie nous dépasse' ('the epidemic is overwhelming us') in remarks today, alongside a figure of 'at least 220 suspected Ebola deaths' across DRC and Uganda combined. The 220 figure is materially higher than the 119 suspected deaths in our May 24/25 rows (post-Sunday DRC reclassification) and aligns with the earlier CNN figure of '220 deaths thought to be linked'. Possible interpretations: (a) pre-reclassification gross count, (b) different inclusion criteria, (c) post-Sunday upward trend. No WHO primary source has published the 220 figure with a dated 'as of' attribution. NOT applying as a revision; flagging for next-run reconciliation when WHO Sitrep 02 or DON604 publishes.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-25 (PM run, applying no-dip rule): Reverted the earlier PM-run revision of May 24 and May 25 suspected-deaths from 204 → 119. The 119 figure (DRC Sunday govt reclassification via Reuters/AP) is a single-source downward proposal not corroborated by other high-value sources. WHO DG Tedros today reportedly cited 'at least 220 suspected Ebola deaths' across DRC + Uganda (per French wire Cerfia citing OMS chief), which contradicts the dip and serves as a high-value upward revision. New values: May 24 suspected deaths 119 → 220 (+85% from PM-run dip, +7.8% from pre-AM-run 204); May 25 suspected deaths 119 → 220 (same). DRC confirmed-cases (101) and confirmed-deaths (10) from the same Sunday update remain in place as upward revisions (no dip issue). The 119 figure is preserved in this NOTES history as the DRC MoH per-source value; if WHO Sitrep 02 or DON604 later confirms the 119 reclassification, the no-dip rule allows applying the dip at that point with multi-source backing.</t>
+          <t>• 2026-05-25 (PM run, xcancel pass): India's Directorate General of Civil Aviation (DGCA) issued an SOP for travelers arriving from DRC and Uganda, per @jagritichandra (The Hindu). Includes mandatory passenger declarations and segregated seating for suspected cases on Indian carriers. New cross-border preparedness signal; informational, no impact on case counts.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-25 (PM run, final state): May 24 row: 904 sus / 106 conf / 1010 total / 220 sus deaths; Uganda 5/1. May 25 row: 904 sus / 108 conf / 1012 total / 220 sus deaths; Uganda 7/1. Cumulative deaths line now rises monotonically: 177 (May 23) → 220 (May 24) → 220 (May 25). 7-day rolling sums recomputed: May 25 = +376 sus, +75 conf, +88 deaths.</t>
+          <t>• 2026-05-25 (PM run, methodology change per Web): Adopted a 'no-dip' rule for cumulative figures. Cumulative metrics (suspected cases, confirmed cases, total cases, suspected deaths) are monotonically non-decreasing. When a source proposes a downward revision, the previous higher value is carried forward UNLESS multiple independent high-value sources confirm the dip. High-value sources: WHO official publications (Sitrep, DON); WHO Director-General statements (briefings, press conferences) even when not yet in a WHO document; DRC MoH official press releases; Uganda MoH official press releases; CDC publications. Single-source dips (e.g., a DRC MoH reclassification carried only by one wire) are held in NOTES pending corroboration. Upward revisions follow normal source-preference rules. Rationale: cumulative drops confuse general readers and almost always reflect definitional changes rather than actual recoveries.</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-25 (evening run): No new high-tier figures published since the PM run. WHO outbreak page still lists DON603 (data as of 21 May), WHO AFRO Sitrep 01 (data as of 18 May), and the 22 May Tedros media briefing as the most recent reconciled publications; no Sitrep 02 or DON604 yet. CDC Situation Summary still dated 16 May. Tedros's 25 May remarks ("at least 220 suspected deaths"; "the epidemic is outpacing us") are now corroborated across multiple credentialed wires (Al Jazeera, Euronews, Xinhua, CNBC Africa) — the 220 figure already carried in the May 24 and May 25 rows under the no-dip rule. 7-day lookback against last 7 rows (May 19–25): no revisions required. xcancel real-time pass skipped on this unattended run (browser-select flow requires user input). Charts and XLSX regenerated; output filenames unchanged (most-recent Report Date still 2026-05-25).</t>
+          <t>• 2026-05-25 (PM run, applying no-dip rule): Reverted the earlier PM-run revision of May 24 and May 25 suspected-deaths from 204 → 119. The 119 figure (DRC Sunday govt reclassification via Reuters/AP) is a single-source downward proposal not corroborated by other high-value sources. WHO DG Tedros today reportedly cited 'at least 220 suspected Ebola deaths' across DRC + Uganda (per French wire Cerfia citing OMS chief), which contradicts the dip and serves as a high-value upward revision. New values: May 24 suspected deaths 119 → 220 (+85% from PM-run dip, +7.8% from pre-AM-run 204); May 25 suspected deaths 119 → 220 (same). DRC confirmed-cases (101) and confirmed-deaths (10) from the same Sunday update remain in place as upward revisions (no dip issue). The 119 figure is preserved in this NOTES history as the DRC MoH per-source value; if WHO Sitrep 02 or DON604 later confirms the 119 reclassification, the no-dip rule allows applying the dip at that point with multi-source backing.</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-25 (schema change, declarations.csv): Added two columns to distinguish CDC's clinician-facing HAN advisory from its traveler-facing Travel Health Notice. New schema: `country, first_report_date, case_status, cdc_advisory, cdc_url, cdc_travel_notice_level, cdc_travel_notice_url, who_status, who_url, notes`. Backfilled both rows: DRC at Level 3 (Reconsider Nonessential Travel, https://wwwnc.cdc.gov/travel/notices/level3/ebola-democratic-republic-of-the-congo), Uganda at Level 1 (Practice Usual Precautions, https://wwwnc.cdc.gov/travel/notices/level1/ebola-uganda). Note: CDC has escalated DRC from Level 2 to Level 3 since the 2026-05-16 CDC Situation Summary publication, which still links to the Level 2 page. METHODOLOGY.md updated to document the new schema and the two-system distinction. Daily-task SKILL.md updated to instruct future runs to check the per-country travel-notice URLs each pass.</t>
+          <t>• 2026-05-25 (PM run, final state): May 24 row: 904 sus / 106 conf / 1010 total / 220 sus deaths; Uganda 5/1. May 25 row: 904 sus / 108 conf / 1012 total / 220 sus deaths; Uganda 7/1. Cumulative deaths line now rises monotonically: 177 (May 23) → 220 (May 24) → 220 (May 25). 7-day rolling sums recomputed: May 25 = +376 sus, +75 conf, +88 deaths.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-25 (index.html render): Added a "CDC travel notice" column to the public declarations table on index.html, positioned between "CDC advisory" (HAN) and "WHO status" so the two CDC systems read left to right. Cell shows the level + meaning (e.g., "Level 3 (Reconsider Nonessential Travel)") and links to the matching wwwnc.cdc.gov page. Empty `cdc_travel_notice_level` cells fall back to a blank cell. Colspan on the loading and empty-state rows bumped from 6 to 7.</t>
+          <t>• 2026-05-25 (evening run): No new high-tier figures published since the PM run. WHO outbreak page still lists DON603 (data as of 21 May), WHO AFRO Sitrep 01 (data as of 18 May), and the 22 May Tedros media briefing as the most recent reconciled publications; no Sitrep 02 or DON604 yet. CDC Situation Summary still dated 16 May. Tedros's 25 May remarks ("at least 220 suspected deaths"; "the epidemic is outpacing us") are now corroborated across multiple credentialed wires (Al Jazeera, Euronews, Xinhua, CNBC Africa) — the 220 figure already carried in the May 24 and May 25 rows under the no-dip rule. 7-day lookback against last 7 rows (May 19–25): no revisions required. xcancel real-time pass skipped on this unattended run (browser-select flow requires user input). Charts and XLSX regenerated; output filenames unchanged (most-recent Report Date still 2026-05-25).</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-25 (validator + retroactive no-dip cleanup): Added src/validate.py as a pre-commit gate that enforces schema, monotonic cumulative columns, total = sus + conf, country-sum-equals-global on the latest date, date format/uniqueness. First run caught four legacy no-dip violations from partial revision reconciliation. Applied retroactive cleanup per the rule as written in METHODOLOGY.md: May 19 row carried forward from revised May 18 (WHO Sitrep 01): suspected 516→528, total 549→561, suspected_deaths 131→132. May 22 row carried forward from revised May 21 (WHO DON603): suspected 744→746, confirmed 83→85, total 827→831. The May 22 lift cascaded into May 23: DRC confirmed bumped 82→83 to stay non-decreasing, lifting global confirmed 87→88 and total 837→838. country_breakdown.csv DRC rows updated to match: May 19 DRC suspected 516→528, suspected_deaths 131→132; May 22 DRC suspected 744→746, confirmed 81→83; May 23 DRC confirmed 82→83. All primary_source fields amended to flag the carry-forward and record the same-day source's original figures for audit. May 24 and May 25 rows unaffected. Validator now passes clean.</t>
+          <t>• 2026-05-25 (schema change, declarations.csv): Added two columns to distinguish CDC's clinician-facing HAN advisory from its traveler-facing Travel Health Notice. New schema: `country, first_report_date, case_status, cdc_advisory, cdc_url, cdc_travel_notice_level, cdc_travel_notice_url, who_status, who_url, notes`. Backfilled both rows: DRC at Level 3 (Reconsider Nonessential Travel, https://wwwnc.cdc.gov/travel/notices/level3/ebola-democratic-republic-of-the-congo), Uganda at Level 1 (Practice Usual Precautions, https://wwwnc.cdc.gov/travel/notices/level1/ebola-uganda). Note: CDC has escalated DRC from Level 2 to Level 3 since the 2026-05-16 CDC Situation Summary publication, which still links to the Level 2 page. METHODOLOGY.md updated to document the new schema and the two-system distinction. Daily-task SKILL.md updated to instruct future runs to check the per-country travel-notice URLs each pass.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-25 (late-evening run): No new numerical figures since the evening run. Citation upgrade applied to May 24 and May 25 rows: WHO DG Tedros's [remarks at the Virtual Ministerial Briefing on the Bundibugyo Ebola Outbreak](https://www.who.int/news-room/speeches/item/who-director-general-s-remarks-at-the-virtual-ministerial-briefing-on-the-bundibugyo-ebola-outbreak-25-may-2026) (25 May 2026) now serve as the primary source for the DRC figures (904 sus / 101 conf / 220 sus deaths / 10 conf deaths). This is a WHO-DG-attributed primary source, higher-tier than the Reuters/AP wires previously cited; corroborated by [UN News (25 May)](https://news.un.org/en/story/2026/05/1167584) and Xinhua. Uganda figures still cite Uganda MoH May 25 press release (+2 health workers in Kampala, total 7 conf / 1 death). The Tedros briefing gave 5 confirmed for Uganda; that figure predates the Uganda MoH same-day +2 release. Per source-preference, the Uganda national MoH remains the authoritative source for Uganda's count. WHO Sitrep 02 and WHO DON604 still not published. CDC Situation Summary still dated 16 May with stale figures; DRC travel notice remains Level 3 (Reconsider Nonessential Travel). 7-day lookback against May 19–25: no numerical revisions required. story.md "Latest update" refreshed to incorporate the WHO DG quote ("the epidemic is outpacing us"), DRC national risk upgraded from "high" to "very high", two treatment centers set alight in eastern DRC, 100,000+ displaced by fighting, $3.9M WHO Contingency Fund release, and WHO clinical-trial prioritization of two monoclonal antibodies + obeldesivir. No declarations.csv change (national risk upgrade is a WHO statement, not a formal declaration change; PHEIC level unchanged). Charts and XLSX regenerated; output filenames unchanged (most-recent Report Date still 2026-05-25).</t>
+          <t>• 2026-05-25 (index.html render): Added a "CDC travel notice" column to the public declarations table on index.html, positioned between "CDC advisory" (HAN) and "WHO status" so the two CDC systems read left to right. Cell shows the level + meaning (e.g., "Level 3 (Reconsider Nonessential Travel)") and links to the matching wwwnc.cdc.gov page. Empty `cdc_travel_notice_level` cells fall back to a blank cell. Colspan on the loading and empty-state rows bumped from 6 to 7.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-26 (methodology change, Real-time signal source): Switched the Real-time signal source from xcancel.com to x.com via Web's signed-in Chrome. Trigger: xcancel.com served an active anti-bot challenge during the 2026-05-26 AM run, blocking the unattended xcancel pass; meanwhile Web's local Chrome is signed in to x.com and the Claude in Chrome MCP can drive it directly. METHODOLOGY.md "Real-time signal" section updated (new URL pattern `https://x.com/search?q=ebola%20outbreak&amp;src=typed_query&amp;f=live`; filtering rules unchanged). The private SKILL.md (project folder) was also updated to: (a) point at the same x.com URL, and (b) replace the previously hardcoded deviceId with a `list_connected_browsers` → pick any → `select_browser` flow, so a rotated deviceId on Web's machine no longer silently breaks the real-time pass.</t>
+          <t>• 2026-05-25 (validator + retroactive no-dip cleanup): Added src/validate.py as a pre-commit gate that enforces schema, monotonic cumulative columns, total = sus + conf, country-sum-equals-global on the latest date, date format/uniqueness. First run caught four legacy no-dip violations from partial revision reconciliation. Applied retroactive cleanup per the rule as written in METHODOLOGY.md: May 19 row carried forward from revised May 18 (WHO Sitrep 01): suspected 516→528, total 549→561, suspected_deaths 131→132. May 22 row carried forward from revised May 21 (WHO DON603): suspected 744→746, confirmed 83→85, total 827→831. The May 22 lift cascaded into May 23: DRC confirmed bumped 82→83 to stay non-decreasing, lifting global confirmed 87→88 and total 837→838. country_breakdown.csv DRC rows updated to match: May 19 DRC suspected 516→528, suspected_deaths 131→132; May 22 DRC suspected 744→746, confirmed 81→83; May 23 DRC confirmed 82→83. All primary_source fields amended to flag the carry-forward and record the same-day source's original figures for audit. May 24 and May 25 rows unaffected. Validator now passes clean.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-26 (post-run x.com real-time pass): Web reconnected his Chrome and authorized a live x.com pass. Credentialed-account filter (`from:` query over WHO/WHOAFRO/DrTedros/AfricaCDC/CDCgov/MinSanteRDC/MinofHealthUG/Reuters/AP/AFP/BNODesk/BNOFeed/BNONews/CIDRAP/HelenBranswell/KrutikaKuppalli) surfaced three material findings, no count changes:</t>
+          <t>• 2026-05-25 (late-evening run): No new numerical figures since the evening run. Citation upgrade applied to May 24 and May 25 rows: WHO DG Tedros's [remarks at the Virtual Ministerial Briefing on the Bundibugyo Ebola Outbreak](https://www.who.int/news-room/speeches/item/who-director-general-s-remarks-at-the-virtual-ministerial-briefing-on-the-bundibugyo-ebola-outbreak-25-may-2026) (25 May 2026) now serve as the primary source for the DRC figures (904 sus / 101 conf / 220 sus deaths / 10 conf deaths). This is a WHO-DG-attributed primary source, higher-tier than the Reuters/AP wires previously cited; corroborated by [UN News (25 May)](https://news.un.org/en/story/2026/05/1167584) and Xinhua. Uganda figures still cite Uganda MoH May 25 press release (+2 health workers in Kampala, total 7 conf / 1 death). The Tedros briefing gave 5 confirmed for Uganda; that figure predates the Uganda MoH same-day +2 release. Per source-preference, the Uganda national MoH remains the authoritative source for Uganda's count. WHO Sitrep 02 and WHO DON604 still not published. CDC Situation Summary still dated 16 May with stale figures; DRC travel notice remains Level 3 (Reconsider Nonessential Travel). 7-day lookback against May 19–25: no numerical revisions required. story.md "Latest update" refreshed to incorporate the WHO DG quote ("the epidemic is outpacing us"), DRC national risk upgraded from "high" to "very high", two treatment centers set alight in eastern DRC, 100,000+ displaced by fighting, $3.9M WHO Contingency Fund release, and WHO clinical-trial prioritization of two monoclonal antibodies + obeldesivir. No declarations.csv change (national risk upgrade is a WHO statement, not a formal declaration change; PHEIC level unchanged). Charts and XLSX regenerated; output filenames unchanged (most-recent Report Date still 2026-05-25).</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-26 (AM run): No new primary-source figures dated 26 May. WHO Sitrep 02 and WHO DON604 still not published; latest reconciled WHO publications remain Sitrep 01 (data as of 18 May) and DON603 (data as of 21 May). CDC Situation Summary still dated 16 May. The latest [BNO News article](https://bnonews.com/index.php/2026/05/ebola-outbreak-in-congo-and-uganda-reaches-more-than-1000-cases/) (publ. 24 May, Sunday DRC figures: 904 sus / 101 conf / 220 sus deaths / 10 conf deaths in DRC, 5 conf / 1 death Uganda) is fully consistent with our May 25 row composition; BNO's "Congo has reported 230 deaths, including 10 confirmed deaths and 220 suspected deaths" is the gross (sus + conf) DRC death count, which matches our 220 + 10 split exactly. The +1 Uganda confirmed-death implied by BNO's combined-country "234 deaths (+15)" Twitter figure is not corroborated by Uganda MoH (Uganda still at 1 confirmed death); BNO summary rounding pending Uganda MoH confirmation. 7-day lookback against May 19–25: no numerical revisions required. New narrative signals (informational, no count change): (1) Italy reported two suspected Ebola cases on 25 May in Lombardy (Como province) — a 31-year-old man in Bulgarograsso and a woman in Lurate Caccivio, both humanitarian aid workers returned from ~3 months in Uganda. [Tests at Sacco Hospital, Milan returned NEGATIVE for Ebola](https://www.euronews.com/my-europe/2026/05/25/ebola-alert-in-italy-two-suspected-cases-in-lombardy-after-return-from-uganda); the woman's neurological symptoms point to cerebral malaria. Italy has stepped up airport screening at Milan Malpensa and Rome Fiumicino; Italian Health Ministry stresses Ebola risk in Italy "remains very low". No declarations.csv row added (no confirmed Italian case). (2) [WSWS analysis (publ. 26 May)](https://www.wsws.org/en/articles/2026/05/26/ddda-m26.html) cites the [Imperial College MRC GIDA modeling update (20 May)](https://www.imperial.ac.uk/mrc-global-infectious-disease-analysis/research-themes/preparedness-and-response-to-emerging-threats/report-ebola-update-20-05-2026/) estimating true early-weeks infections exceeded official counts by ≥2x; not applied as a revision (academic modeling, not surveillance counts). (3) BNO and PBS continue to corroborate the 23 May Mongbwalu MSF facility burning and 18 suspected patients fleeing — already in notes from the 25 May PM xcancel pass. xcancel real-time pass skipped on this unattended run (active anti-bot challenge on xcancel.com — wire services Reuters/AFP/AP/BNO/CIDRAP carry the credentialed-account substance and have been canvassed). No declarations.csv change. No story.md change (no material narrative development since the late-evening 25 May refresh; Italy's negative test does not change the cross-border narrative). Charts and XLSX regenerated; output filenames unchanged (most-recent Report Date still 2026-05-25).</t>
+          <t>• 2026-05-26 (methodology change, Real-time signal source): Switched the Real-time signal source from xcancel.com to x.com via Web's signed-in Chrome. Trigger: xcancel.com served an active anti-bot challenge during the 2026-05-26 AM run, blocking the unattended xcancel pass; meanwhile Web's local Chrome is signed in to x.com and the Claude in Chrome MCP can drive it directly. METHODOLOGY.md "Real-time signal" section updated (new URL pattern `https://x.com/search?q=ebola%20outbreak&amp;src=typed_query&amp;f=live`; filtering rules unchanged). The private SKILL.md (project folder) was also updated to: (a) point at the same x.com URL, and (b) replace the previously hardcoded deviceId with a `list_connected_browsers` → pick any → `select_browser` flow, so a rotated deviceId on Web's machine no longer silently breaks the real-time pass.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-26 (later run, x.com real-time pass): BNO News @BNOFeed Daily Ebola Update for May 25 (situation report image) surfaced as a corroborating wire primary source for the 906/105/223 DRC figures previously circulating in CDC HAN paraphrases / ECDC summary / Wikipedia / search summaries without a clear primary URL. BNO May 25 situation report shows: DR Congo 1,011 cases (906 sus + 105 conf) / 233 deaths (223 sus + 10 conf); Uganda 7 conf / 1 death; TOTAL 1,018 cases (+8 from May 24) / 234 deaths (+3 from May 24). This is a credentialed-wire primary citation under source-preference order (tier 5: BNO News), and the figures supersede the WHO DG Tedros 25 May briefing figures (904/101/220) under the upward-revision rule (single high-value source sufficient for upward revisions). All four revisions are upward, not downward (no-dip rule not triggered).</t>
+          <t>• 2026-05-26 (post-run x.com real-time pass): Web reconnected his Chrome and authorized a live x.com pass. Credentialed-account filter (`from:` query over WHO/WHOAFRO/DrTedros/AfricaCDC/CDCgov/MinSanteRDC/MinofHealthUG/Reuters/AP/AFP/BNODesk/BNOFeed/BNONews/CIDRAP/HelenBranswell/KrutikaKuppalli) surfaced three material findings, no count changes:</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-26 (later run) — May 25 row revised per BNO News @BNOFeed May 25 Situation Report: suspected 904→906 (+0.22%), confirmed 108→112 (+3.70%), total 1012→1018 (+0.59%), suspected_deaths 220→223 (+1.36%). country_breakdown.csv DRC May 25 row updated to match: suspected 904→906, confirmed 101→105, suspected_deaths 220→223 (DRC confirmed_deaths 10 unchanged). Uganda row unchanged at 7 conf / 1 death.</t>
+          <t>• 2026-05-26 (AM run): No new primary-source figures dated 26 May. WHO Sitrep 02 and WHO DON604 still not published; latest reconciled WHO publications remain Sitrep 01 (data as of 18 May) and DON603 (data as of 21 May). CDC Situation Summary still dated 16 May. The latest [BNO News article](https://bnonews.com/index.php/2026/05/ebola-outbreak-in-congo-and-uganda-reaches-more-than-1000-cases/) (publ. 24 May, Sunday DRC figures: 904 sus / 101 conf / 220 sus deaths / 10 conf deaths in DRC, 5 conf / 1 death Uganda) is fully consistent with our May 25 row composition; BNO's "Congo has reported 230 deaths, including 10 confirmed deaths and 220 suspected deaths" is the gross (sus + conf) DRC death count, which matches our 220 + 10 split exactly. The +1 Uganda confirmed-death implied by BNO's combined-country "234 deaths (+15)" Twitter figure is not corroborated by Uganda MoH (Uganda still at 1 confirmed death); BNO summary rounding pending Uganda MoH confirmation. 7-day lookback against May 19–25: no numerical revisions required. New narrative signals (informational, no count change): (1) Italy reported two suspected Ebola cases on 25 May in Lombardy (Como province) — a 31-year-old man in Bulgarograsso and a woman in Lurate Caccivio, both humanitarian aid workers returned from ~3 months in Uganda. [Tests at Sacco Hospital, Milan returned NEGATIVE for Ebola](https://www.euronews.com/my-europe/2026/05/25/ebola-alert-in-italy-two-suspected-cases-in-lombardy-after-return-from-uganda); the woman's neurological symptoms point to cerebral malaria. Italy has stepped up airport screening at Milan Malpensa and Rome Fiumicino; Italian Health Ministry stresses Ebola risk in Italy "remains very low". No declarations.csv row added (no confirmed Italian case). (2) [WSWS analysis (publ. 26 May)](https://www.wsws.org/en/articles/2026/05/26/ddda-m26.html) cites the [Imperial College MRC GIDA modeling update (20 May)](https://www.imperial.ac.uk/mrc-global-infectious-disease-analysis/research-themes/preparedness-and-response-to-emerging-threats/report-ebola-update-20-05-2026/) estimating true early-weeks infections exceeded official counts by ≥2x; not applied as a revision (academic modeling, not surveillance counts). (3) BNO and PBS continue to corroborate the 23 May Mongbwalu MSF facility burning and 18 suspected patients fleeing — already in notes from the 25 May PM xcancel pass. xcancel real-time pass skipped on this unattended run (active anti-bot challenge on xcancel.com — wire services Reuters/AFP/AP/BNO/CIDRAP carry the credentialed-account substance and have been canvassed). No declarations.csv change. No story.md change (no material narrative development since the late-evening 25 May refresh; Italy's negative test does not change the cross-border narrative). Charts and XLSX regenerated; output filenames unchanged (most-recent Report Date still 2026-05-25).</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-26 (later run) — OBSERVED_REVISION_RANGE in generate_charts.py updated from "4-35%" to "&lt;1-35%" to bracket the new lower bound. May 25 suspected (+0.22%) and total (+0.59%) revisions land below 1%, so the previous "4-35%" range no longer brackets the observed upward-revision history. New range expressed as "&lt;1-35%" to communicate that minor sub-1% refinements occur alongside the larger 4-35% reconciliation events from WHO Sitrep/DON publications.</t>
+          <t>• 2026-05-26 (later run, x.com real-time pass): BNO News @BNOFeed Daily Ebola Update for May 25 (situation report image) surfaced as a corroborating wire primary source for the 906/105/223 DRC figures previously circulating in CDC HAN paraphrases / ECDC summary / Wikipedia / search summaries without a clear primary URL. BNO May 25 situation report shows: DR Congo 1,011 cases (906 sus + 105 conf) / 233 deaths (223 sus + 10 conf); Uganda 7 conf / 1 death; TOTAL 1,018 cases (+8 from May 24) / 234 deaths (+3 from May 24). This is a credentialed-wire primary citation under source-preference order (tier 5: BNO News), and the figures supersede the WHO DG Tedros 25 May briefing figures (904/101/220) under the upward-revision rule (single high-value source sufficient for upward revisions). All four revisions are upward, not downward (no-dip rule not triggered).</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-26 (later run, x.com real-time pass — credentialed-account narrative items, no count change):</t>
+          <t>• 2026-05-26 (later run) — May 25 row revised per BNO News @BNOFeed May 25 Situation Report: suspected 904→906 (+0.22%), confirmed 108→112 (+3.70%), total 1012→1018 (+0.59%), suspected_deaths 220→223 (+1.36%). country_breakdown.csv DRC May 25 row updated to match: suspected 904→906, confirmed 101→105, suspected_deaths 220→223 (DRC confirmed_deaths 10 unchanged). Uganda row unchanged at 7 conf / 1 death.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-26 (later run): No new WHO Sitrep 02 published. No new WHO DON604 published. CDC Situation Summary still dated May 16. CDC HAN still dated May 19. ECDC page still dated May 21. WHO outbreak page unchanged. Latest BNO News article remains [Sunday May 24 "1,000 cases" report](https://bnonews.com/index.php/2026/05/ebola-outbreak-in-congo-and-uganda-reaches-more-than-1000-cases/); the May 25 BNO situation report appears on @BNOFeed X account but no linked article URL surfaced. 7-day lookback against May 19–25: only the May 25 row revision applied. No declarations.csv change (CDC HAN dated May 19; DRC still Level 3, Uganda still Level 1; no PHEIC change). No story.md change (the May 25 narrative update remains accurate; the +2/+4/+3 refinements are not a material narrative event). Charts and XLSX regenerated; output filenames unchanged (most-recent Report Date still 2026-05-25).</t>
+          <t>• 2026-05-26 (later run) — OBSERVED_REVISION_RANGE in generate_charts.py updated from "4-35%" to "&lt;1-35%" to bracket the new lower bound. May 25 suspected (+0.22%) and total (+0.59%) revisions land below 1%, so the previous "4-35%" range no longer brackets the observed upward-revision history. New range expressed as "&lt;1-35%" to communicate that minor sub-1% refinements occur alongside the larger 4-35% reconciliation events from WHO Sitrep/DON publications.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-26 (late-evening run): [CDC Situation Summary refreshed 25 May 2026](https://www.cdc.gov/ebola/situation-summary/index.html) (page metadata: cdc:last_updated 2026-05-25T18:06:48Z). CDC reports DRC 906 sus / 105 conf / 223 sus deaths / 10 conf deaths and Uganda 7 conf / 1 death — matches the May 25 row exactly. Citation upgrade applied: May 25 primary_source promoted from BNO News (tier 5) to CDC Situation Summary (tier 3) as the lead citation, with BNO retained as corroborating wire source and Uganda MoH retained for the +2 Kampala health-worker detail. No numerical change. country_breakdown.csv DRC May 25 row mirrored. The CDC update also notes the first lab-confirmed case in **Sud-Kivu Province** (previously Ituri + Nord-Kivu only had confirmed cases, even though suspected cases spanned all three provinces). This is a geographic detail; the global confirmed count (105) is unchanged.</t>
+          <t>• 2026-05-26 (later run, x.com real-time pass — credentialed-account narrative items, no count change):</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-26 (late-evening run, x.com real-time pass): Web's signed-in Chrome reachable via the `list_connected_browsers` → `select_browser` flow. Credentialed-account filter (`from:` query over WHO/WHOAFRO/DrTedros/AfricaCDC/CDCgov/MinSanteRDC/MinofHealthUG/Reuters/AP/AFP/BNODesk/BNOFeed/BNONews/CIDRAP/HelenBranswell/KrutikaKuppalli) surfaced operational/awareness content, no count changes: (a) [DrTedros (~11h)](https://x.com/DrTedros) IPC hunger data already in earlier notes; (b) [MinofHealthUG (~9-10h)](https://x.com/MinofHealthUG) community-sensitization activities across Kampala, Wakiso, Kasese, Kisoro, Bundibugyo, Kikuube, Arua Districts plus generic early-treatment messaging; (c) [Reuters (~9-11h)](https://x.com/Reuters) Bukavu handwashing-station surge, doctor hostility, unsafe-burials transmission driver — already in earlier notes. Trending sidebar surfaced two narrative signals not from credentialed accounts and not yet supported by primary sources, logged for transparency only: (1) [Bengaluru reports first suspected case](https://www.oneindia.com/bengaluru/ebola-case-bengaluru-records-first-suspected-ebola-case-as-ugandan-woman-shifted-to-isolation-ward-8100173.html), a 28-year-old Ugandan woman shifted to the Epidemic Diseases Hospital, blood and swab samples sent to NIV Pune for testing — analogous to the 25 May Italy suspected cases that ultimately tested negative; no declarations.csv row added (no confirmed Indian case); (2) "U.S. Sets Up Ebola Quarantine Site in Kenya" trending headline not substantiated by primary CDC, State Department, or Kenya MoH sources — Kenya is intensifying its own surveillance and the U.S. has enhanced travel screening at IAD and ATL airports, but no U.S.-operated Kenya quarantine facility appears in the searched sources. Not applied.</t>
+          <t>• 2026-05-26 (later run): No new WHO Sitrep 02 published. No new WHO DON604 published. CDC Situation Summary still dated May 16. CDC HAN still dated May 19. ECDC page still dated May 21. WHO outbreak page unchanged. Latest BNO News article remains [Sunday May 24 "1,000 cases" report](https://bnonews.com/index.php/2026/05/ebola-outbreak-in-congo-and-uganda-reaches-more-than-1000-cases/); the May 25 BNO situation report appears on @BNOFeed X account but no linked article URL surfaced. 7-day lookback against May 19–25: only the May 25 row revision applied. No declarations.csv change (CDC HAN dated May 19; DRC still Level 3, Uganda still Level 1; no PHEIC change). No story.md change (the May 25 narrative update remains accurate; the +2/+4/+3 refinements are not a material narrative event). Charts and XLSX regenerated; output filenames unchanged (most-recent Report Date still 2026-05-25).</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-26 (late-evening run, summary): No numerical revisions to timeseries.csv beyond the citation upgrade. country_breakdown.csv May 25 DRC row primary_source updated. declarations.csv unchanged. story.md unchanged. LAST_SITREP_STABLE_DATE unchanged (still 2026-05-18; no WHO Sitrep 02 yet). OBSERVED_REVISION_RANGE unchanged at "&lt;1-35%". Charts and XLSX regenerated; output filenames unchanged (most-recent Report Date still 2026-05-25).</t>
+          <t>• 2026-05-26 (late-evening run): [CDC Situation Summary refreshed 25 May 2026](https://www.cdc.gov/ebola/situation-summary/index.html) (page metadata: cdc:last_updated 2026-05-25T18:06:48Z). CDC reports DRC 906 sus / 105 conf / 223 sus deaths / 10 conf deaths and Uganda 7 conf / 1 death — matches the May 25 row exactly. Citation upgrade applied: May 25 primary_source promoted from BNO News (tier 5) to CDC Situation Summary (tier 3) as the lead citation, with BNO retained as corroborating wire source and Uganda MoH retained for the +2 Kampala health-worker detail. No numerical change. country_breakdown.csv DRC May 25 row mirrored. The CDC update also notes the first lab-confirmed case in **Sud-Kivu Province** (previously Ituri + Nord-Kivu only had confirmed cases, even though suspected cases spanned all three provinces). This is a geographic detail; the global confirmed count (105) is unchanged.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-26 (post-run correction — miss caught by Web): The late-evening run's x.com real-time pass missed a fresh BNO News @BNOFeed Daily Ebola Update for May 26 (Situation Report graphic posted ~2h before the original run). Root cause: the agent navigated to https://x.com/BNOFeed directly to check for the daily situation report, the profile page was still loading (visible spinner in screenshot), and the agent bailed early with "I have enough for the real-time pass." That was a procedural failure — BNO's Daily Ebola Update is one of the highest-value wire sources in the source-preference order and should be confirmed before declaring the pass complete. Fix going forward: never declare the real-time pass complete without explicitly confirming BNO @BNOFeed's most recent post (either via the profile page after waiting for it to render, or by running a targeted `from:BNOFeed` search). The BNO May 26 graphic (citing DRC MoH + Uganda MoH + WHO) reports: DRC 1,042 cases (+31) / 240 deaths (+7); Uganda 7 conf / 1 death (unchanged); TOTAL 1,049 / 241.</t>
+          <t>• 2026-05-26 (late-evening run, x.com real-time pass): Web's signed-in Chrome reachable via the `list_connected_browsers` → `select_browser` flow. Credentialed-account filter (`from:` query over WHO/WHOAFRO/DrTedros/AfricaCDC/CDCgov/MinSanteRDC/MinofHealthUG/Reuters/AP/AFP/BNODesk/BNOFeed/BNONews/CIDRAP/HelenBranswell/KrutikaKuppalli) surfaced operational/awareness content, no count changes: (a) [DrTedros (~11h)](https://x.com/DrTedros) IPC hunger data already in earlier notes; (b) [MinofHealthUG (~9-10h)](https://x.com/MinofHealthUG) community-sensitization activities across Kampala, Wakiso, Kasese, Kisoro, Bundibugyo, Kikuube, Arua Districts plus generic early-treatment messaging; (c) [Reuters (~9-11h)](https://x.com/Reuters) Bukavu handwashing-station surge, doctor hostility, unsafe-burials transmission driver — already in earlier notes. Trending sidebar surfaced two narrative signals not from credentialed accounts and not yet supported by primary sources, logged for transparency only: (1) [Bengaluru reports first suspected case](https://www.oneindia.com/bengaluru/ebola-case-bengaluru-records-first-suspected-ebola-case-as-ugandan-woman-shifted-to-isolation-ward-8100173.html), a 28-year-old Ugandan woman shifted to the Epidemic Diseases Hospital, blood and swab samples sent to NIV Pune for testing — analogous to the 25 May Italy suspected cases that ultimately tested negative; no declarations.csv row added (no confirmed Indian case); (2) "U.S. Sets Up Ebola Quarantine Site in Kenya" trending headline not substantiated by primary CDC, State Department, or Kenya MoH sources — Kenya is intensifying its own surveillance and the U.S. has enhanced travel screening at IAD and ATL airports, but no U.S.-operated Kenya quarantine facility appears in the searched sources. Not applied.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-26 (correction) — Appended May 26 row to timeseries.csv: total_global 1,049 (+31), suspected_deaths_global 230 (+7). The BNO graphic does NOT provide a DRC sus/conf split. To keep the chart pipeline correct (generate_charts.py treats blank cells as 0 and would compute large negative deltas otherwise), the +31 DRC cases are attributed entirely to suspected (sus 906→937), DRC confirmed held at 105 (matches CDC Situation Summary 25 May DRC confirmed count). DRC deaths 240 split as 230 sus + 10 conf, with DRC conf deaths carried forward. This is an INFERENCE, openly flagged in primary_source. WHO Sitrep 02 / DON604 / DRC MoH formal release with a sus/conf split will likely revise these numbers. country_breakdown.csv mirrored with the same DRC inference + an unchanged Uganda row.</t>
+          <t>• 2026-05-26 (late-evening run, summary): No numerical revisions to timeseries.csv beyond the citation upgrade. country_breakdown.csv May 25 DRC row primary_source updated. declarations.csv unchanged. story.md unchanged. LAST_SITREP_STABLE_DATE unchanged (still 2026-05-18; no WHO Sitrep 02 yet). OBSERVED_REVISION_RANGE unchanged at "&lt;1-35%". Charts and XLSX regenerated; output filenames unchanged (most-recent Report Date still 2026-05-25).</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-26 (correction): Validator passes. Cumulative non-decreasing maintained on all four columns (sus 906→937, conf 112→112, total 1018→1049, sus_deaths 223→230). story.md unchanged on this correction pass — the May 25 WHO DG Tedros briefing remains the lead narrative event; the May 26 BNO situation report is a wire-level data point not a material new narrative. declarations.csv unchanged. LAST_SITREP_STABLE_DATE unchanged. OBSERVED_REVISION_RANGE unchanged. Charts and XLSX regenerated; output PNG filenames now dated 2026-05-26.</t>
+          <t>• 2026-05-26 (post-run correction — miss caught by Web): The late-evening run's x.com real-time pass missed a fresh BNO News @BNOFeed Daily Ebola Update for May 26 (Situation Report graphic posted ~2h before the original run). Root cause: the agent navigated to https://x.com/BNOFeed directly to check for the daily situation report, the profile page was still loading (visible spinner in screenshot), and the agent bailed early with "I have enough for the real-time pass." That was a procedural failure — BNO's Daily Ebola Update is one of the highest-value wire sources in the source-preference order and should be confirmed before declaring the pass complete. Fix going forward: never declare the real-time pass complete without explicitly confirming BNO @BNOFeed's most recent post (either via the profile page after waiting for it to render, or by running a targeted `from:BNOFeed` search). The BNO May 26 graphic (citing DRC MoH + Uganda MoH + WHO) reports: DRC 1,042 cases (+31) / 240 deaths (+7); Uganda 7 conf / 1 death (unchanged); TOTAL 1,049 / 241.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-27 (AM run): No new primary-source figures dated 27 May. WHO Sitrep 02 and WHO DON604 still not published; latest reconciled WHO publications remain Sitrep 01 (data as of 18 May) and DON603 (data as of 21 May). The WHO outbreak page lists no new news items since the 22 May IHR Emergency Committee statement; the 25 May Tedros virtual ministerial briefing speech remains the most recent WHO-DG-attributed primary source. CDC Situation Summary now appears dated May 16 with stale figures (8 confirmed / 248 suspected) and references the Level 2 DRC travel notice — the May 25 refreshed state observed in yesterday's late-evening run is no longer visible at the canonical URL. Possible explanations: CDC reverted the page, the May 25 state was a brief refresh that was rolled back, or this fetch hit a different cache. Declarations.csv kept unchanged (DRC still Level 3 per yesterday's verified travel-notice URL); will recheck on the next run.</t>
+          <t>• 2026-05-26 (correction) — Appended May 26 row to timeseries.csv: total_global 1,049 (+31), suspected_deaths_global 230 (+7). The BNO graphic does NOT provide a DRC sus/conf split. To keep the chart pipeline correct (generate_charts.py treats blank cells as 0 and would compute large negative deltas otherwise), the +31 DRC cases are attributed entirely to suspected (sus 906→937), DRC confirmed held at 105 (matches CDC Situation Summary 25 May DRC confirmed count). DRC deaths 240 split as 230 sus + 10 conf, with DRC conf deaths carried forward. This is an INFERENCE, openly flagged in primary_source. WHO Sitrep 02 / DON604 / DRC MoH formal release with a sus/conf split will likely revise these numbers. country_breakdown.csv mirrored with the same DRC inference + an unchanged Uganda row.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-27 (AM run, x.com real-time pass): Web's signed-in Chrome reachable via select_browser (deviceId 5fdc215b-0b1a-4a16-9f71-01f672b11fbf). BNO @BNOFeed's most recent post (13h before pass) is the May 26 Daily Ebola Update graphic already cited in the May 26 row (DRC 1,042 cases (+31) / 240 deaths (+7); Uganda unchanged). No newer BNO Daily Update has posted. Credentialed-account search surfaced one new narrative-level item: [Krutika Kuppalli, MD FIDSA @KrutikaKuppalli (~2h)](https://x.com/KrutikaKuppalli) quote-tweet of a Forbes/AFP framing ("Ebola Outbreak At Risk Of Becoming 'Deadliest On Record,' Humanitarian Group Warns") commenting that "it is appalling to see how U.S. actions have contributed to the conditions that allowed this #Ebola outbreak to escalate and continue to complicate the response." Commentary, not surveillance data; no count change. Other credentialed accounts (WHO, WHOAFRO, DrTedros, MinofHealthUG, Reuters, AP, AFP, CIDRAP, HelenBranswell) showed no new posts since yesterday's late-evening pass.</t>
+          <t>• 2026-05-26 (correction): Validator passes. Cumulative non-decreasing maintained on all four columns (sus 906→937, conf 112→112, total 1018→1049, sus_deaths 223→230). story.md unchanged on this correction pass — the May 25 WHO DG Tedros briefing remains the lead narrative event; the May 26 BNO situation report is a wire-level data point not a material new narrative. declarations.csv unchanged. LAST_SITREP_STABLE_DATE unchanged. OBSERVED_REVISION_RANGE unchanged. Charts and XLSX regenerated; output PNG filenames now dated 2026-05-26.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-27 (AM run, BNO News article surfaced): [BNO News article](https://bnonews.com/index.php/2026/05/ebola-outbreak-in-congo-and-uganda-grows-to-1049-cases-241-deaths/) "Ebola outbreak in Congo and Uganda grows to 1,049 cases; 241 deaths" (published May 26 Tuesday) provides the primary DRC sus/conf split that the May 26 row had previously inferred. BNO article reports: DRC 930 sus / 112 conf / 223 sus deaths / 17 conf deaths; Uganda 7 conf / 1 death (unchanged); TOTAL 1,049 cases / 241 deaths (unchanged from the BNOFeed graphic). Article also reports: outbreak spans 13 health zones across three DRC provinces (up from 12 in earlier reporting); 2,231 contacts identified in DRC; WHO says contact follow-up remains a major challenge.</t>
+          <t>• 2026-05-27 (AM run): No new primary-source figures dated 27 May. WHO Sitrep 02 and WHO DON604 still not published; latest reconciled WHO publications remain Sitrep 01 (data as of 18 May) and DON603 (data as of 21 May). The WHO outbreak page lists no new news items since the 22 May IHR Emergency Committee statement; the 25 May Tedros virtual ministerial briefing speech remains the most recent WHO-DG-attributed primary source. CDC Situation Summary now appears dated May 16 with stale figures (8 confirmed / 248 suspected) and references the Level 2 DRC travel notice — the May 25 refreshed state observed in yesterday's late-evening run is no longer visible at the canonical URL. Possible explanations: CDC reverted the page, the May 25 state was a brief refresh that was rolled back, or this fetch hit a different cache. Declarations.csv kept unchanged (DRC still Level 3 per yesterday's verified travel-notice URL); will recheck on the next run.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-27 (AM run) — May 26 row revised per BNO News May 26 article: suspected_global 937→930 (-0.75%), confirmed_global 112→119 (+6.25%), total_global 1049→1049 (unchanged), suspected_deaths_global 230→223 (-3.04%). The TOTAL figures (cases and deaths) are unchanged; only the internal sus/conf attribution shifts to match the primary source split. Treated as an inference correction rather than a no-dip-rule dip event: (a) the May 26 row's primary_source field explicitly announced it was an inference pending refinement when a primary sus/conf split published, (b) cumulative TOTAL cases and TOTAL deaths are unchanged so no real-world reclassification is being proposed, (c) the BNO News article is a primary citation under the source-preference order (tier 5) and supersedes our own attribution. Validator constraints preserved: May 26 sus 930 ≥ May 25 sus 906 ✓; conf 119 ≥ 112 ✓; total 1049 ≥ 1018 ✓; sus_deaths 223 ≥ 223 ✓ (equal to May 25, satisfies monotonic non-decreasing). country_breakdown.csv DRC May 26 row mirrored: sus 937→930, conf 105→112, sus_deaths 230→223, confirmed_deaths 10→17.</t>
+          <t>• 2026-05-27 (AM run, x.com real-time pass): Web's signed-in Chrome reachable via select_browser (deviceId 5fdc215b-0b1a-4a16-9f71-01f672b11fbf). BNO @BNOFeed's most recent post (13h before pass) is the May 26 Daily Ebola Update graphic already cited in the May 26 row (DRC 1,042 cases (+31) / 240 deaths (+7); Uganda unchanged). No newer BNO Daily Update has posted. Credentialed-account search surfaced one new narrative-level item: [Krutika Kuppalli, MD FIDSA @KrutikaKuppalli (~2h)](https://x.com/KrutikaKuppalli) quote-tweet of a Forbes/AFP framing ("Ebola Outbreak At Risk Of Becoming 'Deadliest On Record,' Humanitarian Group Warns") commenting that "it is appalling to see how U.S. actions have contributed to the conditions that allowed this #Ebola outbreak to escalate and continue to complicate the response." Commentary, not surveillance data; no count change. Other credentialed accounts (WHO, WHOAFRO, DrTedros, MinofHealthUG, Reuters, AP, AFP, CIDRAP, HelenBranswell) showed no new posts since yesterday's late-evening pass.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-27 (AM run): OBSERVED_REVISION_RANGE unchanged at "&lt;1-35%". Today's upward revision: conf +6.25% (within range). Today's downward revisions (-0.75% sus, -3.04% sus_deaths) are inference corrections of an explicitly-flagged provisional split, not real-world reclassifications, and the chart-footnote text describes upward revisions only. LAST_SITREP_STABLE_DATE unchanged at 2026-05-18 (no WHO Sitrep 02 yet). declarations.csv unchanged. story.md unchanged — the 25 May WHO DG Tedros briefing remains the lead narrative event; today's run is a wire-level data refinement (sus/conf split + contact-tracing scale) not a material new narrative. Charts and XLSX regenerated; output PNG filenames stay dated 2026-05-26 (latest Report Date unchanged).</t>
+          <t>• 2026-05-27 (AM run, BNO News article surfaced): [BNO News article](https://bnonews.com/index.php/2026/05/ebola-outbreak-in-congo-and-uganda-grows-to-1049-cases-241-deaths/) "Ebola outbreak in Congo and Uganda grows to 1,049 cases; 241 deaths" (published May 26 Tuesday) provides the primary DRC sus/conf split that the May 26 row had previously inferred. BNO article reports: DRC 930 sus / 112 conf / 223 sus deaths / 17 conf deaths; Uganda 7 conf / 1 death (unchanged); TOTAL 1,049 cases / 241 deaths (unchanged from the BNOFeed graphic). Article also reports: outbreak spans 13 health zones across three DRC provinces (up from 12 in earlier reporting); 2,231 contacts identified in DRC; WHO says contact follow-up remains a major challenge.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-27 (AM run, Sitrep 02 application — caught by Web post-run): [WHO AFRO Weekly External Situation Report 02 (data as of 24 May 2026)](https://www.afro.who.int/countries/democratic-republic-of-congo/publication/ebola-bundibugyo-virus-disease-outbreak-0) published this morning, linked from the right sidebar of the WHO AFRO outbreak page (https://www.afro.who.int/health-topics/ebola-disease/outbreak-drc-26) but not yet listed on the DRC publications index. Sitrep cover date is 24 May 2026 with a publication date of 27 May 2026 — three-day publication lag is typical. The publications-index page only returned Sitrep 01 in this morning's earlier fetch; the sidebar pre-empted the index, which is the failure mode. Lesson: scan the WHO AFRO outbreak page's Situation Reports sidebar in addition to the publications index. The agent will add this pass to future runs.</t>
+          <t>• 2026-05-27 (AM run) — May 26 row revised per BNO News May 26 article: suspected_global 937→930 (-0.75%), confirmed_global 112→119 (+6.25%), total_global 1049→1049 (unchanged), suspected_deaths_global 230→223 (-3.04%). The TOTAL figures (cases and deaths) are unchanged; only the internal sus/conf attribution shifts to match the primary source split. Treated as an inference correction rather than a no-dip-rule dip event: (a) the May 26 row's primary_source field explicitly announced it was an inference pending refinement when a primary sus/conf split published, (b) cumulative TOTAL cases and TOTAL deaths are unchanged so no real-world reclassification is being proposed, (c) the BNO News article is a primary citation under the source-preference order (tier 5) and supersedes our own attribution. Validator constraints preserved: May 26 sus 930 ≥ May 25 sus 906 ✓; conf 119 ≥ 112 ✓; total 1049 ≥ 1018 ✓; sus_deaths 223 ≥ 223 ✓ (equal to May 25, satisfies monotonic non-decreasing). country_breakdown.csv DRC May 26 row mirrored: sus 937→930, conf 105→112, sus_deaths 230→223, confirmed_deaths 10→17.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-27 (AM run) — May 24 row revised per WHO Sitrep 02: suspected_global 904→906 (+0.22%), confirmed_global 106→112 (+5.66%), total_global 1010→1018 (+0.79%), suspected_deaths_global 220→223 (+1.36%). All revisions upward; no no-dip-rule trigger. country_breakdown.csv May 24: DRC 904/101/220/10 → 906/105/223/10 (sus +2, conf +4, sus_deaths +3, conf_deaths unchanged); Uganda confirmed 5 → 7 (Sitrep 02 retroactively credits the +2 Kampala health-worker cases publicly announced 25 May under the May 24 cutoff). Primary_source upgraded from "DRC govt Sunday figures + 25 May Tedros briefing" to WHO Sitrep 02. May 25 row left unchanged — its totals (906/112/1018/223) already match Sitrep 02's May 24 cutoff exactly, meaning May 24 and May 25 now represent the same data point as observed in two source channels (Sitrep 02 reconciled vs CDC+BNO+Uganda MoH same-day reporting).</t>
+          <t>• 2026-05-27 (AM run): OBSERVED_REVISION_RANGE unchanged at "&lt;1-35%". Today's upward revision: conf +6.25% (within range). Today's downward revisions (-0.75% sus, -3.04% sus_deaths) are inference corrections of an explicitly-flagged provisional split, not real-world reclassifications, and the chart-footnote text describes upward revisions only. LAST_SITREP_STABLE_DATE unchanged at 2026-05-18 (no WHO Sitrep 02 yet). declarations.csv unchanged. story.md unchanged — the 25 May WHO DG Tedros briefing remains the lead narrative event; today's run is a wire-level data refinement (sus/conf split + contact-tracing scale) not a material new narrative. Charts and XLSX regenerated; output PNG filenames stay dated 2026-05-26 (latest Report Date unchanged).</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-27 (AM run) — LAST_SITREP_STABLE_DATE updated from "2026-05-18" to "2026-05-24". This shifts the hatched/provisional boundary on both charts forward by 6 days; May 19 through May 24 rows now render as Sitrep-stable solid bars (was hatched), May 25 and May 26 remain hatched (provisional pending Sitrep 03 / DON604). OBSERVED_REVISION_RANGE unchanged at "&lt;1-35%" — today's May 24 revisions all sit inside the range (largest is conf +5.66%). Second commit follows the morning's first commit so the Sitrep 02 application is its own audit trail entry.</t>
+          <t>• 2026-05-27 (AM run, Sitrep 02 application — caught by Web post-run): [WHO AFRO Weekly External Situation Report 02 (data as of 24 May 2026)](https://www.afro.who.int/countries/democratic-republic-of-congo/publication/ebola-bundibugyo-virus-disease-outbreak-0) published this morning, linked from the right sidebar of the WHO AFRO outbreak page (https://www.afro.who.int/health-topics/ebola-disease/outbreak-drc-26) but not yet listed on the DRC publications index. Sitrep cover date is 24 May 2026 with a publication date of 27 May 2026 — three-day publication lag is typical. The publications-index page only returned Sitrep 01 in this morning's earlier fetch; the sidebar pre-empted the index, which is the failure mode. Lesson: scan the WHO AFRO outbreak page's Situation Reports sidebar in addition to the publications index. The agent will add this pass to future runs.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-27 (PM run): Material narrative event — [Uganda ordered four-week border closure with DRC effective immediately](https://www.pbs.org/newshour/health/uganda-closes-its-border-with-congo-where-suspected-cases-of-rare-ebola-type-are-surging) (AP via PBS NewsHour 27 May 19:37 EDT; Bloomberg; Washington Post; NYT via UNMC Transmission). Dr Diana Atwine (Uganda MoH Director General) announced: emergency crossings for Ebola response / humanitarian / cargo / security only, with mandatory 21-day isolation on entry. Measure goes against WHO guidance, which warns closures push movement to unmonitored informal crossings. declarations.csv Uganda row updated (case_status amended; notes appended). story.md "Latest update" rewritten from the 25 May Tedros briefing to the 27 May border closure + DRC MoH situation report.</t>
+          <t>• 2026-05-27 (AM run) — May 24 row revised per WHO Sitrep 02: suspected_global 904→906 (+0.22%), confirmed_global 106→112 (+5.66%), total_global 1010→1018 (+0.79%), suspected_deaths_global 220→223 (+1.36%). All revisions upward; no no-dip-rule trigger. country_breakdown.csv May 24: DRC 904/101/220/10 → 906/105/223/10 (sus +2, conf +4, sus_deaths +3, conf_deaths unchanged); Uganda confirmed 5 → 7 (Sitrep 02 retroactively credits the +2 Kampala health-worker cases publicly announced 25 May under the May 24 cutoff). Primary_source upgraded from "DRC govt Sunday figures + 25 May Tedros briefing" to WHO Sitrep 02. May 25 row left unchanged — its totals (906/112/1018/223) already match Sitrep 02's May 24 cutoff exactly, meaning May 24 and May 25 now represent the same data point as observed in two source channels (Sitrep 02 reconciled vs CDC+BNO+Uganda MoH same-day reporting).</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-27 (PM run, DRC MoH 27 May situation report): [Xinhua, dated 28 May 00:39 UTC](https://english.news.cn/africa/20260528/1bc05fdf07f44f6e837a9117e6a715ec/c.html), datelined Kinshasa 27 May, reports the DRC MoH situation report "released Wednesday" with "figures compiled as of Tuesday [26 May]": DRC 1,077 sus / 121 conf / 238 sus deaths / 17 conf deaths; 13 health zones across Ituri / Nord-Kivu / Sud-Kivu (Ituri remains epicenter). Cumulative since 15 May outbreak declaration. Uganda unchanged at 7 conf / 1 death per Uganda MoH (corroborated by AP / PBS 27 May which also cites &gt;3,000 possible contacts under investigation in DRC). Treated as fresher reconciled DRC MoH snapshot superseding the BNO News May 26 article (DRC 930/112/223/17), which was based on the DRC MoH morning May 26 bulletin (likely as-of-25 May cutoff).</t>
+          <t>• 2026-05-27 (AM run) — LAST_SITREP_STABLE_DATE updated from "2026-05-18" to "2026-05-24". This shifts the hatched/provisional boundary on both charts forward by 6 days; May 19 through May 24 rows now render as Sitrep-stable solid bars (was hatched), May 25 and May 26 remain hatched (provisional pending Sitrep 03 / DON604). OBSERVED_REVISION_RANGE unchanged at "&lt;1-35%" — today's May 24 revisions all sit inside the range (largest is conf +5.66%). Second commit follows the morning's first commit so the Sitrep 02 application is its own audit trail entry.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-27 (PM run) — May 26 row revised per DRC MoH 27 May situation report (via Xinhua): suspected_global 930→1077 (+15.81%), confirmed_global 119→128 (+7.56%), total_global 1049→1205 (+14.87%), suspected_deaths_global 223→238 (+6.73%). All four revisions upward; no no-dip-rule trigger. country_breakdown.csv May 26 DRC row mirrored: sus 930→1077, conf 112→121, sus_deaths 223→238, confirmed_deaths 17 (unchanged). Uganda May 26 row unchanged at 7 conf / 1 death; primary_source updated to cite AP / PBS / Bloomberg / Washington Post 27 May coverage. The DRC MoH situation report is a single high-value source (per METHODOLOGY.md: "DRC Ministry of Health official press releases" are high-value), and all revisions are upward, so single-source backing is sufficient.</t>
+          <t>• 2026-05-27 (PM run): Material narrative event — [Uganda ordered four-week border closure with DRC effective immediately](https://www.pbs.org/newshour/health/uganda-closes-its-border-with-congo-where-suspected-cases-of-rare-ebola-type-are-surging) (AP via PBS NewsHour 27 May 19:37 EDT; Bloomberg; Washington Post; NYT via UNMC Transmission). Dr Diana Atwine (Uganda MoH Director General) announced: emergency crossings for Ebola response / humanitarian / cargo / security only, with mandatory 21-day isolation on entry. Measure goes against WHO guidance, which warns closures push movement to unmonitored informal crossings. declarations.csv Uganda row updated (case_status amended; notes appended). story.md "Latest update" rewritten from the 25 May Tedros briefing to the 27 May border closure + DRC MoH situation report.</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-27 (PM run) — Appended May 27 row to timeseries.csv: 1077/128/1205/238 carried forward from revised May 26 row, since DRC MoH 27 May situation report has data cutoff 26 May and no fresher cumulative figure has been published for 27 May. The 27 May row carries the material narrative event (Uganda border closure, Tedros ceasefire call, first survivor released) in primary_source. country_breakdown.csv mirrored with DRC and Uganda 27 May rows (DRC 1077/121/238/17 carried forward; Uganda 0/7/0/1 carried forward).</t>
+          <t>• 2026-05-27 (PM run, DRC MoH 27 May situation report): [Xinhua, dated 28 May 00:39 UTC](https://english.news.cn/africa/20260528/1bc05fdf07f44f6e837a9117e6a715ec/c.html), datelined Kinshasa 27 May, reports the DRC MoH situation report "released Wednesday" with "figures compiled as of Tuesday [26 May]": DRC 1,077 sus / 121 conf / 238 sus deaths / 17 conf deaths; 13 health zones across Ituri / Nord-Kivu / Sud-Kivu (Ituri remains epicenter). Cumulative since 15 May outbreak declaration. Uganda unchanged at 7 conf / 1 death per Uganda MoH (corroborated by AP / PBS 27 May which also cites &gt;3,000 possible contacts under investigation in DRC). Treated as fresher reconciled DRC MoH snapshot superseding the BNO News May 26 article (DRC 930/112/223/17), which was based on the DRC MoH morning May 26 bulletin (likely as-of-25 May cutoff).</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-27 (PM run): OBSERVED_REVISION_RANGE updated from "&lt;1-35%" to "&lt;1-35%" — today's upward revisions (sus +15.81%, conf +7.56%, total +14.87%, sus_deaths +6.73%) all sit inside the existing range; no constant change needed. LAST_SITREP_STABLE_DATE unchanged at 2026-05-24 (Sitrep 02 still the latest WHO publication). Real-time signal pass on x.com skipped on this PM run (the DRC MoH situation report via Xinhua and the AP wire on Uganda's border closure are higher-tier sources than any x.com tweet would be; the wire services have already absorbed the credentialed-account substance). Charts and XLSX regenerated; output PNG filenames now dated 2026-05-27.</t>
+          <t>• 2026-05-27 (PM run) — May 26 row revised per DRC MoH 27 May situation report (via Xinhua): suspected_global 930→1077 (+15.81%), confirmed_global 119→128 (+7.56%), total_global 1049→1205 (+14.87%), suspected_deaths_global 223→238 (+6.73%). All four revisions upward; no no-dip-rule trigger. country_breakdown.csv May 26 DRC row mirrored: sus 930→1077, conf 112→121, sus_deaths 223→238, confirmed_deaths 17 (unchanged). Uganda May 26 row unchanged at 7 conf / 1 death; primary_source updated to cite AP / PBS / Bloomberg / Washington Post 27 May coverage. The DRC MoH situation report is a single high-value source (per METHODOLOGY.md: "DRC Ministry of Health official press releases" are high-value), and all revisions are upward, so single-source backing is sufficient.</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-27 (PM run, post-commit correction — caught by Web): The PM run skipped the x.com pass against the explicit SKILL.md rule never to declare the real-time pass complete without confirming BNO @BNOFeed's most recent post. Web flagged the miss. Subsequent x.com pass via Web's signed-in Chrome surfaced the BNO @BNOFeed Daily Ebola Update for May 27 (graphic posted ~13h before this check), sourced to DRC MoH + Uganda MoH + WHO. Graphic reports: DR Congo 1,198 cases (+156) / 263 deaths (+23); Uganda 7 conf / 1 death (unchanged); TOTAL 1,205 cases / 264 deaths. Total cases (1,205) matches our committed May 26/27 rows exactly and reconciles with Xinhua/DRC MoH (1,077 sus + 121 conf + Uganda 7 = 1,205). Total deaths (264) implies DRC conf_deaths = 25 (264 - 1 Uganda - 238 sus = 25), revising the value carried from the prior BNO May 26 article from 17 to 25 (+8). BNO website (bnonews.com/index.php/category/health/) has not yet published a May 27 article; the @BNOFeed graphic is the primary citation for the conf_deaths refinement. The BNO graphic is a credentialed-wire primary source under METHODOLOGY.md tier 5, and the revision is upward, so single-source backing is sufficient.</t>
+          <t>• 2026-05-27 (PM run) — Appended May 27 row to timeseries.csv: 1077/128/1205/238 carried forward from revised May 26 row, since DRC MoH 27 May situation report has data cutoff 26 May and no fresher cumulative figure has been published for 27 May. The 27 May row carries the material narrative event (Uganda border closure, Tedros ceasefire call, first survivor released) in primary_source. country_breakdown.csv mirrored with DRC and Uganda 27 May rows (DRC 1077/121/238/17 carried forward; Uganda 0/7/0/1 carried forward).</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-27 (PM run, post-commit correction) — country_breakdown.csv May 26 DRC confirmed_deaths revised 17→25 per BNO @BNOFeed Daily Ebola Update May 27 graphic; May 27 DRC row carried forward at 25. timeseries.csv tracks suspected_deaths_global only and is unchanged (238). Primary_source fields on the May 26 and May 27 timeseries rows amended to flag both the Xinhua/DRC MoH and the BNO @BNOFeed graphic as the reconciling sources, with the 17→25 conf_deaths split called out explicitly. story.md unchanged (narrative event is still Uganda border closure + DRC MoH situation report; conf_deaths refinement is wire-level data, not a narrative shift). declarations.csv unchanged. LAST_SITREP_STABLE_DATE and OBSERVED_REVISION_RANGE unchanged.</t>
+          <t>• 2026-05-27 (PM run): OBSERVED_REVISION_RANGE updated from "&lt;1-35%" to "&lt;1-35%" — today's upward revisions (sus +15.81%, conf +7.56%, total +14.87%, sus_deaths +6.73%) all sit inside the existing range; no constant change needed. LAST_SITREP_STABLE_DATE unchanged at 2026-05-24 (Sitrep 02 still the latest WHO publication). Real-time signal pass on x.com skipped on this PM run (the DRC MoH situation report via Xinhua and the AP wire on Uganda's border closure are higher-tier sources than any x.com tweet would be; the wire services have already absorbed the credentialed-account substance). Charts and XLSX regenerated; output PNG filenames now dated 2026-05-27.</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-27 (PM run, methodology refinement per Web): When x.com is throttling, BNO's website (https://bnonews.com/index.php/category/health/) is an easier-to-scrape alternative for the BNO Daily Ebola Update — though as of this run the website's latest Ebola article is still the May 26 "1,049 cases / 241 deaths" piece, while @BNOFeed has already posted the May 27 graphic. The website lags @BNOFeed by ~1 day. Procedure going forward: scan BOTH sources before declaring the BNO check complete — the website for stable URLs and earlier-day articles, the @BNOFeed X account for the latest Daily Update graphic. SKILL.md is the place to record this; will note in commit message.</t>
+          <t>• 2026-05-27 (PM run, post-commit correction — caught by Web): The PM run skipped the x.com pass against the explicit SKILL.md rule never to declare the real-time pass complete without confirming BNO @BNOFeed's most recent post. Web flagged the miss. Subsequent x.com pass via Web's signed-in Chrome surfaced the BNO @BNOFeed Daily Ebola Update for May 27 (graphic posted ~13h before this check), sourced to DRC MoH + Uganda MoH + WHO. Graphic reports: DR Congo 1,198 cases (+156) / 263 deaths (+23); Uganda 7 conf / 1 death (unchanged); TOTAL 1,205 cases / 264 deaths. Total cases (1,205) matches our committed May 26/27 rows exactly and reconciles with Xinhua/DRC MoH (1,077 sus + 121 conf + Uganda 7 = 1,205). Total deaths (264) implies DRC conf_deaths = 25 (264 - 1 Uganda - 238 sus = 25), revising the value carried from the prior BNO May 26 article from 17 to 25 (+8). BNO website (bnonews.com/index.php/category/health/) has not yet published a May 27 article; the @BNOFeed graphic is the primary citation for the conf_deaths refinement. The BNO graphic is a credentialed-wire primary source under METHODOLOGY.md tier 5, and the revision is upward, so single-source backing is sufficient.</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-27 (PM run, methodology change per Web): Lookback window reduced from 7 days to 3 days. Rationale: after a week of observed revisions, the actual revision pattern is concentrated in the last 1-3 days. WHO Sitrep publications give a single "as of" date data point rather than revising a multi-day window, so the 7-day scan was checking many rows that never get revised. METHODOLOGY.md updated accordingly. No tracker rows changed by this; future runs will spend less time re-checking stable rows.</t>
+          <t>• 2026-05-27 (PM run, post-commit correction) — country_breakdown.csv May 26 DRC confirmed_deaths revised 17→25 per BNO @BNOFeed Daily Ebola Update May 27 graphic; May 27 DRC row carried forward at 25. timeseries.csv tracks suspected_deaths_global only and is unchanged (238). Primary_source fields on the May 26 and May 27 timeseries rows amended to flag both the Xinhua/DRC MoH and the BNO @BNOFeed graphic as the reconciling sources, with the 17→25 conf_deaths split called out explicitly. story.md unchanged (narrative event is still Uganda border closure + DRC MoH situation report; conf_deaths refinement is wire-level data, not a narrative shift). declarations.csv unchanged. LAST_SITREP_STABLE_DATE and OBSERVED_REVISION_RANGE unchanged.</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-28 (scheduled run): Appended May 28 row to timeseries.csv at 1,077 sus / 137 conf / 1,214 total / 246 sus_deaths, sourced to the [Africa CDC press briefing (DG Jean Kaseya), reported via CIDRAP](https://www.cidrap.umn.edu/ebola/uganda-shuts-dr-congo-border-ebola-outbreak-continues-grow). Africa CDC's reconciled DRC figures: 1,077 sus / 129 conf / 246 sus_deaths / 18 conf_deaths. Uganda: 8 conf / 1 death (conf +1 vs May 27 row's 7). Global revisions vs May 27 row: sus unchanged (1,077), conf +9 (128→137), total +9 (1,205→1,214), sus_deaths +8 (238→246). All revisions upward; no no-dip trigger on timeseries cumulative columns. 3-day lookback against May 26 and May 27 rows: no revisions required (those rows already reflect DRC MoH 27 May situation report cutoff for May 26 data; Africa CDC May 28 cutoff goes into the new row).</t>
+          <t>• 2026-05-27 (PM run, methodology refinement per Web): When x.com is throttling, BNO's website (https://bnonews.com/index.php/category/health/) is an easier-to-scrape alternative for the BNO Daily Ebola Update — though as of this run the website's latest Ebola article is still the May 26 "1,049 cases / 241 deaths" piece, while @BNOFeed has already posted the May 27 graphic. The website lags @BNOFeed by ~1 day. Procedure going forward: scan BOTH sources before declaring the BNO check complete — the website for stable URLs and earlier-day articles, the @BNOFeed X account for the latest Daily Update graphic. SKILL.md is the place to record this; will note in commit message.</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-28 (scheduled run, country_breakdown handling, lookback revision): Validator flagged a per-country no-dip violation on the first pass (DRC conf_deaths 25 May 27 → 18 May 28). Applied the Africa CDC reconciled split retroactively to May 26 and May 27 rows under the lookback policy, since the prior 25 was inferred from the BNO @BNOFeed 27 May graphic's DRC total deaths (263) minus suspected (238) — Africa CDC's directly-stated DRC split (246 sus_deaths / 18 conf_deaths) is the higher-tier reconciled figure and supersedes the inferred wire-graphic value. Revisions: timeseries.csv May 26 sus_deaths_global 238→246 (+3.36% upward), May 27 sus_deaths_global 238→246 (carried). country_breakdown.csv DRC May 26 sus_deaths 238→246 and conf_deaths 25→18; DRC May 27 sus_deaths 238→246 and conf_deaths 25→18. All cumulative columns now non-decreasing per country (sus_deaths 223→246→246→246; conf_deaths 10→18→18→18). Cumulative TOTAL DRC deaths rises from 263 (BNO 27 May graphic) to 264 (Africa CDC reconciled), +1 net upward — not a dip. country_breakdown.csv May 28 DRC: 1,077 / 129 / 246 / 18; Uganda 0 / 8 / 0 / 1. Validator passes after revision.</t>
+          <t>• 2026-05-27 (PM run, methodology change per Web): Lookback window reduced from 7 days to 3 days. Rationale: after a week of observed revisions, the actual revision pattern is concentrated in the last 1-3 days. WHO Sitrep publications give a single "as of" date data point rather than revising a multi-day window, so the 7-day scan was checking many rows that never get revised. METHODOLOGY.md updated accordingly. No tracker rows changed by this; future runs will spend less time re-checking stable rows.</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-28 (scheduled run, BNO real-time pass): BNO website (bnonews.com/index.php/category/health/) latest Ebola article remains the May 26 "1,049 cases / 241 deaths" piece — website lag of ~2 days. BNO @BNOFeed Daily Ebola Update for May 28 (posted 6:15 PM May 28, status 2060122917665415544) reports anomalously low figures: "Total cases: 1,038 / Total deaths: 241" with no delta in parens (breaking BNOFeed's prior "(+X)" format). Both figures are below the May 26 BNO News article (1,049 / 241) and far below the May 27 BNOFeed graphic (1,205 / 264) and today's Africa CDC briefing (1,214 / 265). Treated as a stale or inconsistent automated BNO wire snapshot and NOT applied. Africa CDC's directly-attributed briefing figures take precedence under source-preference order. Will recheck BNO next run for a corrected post.</t>
+          <t>• 2026-05-28 (scheduled run): Appended May 28 row to timeseries.csv at 1,077 sus / 137 conf / 1,214 total / 246 sus_deaths, sourced to the [Africa CDC press briefing (DG Jean Kaseya), reported via CIDRAP](https://www.cidrap.umn.edu/ebola/uganda-shuts-dr-congo-border-ebola-outbreak-continues-grow). Africa CDC's reconciled DRC figures: 1,077 sus / 129 conf / 246 sus_deaths / 18 conf_deaths. Uganda: 8 conf / 1 death (conf +1 vs May 27 row's 7). Global revisions vs May 27 row: sus unchanged (1,077), conf +9 (128→137), total +9 (1,205→1,214), sus_deaths +8 (238→246). All revisions upward; no no-dip trigger on timeseries cumulative columns. 3-day lookback against May 26 and May 27 rows: no revisions required (those rows already reflect DRC MoH 27 May situation report cutoff for May 26 data; Africa CDC May 28 cutoff goes into the new row).</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-28 (scheduled run, x.com credentialed-account pass): Web's signed-in Chrome reachable via list_connected_browsers → select_browser (deviceId 5fdc215b-0b1a-4a16-9f71-01f672b11fbf). Credentialed-account pass surfaced the BNO @BNOFeed anomaly above plus narrative items already captured in the CIDRAP write-up (Tedros Bunia visit + ceasefire call; EU aid arrived in Bunia; US State Dept $80M + $50M allocations; US-Kenya 50-bed quarantine unit confirmed; Africa CDC $500M→$290M funding gap; Save the Children: ~25% of DRC confirmed deaths in children; The Guardian: several DRC doctors and nurses have died after contracting Ebola). No additional numerical revisions warranted from real-time pass.</t>
+          <t>• 2026-05-28 (scheduled run, country_breakdown handling, lookback revision): Validator flagged a per-country no-dip violation on the first pass (DRC conf_deaths 25 May 27 → 18 May 28). Applied the Africa CDC reconciled split retroactively to May 26 and May 27 rows under the lookback policy, since the prior 25 was inferred from the BNO @BNOFeed 27 May graphic's DRC total deaths (263) minus suspected (238) — Africa CDC's directly-stated DRC split (246 sus_deaths / 18 conf_deaths) is the higher-tier reconciled figure and supersedes the inferred wire-graphic value. Revisions: timeseries.csv May 26 sus_deaths_global 238→246 (+3.36% upward), May 27 sus_deaths_global 238→246 (carried). country_breakdown.csv DRC May 26 sus_deaths 238→246 and conf_deaths 25→18; DRC May 27 sus_deaths 238→246 and conf_deaths 25→18. All cumulative columns now non-decreasing per country (sus_deaths 223→246→246→246; conf_deaths 10→18→18→18). Cumulative TOTAL DRC deaths rises from 263 (BNO 27 May graphic) to 264 (Africa CDC reconciled), +1 net upward — not a dip. country_breakdown.csv May 28 DRC: 1,077 / 129 / 246 / 18; Uganda 0 / 8 / 0 / 1. Validator passes after revision.</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-28 (scheduled run, declarations.csv): No change. Uganda border closure was logged 27 May. CDC HAN unchanged. CDC Travel Health Notice levels unchanged (DRC remains Level 3; Uganda remains Level 1). CDC Situation Summary page at https://www.cdc.gov/ebola/situation-summary/index.html still reflects the May 16 state (8 confirmed / 248 suspected) with Resources block pointing at the DRC Level 2 travel notice — consistent with the 2026-05-27 AM-run observation that the brief May 25 refresh appears to have been rolled back. The live DRC travel notice URL still resolves to Level 3, so declarations.csv DRC `cdc_travel_notice_level` is unchanged.</t>
+          <t>• 2026-05-28 (scheduled run, BNO real-time pass): BNO website (bnonews.com/index.php/category/health/) latest Ebola article remains the May 26 "1,049 cases / 241 deaths" piece — website lag of ~2 days. BNO @BNOFeed Daily Ebola Update for May 28 (posted 6:15 PM May 28, status 2060122917665415544) reports anomalously low figures: "Total cases: 1,038 / Total deaths: 241" with no delta in parens (breaking BNOFeed's prior "(+X)" format). Both figures are below the May 26 BNO News article (1,049 / 241) and far below the May 27 BNOFeed graphic (1,205 / 264) and today's Africa CDC briefing (1,214 / 265). Treated as a stale or inconsistent automated BNO wire snapshot and NOT applied. Africa CDC's directly-attributed briefing figures take precedence under source-preference order. Will recheck BNO next run for a corrected post.</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-28 (scheduled run, story.md): Refreshed "Latest update" section from May 27 (Uganda border closure, DRC MoH 1,077/121/238/17 figures, Tedros ceasefire tweet, first survivor release) to May 28 (Africa CDC briefing reconciled figures 1,077/129/246/18 DRC plus Uganda 8/1; Tedros message to people of DRC + Bunia travel announcement; EU aid delivery to Bunia; US State Dept $80M + $50M allocations; US-Kenya 50-bed quarantine unit confirmed and IDSA criticism; Africa CDC funding-gap warning $500M→$290M; Save the Children children death share). "Story so far" section unchanged (slow-moving context).</t>
+          <t>• 2026-05-28 (scheduled run, x.com credentialed-account pass): Web's signed-in Chrome reachable via list_connected_browsers → select_browser (deviceId 5fdc215b-0b1a-4a16-9f71-01f672b11fbf). Credentialed-account pass surfaced the BNO @BNOFeed anomaly above plus narrative items already captured in the CIDRAP write-up (Tedros Bunia visit + ceasefire call; EU aid arrived in Bunia; US State Dept $80M + $50M allocations; US-Kenya 50-bed quarantine unit confirmed; Africa CDC $500M→$290M funding gap; Save the Children: ~25% of DRC confirmed deaths in children; The Guardian: several DRC doctors and nurses have died after contracting Ebola). No additional numerical revisions warranted from real-time pass.</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-28 (scheduled run, chart constants): LAST_SITREP_STABLE_DATE unchanged at 2026-05-24 (no Sitrep 03 yet; latest WHO publication remains Sitrep 02 from 27 May with 24 May cutoff). OBSERVED_REVISION_RANGE unchanged at "&lt;1-35%" — today's upward revisions sit inside the range (conf +0.78% scale, sus_deaths +3.36%, Uganda conf +14.3%). Charts and XLSX regenerated; output PNG filenames now dated 2026-05-28.</t>
+          <t>• 2026-05-28 (scheduled run, declarations.csv): No change. Uganda border closure was logged 27 May. CDC HAN unchanged. CDC Travel Health Notice levels unchanged (DRC remains Level 3; Uganda remains Level 1). CDC Situation Summary page at https://www.cdc.gov/ebola/situation-summary/index.html still reflects the May 16 state (8 confirmed / 248 suspected) with Resources block pointing at the DRC Level 2 travel notice — consistent with the 2026-05-27 AM-run observation that the brief May 25 refresh appears to have been rolled back. The live DRC travel notice URL still resolves to Level 3, so declarations.csv DRC `cdc_travel_notice_level` is unchanged.</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-28 (scheduled run, sweeper health): No stale .git/*.lock or .git/objects/*/tmp_obj_* files at session start — launchd job com.webbegole.gitlock-sweep working as designed.</t>
+          <t>• 2026-05-28 (scheduled run, story.md): Refreshed "Latest update" section from May 27 (Uganda border closure, DRC MoH 1,077/121/238/17 figures, Tedros ceasefire tweet, first survivor release) to May 28 (Africa CDC briefing reconciled figures 1,077/129/246/18 DRC plus Uganda 8/1; Tedros message to people of DRC + Bunia travel announcement; EU aid delivery to Bunia; US State Dept $80M + $50M allocations; US-Kenya 50-bed quarantine unit confirmed and IDSA criticism; Africa CDC funding-gap warning $500M→$290M; Save the Children children death share). "Story so far" section unchanged (slow-moving context).</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-28 (scheduled run, user message during run): Web sent an in-run message asking to "update instructions to clarify that I am just a researcher." The existing project CLAUDE.md ("public health data tracker for academic research purposes") and SKILL.md ("public-health data tracker compiling publicly available case counts from official sources. Academic / journalistic use. No medical advice.") already specify academic-research framing. No changes made to project instructions or SKILL.md during this run — surfaced in the final report so Web can edit the Cowork project instructions or SKILL.md himself if he wants additional explicit "individual academic researcher" language.</t>
+          <t>• 2026-05-28 (scheduled run, chart constants): LAST_SITREP_STABLE_DATE unchanged at 2026-05-24 (no Sitrep 03 yet; latest WHO publication remains Sitrep 02 from 27 May with 24 May cutoff). OBSERVED_REVISION_RANGE unchanged at "&lt;1-35%" — today's upward revisions sit inside the range (conf +0.78% scale, sus_deaths +3.36%, Uganda conf +14.3%). Charts and XLSX regenerated; output PNG filenames now dated 2026-05-28.</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-30 (scheduled run, major reconciliation): [WHO DON605](https://www.who.int/emergencies/disease-outbreak-news/item/2026-DON605) published 29 May 2026 (URL active 30 May) supersedes the DRC-MoH-attributed running counts that had been in the May 26, 27, 28 rows. WHO-reconciled DRC figures as of 27 May: 906 sus / 125 conf / 223 sus_deaths / 17 conf_deaths. Uganda 9 conf / 1 death as of 29 May. Global confirmed 134 (DRC 125 + Uganda 9) and global confirmed deaths 18 (DRC 17 + Uganda 1). Plus one US doctor case in Germany, treated as DRC case per country-of-exposure convention. WHO Sitrep 02 (24 May cutoff) had DRC sus 906 — DON605's 27 May cutoff confirms WHO has NOT reconciled the post-Sitrep-02 DRC MoH-attributed surge to 1,077 carried by Xinhua / Africa CDC briefing.</t>
+          <t>• 2026-05-28 (scheduled run, sweeper health): No stale .git/*.lock or .git/objects/*/tmp_obj_* files at session start — launchd job com.webbegole.gitlock-sweep working as designed.</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-30 (scheduled run, no-dip rule application): No-dip-rule two-source threshold met by (1) WHO DON605 and (2) WHO DG Tedros's remarks on 29 May, carried by [PBS via AP, 30 May](https://www.pbs.org/newshour/world/who-chief-visits-congo-ebola-epicenter-as-cases-outpace-response) and [NBC via AP, 30 May](https://www.nbcnews.com/world/africa/who-tedros-eastern-congo-epicenter-ebola-outbreak-rcna347668): "The WHO said Friday authorities have reported 906 suspected cases and 223 suspected deaths." Both WHO official publication and WHO DG statement are listed in METHODOLOGY.md "High-value sources." The DRC-MoH-attributed higher figures (still being reported via BNO @BNOFeed daily graphics) are tier-5 wire snapshots; per source-preference order WHO &gt; DRC MoH, and the dip is applied.</t>
+          <t>• 2026-05-28 (scheduled run, user message during run): Web sent an in-run message asking to "update instructions to clarify that I am just a researcher." The existing project CLAUDE.md ("public health data tracker for academic research purposes") and SKILL.md ("public-health data tracker compiling publicly available case counts from official sources. Academic / journalistic use. No medical advice.") already specify academic-research framing. No changes made to project instructions or SKILL.md during this run — surfaced in the final report so Web can edit the Cowork project instructions or SKILL.md himself if he wants additional explicit "individual academic researcher" language.</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-30 (scheduled run) — May 26 row revised per WHO DON605: suspected_global 1077→906 (-15.88%), confirmed_global 128→112 (-12.50%), total_global 1205→1018 (-15.51%), suspected_deaths_global 246→223 (-9.35%). country_breakdown.csv May 26 DRC: 1077/121/246/18 → 906/105/223/10. Uganda row unchanged at 7/1. DRC confirmed and conf_deaths use Sitrep 02 carry-forward (no DON605 26 May-specific confirmed figure).</t>
+          <t>• 2026-05-30 (scheduled run, major reconciliation): [WHO DON605](https://www.who.int/emergencies/disease-outbreak-news/item/2026-DON605) published 29 May 2026 (URL active 30 May) supersedes the DRC-MoH-attributed running counts that had been in the May 26, 27, 28 rows. WHO-reconciled DRC figures as of 27 May: 906 sus / 125 conf / 223 sus_deaths / 17 conf_deaths. Uganda 9 conf / 1 death as of 29 May. Global confirmed 134 (DRC 125 + Uganda 9) and global confirmed deaths 18 (DRC 17 + Uganda 1). Plus one US doctor case in Germany, treated as DRC case per country-of-exposure convention. WHO Sitrep 02 (24 May cutoff) had DRC sus 906 — DON605's 27 May cutoff confirms WHO has NOT reconciled the post-Sitrep-02 DRC MoH-attributed surge to 1,077 carried by Xinhua / Africa CDC briefing.</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-30 (scheduled run) — May 27 row revised per WHO DON605 (data as of 27 May): suspected_global 1077→906 (-15.88%), confirmed_global 128→132 (+3.13% — DRC conf rose to 125 per DON605 explicit), total_global 1205→1038 (-13.86%), suspected_deaths_global 246→223 (-9.35%). country_breakdown.csv May 27 DRC: 1077/121/246/18 → 906/125/223/17. Uganda 7/1 unchanged.</t>
+          <t>• 2026-05-30 (scheduled run, no-dip rule application): No-dip-rule two-source threshold met by (1) WHO DON605 and (2) WHO DG Tedros's remarks on 29 May, carried by [PBS via AP, 30 May](https://www.pbs.org/newshour/world/who-chief-visits-congo-ebola-epicenter-as-cases-outpace-response) and [NBC via AP, 30 May](https://www.nbcnews.com/world/africa/who-tedros-eastern-congo-epicenter-ebola-outbreak-rcna347668): "The WHO said Friday authorities have reported 906 suspected cases and 223 suspected deaths." Both WHO official publication and WHO DG statement are listed in METHODOLOGY.md "High-value sources." The DRC-MoH-attributed higher figures (still being reported via BNO @BNOFeed daily graphics) are tier-5 wire snapshots; per source-preference order WHO &gt; DRC MoH, and the dip is applied.</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-30 (scheduled run) — May 28 row revised: suspected_global 1077→906 (-15.88%), confirmed_global 137→133 (-2.92%), total_global 1214→1039 (-14.41%), suspected_deaths_global 246→223 (-9.35%). country_breakdown.csv May 28 DRC: 1077/129/246/18 → 906/125/223/17. Uganda 8/1 unchanged (Africa CDC May 28 briefing +1 vs May 27 preserved; consistent with DON605's 9 by 29 May).</t>
+          <t>• 2026-05-30 (scheduled run) — May 26 row revised per WHO DON605: suspected_global 1077→906 (-15.88%), confirmed_global 128→112 (-12.50%), total_global 1205→1018 (-15.51%), suspected_deaths_global 246→223 (-9.35%). country_breakdown.csv May 26 DRC: 1077/121/246/18 → 906/105/223/10. Uganda row unchanged at 7/1. DRC confirmed and conf_deaths use Sitrep 02 carry-forward (no DON605 26 May-specific confirmed figure).</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-30 (scheduled run) — Appended May 29 row to timeseries.csv: 906/134/1040/223 per WHO DON605 (sus and sus_deaths from 27 May cutoff carried forward; conf 134 = DRC 125 + Uganda 9 from 29 May cutoff). country_breakdown.csv May 29: DRC 906/125/223/17 (DON605 explicit); Uganda 9/1 (DON605 + BNO @BNOFeed post-confirmation of +2 Kampala Congolese nationals on 29 May).</t>
+          <t>• 2026-05-30 (scheduled run) — May 27 row revised per WHO DON605 (data as of 27 May): suspected_global 1077→906 (-15.88%), confirmed_global 128→132 (+3.13% — DRC conf rose to 125 per DON605 explicit), total_global 1205→1038 (-13.86%), suspected_deaths_global 246→223 (-9.35%). country_breakdown.csv May 27 DRC: 1077/121/246/18 → 906/125/223/17. Uganda 7/1 unchanged.</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-30 (scheduled run, source-view divergence flag): DRC MoH-attributed running count via BNO @BNOFeed Daily Ebola Update graphics shows materially higher figures than WHO-reconciled: BNO 28 May graphic DRC 1,031 cases / 240 deaths; BNO 29 May graphic ~1,028 sus / 225 conf / 240 deaths (DRC MoH ramped up lab testing 29 May, +100 confirmed in one day). DRC MoH cumulative TOTAL (~1,253 cases) is +213 above WHO DON605's reconciled total (1,040). The +100 lab-confirmation surge is operationally significant and represents real epidemiological work, but WHO has not yet integrated it into a WHO publication. WHO Sitrep 03 expected Tue 2 Jun will likely reflect partial catch-up. Per source-preference order, WHO DON605 wins for the row's cumulative attribution; DRC MoH running counts recorded in primary_source fields and country_breakdown notes for transparency.</t>
+          <t>• 2026-05-30 (scheduled run) — May 28 row revised: suspected_global 1077→906 (-15.88%), confirmed_global 137→133 (-2.92%), total_global 1214→1039 (-14.41%), suspected_deaths_global 246→223 (-9.35%). country_breakdown.csv May 28 DRC: 1077/129/246/18 → 906/125/223/17. Uganda 8/1 unchanged (Africa CDC May 28 briefing +1 vs May 27 preserved; consistent with DON605's 9 by 29 May).</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-30 (scheduled run, BNO real-time pass): Web's signed-in Chrome reachable via list_connected_browsers → select_browser (deviceId 5fdc215b-0b1a-4a16-9f71-01f672b11fbf). BNO @BNOFeed most recent post is 29 May Daily Ebola Update graphic (18h before pass) — Total cases 1,262 / Total deaths 241 / DRC suspected ~1,028 / DRC confirmed 225 / Uganda 9. The +100 DRC confirmed surge on 29 May was captured. BNO website (bnonews.com/index.php/category/health/) front page no longer shows any Ebola article (lag of ~3 days vs @BNOFeed).</t>
+          <t>• 2026-05-30 (scheduled run) — Appended May 29 row to timeseries.csv: 906/134/1040/223 per WHO DON605 (sus and sus_deaths from 27 May cutoff carried forward; conf 134 = DRC 125 + Uganda 9 from 29 May cutoff). country_breakdown.csv May 29: DRC 906/125/223/17 (DON605 explicit); Uganda 9/1 (DON605 + BNO @BNOFeed post-confirmation of +2 Kampala Congolese nationals on 29 May).</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-30 (scheduled run, x.com credentialed-account pass): Other credentialed-account posts on the @BNOFeed timeline and surrounding context already absorbed into the WHO DON605-based reconciliation; no additional numerical revisions warranted. Material narrative events captured in story.md "Latest update" refresh: WHO DG Tedros arrived in Bunia 30 May; MSF DDoO Dr Alan Gonzalez statement ("Never before has an Ebola outbreak recorded so many cases so soon after its declaration"); Kenyan court blocked US Ebola quarantine center plan; Trump administration entry ban on non-US passport holders from DRC/Uganda/South Sudan.</t>
+          <t>• 2026-05-30 (scheduled run, source-view divergence flag): DRC MoH-attributed running count via BNO @BNOFeed Daily Ebola Update graphics shows materially higher figures than WHO-reconciled: BNO 28 May graphic DRC 1,031 cases / 240 deaths; BNO 29 May graphic ~1,028 sus / 225 conf / 240 deaths (DRC MoH ramped up lab testing 29 May, +100 confirmed in one day). DRC MoH cumulative TOTAL (~1,253 cases) is +213 above WHO DON605's reconciled total (1,040). The +100 lab-confirmation surge is operationally significant and represents real epidemiological work, but WHO has not yet integrated it into a WHO publication. WHO Sitrep 03 expected Tue 2 Jun will likely reflect partial catch-up. Per source-preference order, WHO DON605 wins for the row's cumulative attribution; DRC MoH running counts recorded in primary_source fields and country_breakdown notes for transparency.</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-30 (scheduled run, story.md): Refreshed "Latest update" from 28 May Africa CDC briefing to 30 May Tedros Bunia visit + WHO DON605 reconciled figures + DRC MoH lab-testing ramp-up + MSF "Nobody knows the true scale and severity of this outbreak" warning + Kenyan court block on US quarantine plan. "Story so far" section unchanged (slow-moving context).</t>
+          <t>• 2026-05-30 (scheduled run, BNO real-time pass): Web's signed-in Chrome reachable via list_connected_browsers → select_browser (deviceId 5fdc215b-0b1a-4a16-9f71-01f672b11fbf). BNO @BNOFeed most recent post is 29 May Daily Ebola Update graphic (18h before pass) — Total cases 1,262 / Total deaths 241 / DRC suspected ~1,028 / DRC confirmed 225 / Uganda 9. The +100 DRC confirmed surge on 29 May was captured. BNO website (bnonews.com/index.php/category/health/) front page no longer shows any Ebola article (lag of ~3 days vs @BNOFeed).</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-30 (scheduled run, declarations.csv): No change. CDC HAN 00530 unchanged. CDC Travel Health Notice levels unchanged (DRC remains Level 3 per verified URL https://wwwnc.cdc.gov/travel/notices/level3/ebola-democratic-republic-of-the-congo; Uganda remains Level 1 per https://wwwnc.cdc.gov/travel/notices/level1/ebola-uganda). The Trump administration entry ban on non-US passport holders who recently visited DRC/Uganda/South Sudan (per PBS/NBC AP wires) is a separate executive-branch travel restriction beyond CDC Travel Health Notices and was instituted "last week" per the PBS report; that policy is informational here, not a CDC HAN or Travel Notice level change. Will surface in declarations.csv `notes` field if it becomes a CDC HAN amendment.</t>
+          <t>• 2026-05-30 (scheduled run, x.com credentialed-account pass): Other credentialed-account posts on the @BNOFeed timeline and surrounding context already absorbed into the WHO DON605-based reconciliation; no additional numerical revisions warranted. Material narrative events captured in story.md "Latest update" refresh: WHO DG Tedros arrived in Bunia 30 May; MSF DDoO Dr Alan Gonzalez statement ("Never before has an Ebola outbreak recorded so many cases so soon after its declaration"); Kenyan court blocked US Ebola quarantine center plan; Trump administration entry ban on non-US passport holders from DRC/Uganda/South Sudan.</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-30 (scheduled run, chart constants): LAST_SITREP_STABLE_DATE unchanged at 2026-05-24 (no Sitrep 03 yet; latest WHO Sitrep remains Sitrep 02 from 27 May with 24 May cutoff). DON605 doesn't update LAST_SITREP_STABLE_DATE — that constant is specifically for WHO Weekly Sitreps per the comment in generate_charts.py. OBSERVED_REVISION_RANGE unchanged at "&lt;1-35%" — today's downward revisions (sus -15.88%, conf -12.50% to -2.92%, total -15.51% to -13.86%, sus_deaths -9.35%) sit inside the absolute-magnitude range; the chart-footnote text describes upward revisions only, which remains the historical pattern (today's lookback is a downward reconciliation from a DRC-MoH-attributed surge that exceeded WHO Sitrep 02).</t>
+          <t>• 2026-05-30 (scheduled run, story.md): Refreshed "Latest update" from 28 May Africa CDC briefing to 30 May Tedros Bunia visit + WHO DON605 reconciled figures + DRC MoH lab-testing ramp-up + MSF "Nobody knows the true scale and severity of this outbreak" warning + Kenyan court block on US quarantine plan. "Story so far" section unchanged (slow-moving context).</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-30 (scheduled run, sweeper health): No stale .git/*.lock or .git/objects/*/tmp_obj_* files at session start — launchd job com.webbegole.gitlock-sweep working as designed.</t>
+          <t>• 2026-05-30 (scheduled run, declarations.csv): No change. CDC HAN 00530 unchanged. CDC Travel Health Notice levels unchanged (DRC remains Level 3 per verified URL https://wwwnc.cdc.gov/travel/notices/level3/ebola-democratic-republic-of-the-congo; Uganda remains Level 1 per https://wwwnc.cdc.gov/travel/notices/level1/ebola-uganda). The Trump administration entry ban on non-US passport holders who recently visited DRC/Uganda/South Sudan (per PBS/NBC AP wires) is a separate executive-branch travel restriction beyond CDC Travel Health Notices and was instituted "last week" per the PBS report; that policy is informational here, not a CDC HAN or Travel Notice level change. Will surface in declarations.csv `notes` field if it becomes a CDC HAN amendment.</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-31 (scheduled run, BNO real-time pass): Web's signed-in Chrome reachable via list_connected_browsers → select_browser (deviceId 5fdc215b-0b1a-4a16-9f71-01f672b11fbf). BNO @BNOFeed Daily Ebola Update graphics surfaced for both May 30 (21h before pass) and May 31 (6h before pass). May 30 graphic reports cleaned-baseline DRC running figures: DR Congo 574 cases / 17 deaths (deltas marked N/A) with caption: "Today, Congo removed nearly 700 suspected cases after they tested negative for Ebola. This follows an increase in testing capabilities. As a result, it's unknown how many new cases were added today." Uganda 9 conf / 1 death (unchanged); TOTAL 583 cases / 18 deaths. May 31 graphic reports DRC running on the cleaned baseline: DR Congo 672 cases (+98) / 55 deaths (+38); Uganda 9 conf / 1 death (unchanged); TOTAL 681 (+98) / 56 (+38). The May 30 BNO graphic resolves the May 28 BNO anomaly (1,038/241 with no deltas) retrospectively as a transitional snapshot during DRC MoH's data cleanup pipeline ramp-up.</t>
+          <t>• 2026-05-30 (scheduled run, chart constants): LAST_SITREP_STABLE_DATE unchanged at 2026-05-24 (no Sitrep 03 yet; latest WHO Sitrep remains Sitrep 02 from 27 May with 24 May cutoff). DON605 doesn't update LAST_SITREP_STABLE_DATE — that constant is specifically for WHO Weekly Sitreps per the comment in generate_charts.py. OBSERVED_REVISION_RANGE unchanged at "&lt;1-35%" — today's downward revisions (sus -15.88%, conf -12.50% to -2.92%, total -15.51% to -13.86%, sus_deaths -9.35%) sit inside the absolute-magnitude range; the chart-footnote text describes upward revisions only, which remains the historical pattern (today's lookback is a downward reconciliation from a DRC-MoH-attributed surge that exceeded WHO Sitrep 02).</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-31 (scheduled run, no-dip rule application): DRC MoH ~700-case removal on 30 May is a DRC-MoH-attributed dip carried only by BNO @BNOFeed (a tier-5 wire source). The dip would imply: cumulative total cases 1,040 → 583 (-43.94%) and cumulative total deaths 224 → 18 (-91.96%). Per METHODOLOGY.md no-dip rule, a single high-value source proposing a downward revision is held pending corroboration by a second high-value source. WHO has not yet published a Sitrep 03 or DON606 reflecting the cleanup. WHO DG Tedros's 30 May Bunia press briefing was qualitative (community ownership, safe burials, calls to reconsider border closures); no figures cited that could serve as the second high-value source. Tedros's prior 29 May / 30 May AP-wire-attributed remarks cited the pre-cleanup 906/223 baseline (the no-dip threshold already met for the earlier DRC MoH surge that ran 1,077/240+). The May 30 cleanup is a different event: it pulls figures BELOW the WHO-reconciled DON605 baseline, which has no precedent in the data so far. Holding 906/134/1040/223 carried forward on the May 30 and May 31 rows.</t>
+          <t>• 2026-05-30 (scheduled run, sweeper health): No stale .git/*.lock or .git/objects/*/tmp_obj_* files at session start — launchd job com.webbegole.gitlock-sweep working as designed.</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-31 (scheduled run) — Appended May 30 row to timeseries.csv: 906/134/1040/223 carried forward per no-dip rule (DRC MoH ~700-case removal via BNO @BNOFeed May 30 graphic is single-source dip held pending WHO corroboration). country_breakdown.csv DRC May 30 row 906/125/223/17 carried forward with BNO graphic details in primary_source; Uganda May 30 row 0/9/0/1 carried forward.</t>
+          <t>• 2026-05-31 (scheduled run, BNO real-time pass): Web's signed-in Chrome reachable via list_connected_browsers → select_browser (deviceId 5fdc215b-0b1a-4a16-9f71-01f672b11fbf). BNO @BNOFeed Daily Ebola Update graphics surfaced for both May 30 (21h before pass) and May 31 (6h before pass). May 30 graphic reports cleaned-baseline DRC running figures: DR Congo 574 cases / 17 deaths (deltas marked N/A) with caption: "Today, Congo removed nearly 700 suspected cases after they tested negative for Ebola. This follows an increase in testing capabilities. As a result, it's unknown how many new cases were added today." Uganda 9 conf / 1 death (unchanged); TOTAL 583 cases / 18 deaths. May 31 graphic reports DRC running on the cleaned baseline: DR Congo 672 cases (+98) / 55 deaths (+38); Uganda 9 conf / 1 death (unchanged); TOTAL 681 (+98) / 56 (+38). The May 30 BNO graphic resolves the May 28 BNO anomaly (1,038/241 with no deltas) retrospectively as a transitional snapshot during DRC MoH's data cleanup pipeline ramp-up.</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-31 (scheduled run) — Appended May 31 row to timeseries.csv: 906/134/1040/223 carried forward per no-dip rule (DRC MoH cleaned-baseline running count via BNO @BNOFeed May 31 graphic is single-source dip held pending WHO corroboration). country_breakdown.csv DRC May 31 row 906/125/223/17 carried forward with BNO graphic details; Uganda May 31 row 0/9/0/1 carried forward.</t>
+          <t>• 2026-05-31 (scheduled run, no-dip rule application): DRC MoH ~700-case removal on 30 May is a DRC-MoH-attributed dip carried only by BNO @BNOFeed (a tier-5 wire source). The dip would imply: cumulative total cases 1,040 → 583 (-43.94%) and cumulative total deaths 224 → 18 (-91.96%). Per METHODOLOGY.md no-dip rule, a single high-value source proposing a downward revision is held pending corroboration by a second high-value source. WHO has not yet published a Sitrep 03 or DON606 reflecting the cleanup. WHO DG Tedros's 30 May Bunia press briefing was qualitative (community ownership, safe burials, calls to reconsider border closures); no figures cited that could serve as the second high-value source. Tedros's prior 29 May / 30 May AP-wire-attributed remarks cited the pre-cleanup 906/223 baseline (the no-dip threshold already met for the earlier DRC MoH surge that ran 1,077/240+). The May 30 cleanup is a different event: it pulls figures BELOW the WHO-reconciled DON605 baseline, which has no precedent in the data so far. Holding 906/134/1040/223 carried forward on the May 30 and May 31 rows.</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-31 (scheduled run, 3-day lookback): May 28, 29 rows checked against latest sources. WHO DON605 remains the latest WHO-reconciled cumulative cutoff (27 May for DRC sus/sus_deaths; 29 May for confirmed). No revisions required on May 28 or May 29 rows. May 27 row also stable per DON605.</t>
+          <t>• 2026-05-31 (scheduled run) — Appended May 30 row to timeseries.csv: 906/134/1040/223 carried forward per no-dip rule (DRC MoH ~700-case removal via BNO @BNOFeed May 30 graphic is single-source dip held pending WHO corroboration). country_breakdown.csv DRC May 30 row 906/125/223/17 carried forward with BNO graphic details in primary_source; Uganda May 30 row 0/9/0/1 carried forward.</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-31 (scheduled run, WHO DG Tedros Bunia press briefing): [WHO DG remarks at the press briefing on the Bundibugyo Ebola outbreak – 30 May 2026](https://www.who.int/news-room/speeches/item/who-director-general-s-remarks-at-the-press-briefing-on-the-on-the-bundibugyo-ebola-outbreak---30-may-2026) is community-focused and qualitative — no global case/death figures cited. Key passages: ""We are not here to tell people what to do. We are here to listen. Communities understand their own challenges and their own solutions."" / ""I would also ask countries that have imposed travel bans or border closures to reconsider. These measures make the response harder, and they discourage the transparency that saves lives."" / ""DRC has faced Ebola before, sixteen times, and has ended every outbreak. This is the seventeenth. That history gives me real confidence."" / ""Hand hygiene matters. Sharing accurate information matters. And safe, dignified burials matter too."" The Bunia visit will continue into 31 May.</t>
+          <t>• 2026-05-31 (scheduled run) — Appended May 31 row to timeseries.csv: 906/134/1040/223 carried forward per no-dip rule (DRC MoH cleaned-baseline running count via BNO @BNOFeed May 31 graphic is single-source dip held pending WHO corroboration). country_breakdown.csv DRC May 31 row 906/125/223/17 carried forward with BNO graphic details; Uganda May 31 row 0/9/0/1 carried forward.</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-31 (scheduled run, story.md): Refreshed ""Latest update"" section to a 31 May lead. New section opens with the WHO DG Tedros 30 May Bunia press briefing reframe (community-led response, border-closure pushback), then explains the 30 May DRC MoH ~700-case reclassification and the WHO-vs-DRC-MoH source-view divergence, then closes with the standing context (no vaccine, conflict, community resistance, MSF warning, Kenya court block). The DRC MoH cycle (suspected surge → lab catch-up → reclassification down) is called out as the surveillance signal working as intended, with the caveat that confirmed cases continue to rise even as the cleaned-baseline suspected count drops. ""Story so far"" section unchanged.</t>
+          <t>• 2026-05-31 (scheduled run, 3-day lookback): May 28, 29 rows checked against latest sources. WHO DON605 remains the latest WHO-reconciled cumulative cutoff (27 May for DRC sus/sus_deaths; 29 May for confirmed). No revisions required on May 28 or May 29 rows. May 27 row also stable per DON605.</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-31 (scheduled run, declarations.csv): No change. CDC HAN 00530 unchanged. CDC Travel Health Notice levels unchanged (DRC remains Level 3 per verified URL https://wwwnc.cdc.gov/travel/notices/level3/ebola-democratic-republic-of-the-congo; Uganda remains Level 1 per https://wwwnc.cdc.gov/travel/notices/level1/ebola-uganda). CDC Situation Summary page at https://www.cdc.gov/ebola/situation-summary/index.html still reflects the May 16 state (8 confirmed / 248 suspected; resources block points at the DRC Level 2 travel notice URL even though the live Level 3 URL resolves correctly) — consistent with prior runs' observation that the May 25 brief refresh appears to have been rolled back. WHO PHEIC declaration of 17 May 2026 unchanged. Uganda border closure with DRC (declared 27 May 2026) unchanged in declarations.csv notes.</t>
+          <t>• 2026-05-31 (scheduled run, WHO DG Tedros Bunia press briefing): [WHO DG remarks at the press briefing on the Bundibugyo Ebola outbreak – 30 May 2026](https://www.who.int/news-room/speeches/item/who-director-general-s-remarks-at-the-press-briefing-on-the-on-the-bundibugyo-ebola-outbreak---30-may-2026) is community-focused and qualitative — no global case/death figures cited. Key passages: ""We are not here to tell people what to do. We are here to listen. Communities understand their own challenges and their own solutions."" / ""I would also ask countries that have imposed travel bans or border closures to reconsider. These measures make the response harder, and they discourage the transparency that saves lives."" / ""DRC has faced Ebola before, sixteen times, and has ended every outbreak. This is the seventeenth. That history gives me real confidence."" / ""Hand hygiene matters. Sharing accurate information matters. And safe, dignified burials matter too."" The Bunia visit will continue into 31 May.</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-31 (scheduled run, chart constants): LAST_SITREP_STABLE_DATE unchanged at 2026-05-24 (no Sitrep 03 yet; latest WHO Sitrep remains Sitrep 02 from 27 May with 24 May cutoff). OBSERVED_REVISION_RANGE unchanged at ""&lt;1-35%"" — today's run did not apply any revisions; only carry-forward appends. The hypothetical DRC MoH dip (if applied) would land at -44% / -92%, well outside the current range, but is held pending corroboration and would prompt a constant update when applied.</t>
+          <t>• 2026-05-31 (scheduled run, story.md): Refreshed ""Latest update"" section to a 31 May lead. New section opens with the WHO DG Tedros 30 May Bunia press briefing reframe (community-led response, border-closure pushback), then explains the 30 May DRC MoH ~700-case reclassification and the WHO-vs-DRC-MoH source-view divergence, then closes with the standing context (no vaccine, conflict, community resistance, MSF warning, Kenya court block). The DRC MoH cycle (suspected surge → lab catch-up → reclassification down) is called out as the surveillance signal working as intended, with the caveat that confirmed cases continue to rise even as the cleaned-baseline suspected count drops. ""Story so far"" section unchanged.</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-31 (scheduled run, sweeper health): No stale .git/*.lock or .git/objects/*/tmp_obj_* files at session start — launchd job com.webbegole.gitlock-sweep working as designed.</t>
+          <t>• 2026-05-31 (scheduled run, declarations.csv): No change. CDC HAN 00530 unchanged. CDC Travel Health Notice levels unchanged (DRC remains Level 3 per verified URL https://wwwnc.cdc.gov/travel/notices/level3/ebola-democratic-republic-of-the-congo; Uganda remains Level 1 per https://wwwnc.cdc.gov/travel/notices/level1/ebola-uganda). CDC Situation Summary page at https://www.cdc.gov/ebola/situation-summary/index.html still reflects the May 16 state (8 confirmed / 248 suspected; resources block points at the DRC Level 2 travel notice URL even though the live Level 3 URL resolves correctly) — consistent with prior runs' observation that the May 25 brief refresh appears to have been rolled back. WHO PHEIC declaration of 17 May 2026 unchanged. Uganda border closure with DRC (declared 27 May 2026) unchanged in declarations.csv notes.</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-31 (PM scheduled run, WHO/DRC Joint Statement): [Joint statement by the Government of the DRC and WHO concerning the outbreak of Ebola disease caused by the Bundibugyo virus](https://www.who.int/news/item/31-05-2026-joint-statement-by-the-government-of-the-democratic-republic-of-the-congo-and-who-concerning-the-outbreak-of-ebola-disease-caused-by-the-bundibugyo-virus) published 31 May 2026 (Bunia) closes the Tedros / Kamba / Muyaya joint mission. Statement is qualitative — no global case/death figures cited. Three substantive commitments: (1) "rapidly undertake randomized control trials on candidate vaccines and treatments"; (2) community trust at the center of the response ("Success will depend on the trust, engagement and leadership of local communities"); (3) explicit call to other governments that "borders remain open, and that entry controls do not obstruct the flow of desperately needed medical supplies and personnel" — formalizes Tedros's 30 May press-briefing pushback against border closures as a joint WHO+DRC government position. May 31 timeseries.csv row primary_source updated to cite the Joint Statement alongside the existing WHO DON605 carry-forward and BNO @BNOFeed May 31 graphic. No numerical revisions: the Joint Statement carries no figures.</t>
+          <t>• 2026-05-31 (scheduled run, chart constants): LAST_SITREP_STABLE_DATE unchanged at 2026-05-24 (no Sitrep 03 yet; latest WHO Sitrep remains Sitrep 02 from 27 May with 24 May cutoff). OBSERVED_REVISION_RANGE unchanged at ""&lt;1-35%"" — today's run did not apply any revisions; only carry-forward appends. The hypothetical DRC MoH dip (if applied) would land at -44% / -92%, well outside the current range, but is held pending corroboration and would prompt a constant update when applied.</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-31 (PM scheduled run, real-time signal): BNO website (bnonews.com/index.php/category/health/) front page shows no Ebola article (consistent with prior runs' ~3-day lag observation). BNO @BNOFeed via Web's signed-in Chrome (deviceId 5fdc215b-0b1a-4a16-9f71-01f672b11fbf): latest Daily Ebola Update graphic is the May 31 post already captured in the AM run (Cases 681 (+98) / Deaths 56 (+38) on cleaned baseline; previous post 23h ago is the May 30 cleaned-baseline graphic). No newer BNO Daily Update graphic since the prior run today. Credentialed-account search (DrTedros / WHO / WHOAFRO / AfricaCDC / MinSanteRDC / MinofHealthUG) surfaced three [WHO DG Tedros tweets ~4–5h before pass](https://x.com/DrTedros): (a) opening of a new 42-bed Ebola treatment center in Bunia — a pediatric building at the Centre Évangélique Médical converted to outbreak duty and entrusted to WHO (operational milestone, joins the rehabilitated 60-bed Bunia facility WHO announced 26 May); (b) community-leadership framing tweet from his Bunia listening sessions; (c) UNHAS Wings of the Ebola Response flight thank-you. All narrative, no count change.</t>
+          <t>• 2026-05-31 (scheduled run, sweeper health): No stale .git/*.lock or .git/objects/*/tmp_obj_* files at session start — launchd job com.webbegole.gitlock-sweep working as designed.</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-31 (PM scheduled run, 3-day lookback): May 29, 30, 31 rows checked against the latest sources. WHO DON605 remains the latest WHO-reconciled cumulative cutoff. The WHO/DRC Joint Statement (31 May) carries no figures and does not refresh the cumulative cutoff. No revisions applied. The DRC MoH cleaned-baseline running count via BNO @BNOFeed remains held as a single-source dip pending WHO Sitrep 03 / DON606 corroboration.</t>
+          <t>• 2026-05-31 (PM scheduled run, WHO/DRC Joint Statement): [Joint statement by the Government of the DRC and WHO concerning the outbreak of Ebola disease caused by the Bundibugyo virus](https://www.who.int/news/item/31-05-2026-joint-statement-by-the-government-of-the-democratic-republic-of-the-congo-and-who-concerning-the-outbreak-of-ebola-disease-caused-by-the-bundibugyo-virus) published 31 May 2026 (Bunia) closes the Tedros / Kamba / Muyaya joint mission. Statement is qualitative — no global case/death figures cited. Three substantive commitments: (1) "rapidly undertake randomized control trials on candidate vaccines and treatments"; (2) community trust at the center of the response ("Success will depend on the trust, engagement and leadership of local communities"); (3) explicit call to other governments that "borders remain open, and that entry controls do not obstruct the flow of desperately needed medical supplies and personnel" — formalizes Tedros's 30 May press-briefing pushback against border closures as a joint WHO+DRC government position. May 31 timeseries.csv row primary_source updated to cite the Joint Statement alongside the existing WHO DON605 carry-forward and BNO @BNOFeed May 31 graphic. No numerical revisions: the Joint Statement carries no figures.</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-31 (PM scheduled run, story.md): "Latest update" refreshed to lead with the WHO/DRC Joint Statement (Bunia, 31 May) — the three substantive commitments (RCTs on candidate vaccines/treatments; community trust at the center of the response; borders-open ask) plus the new 42-bed Bunia treatment-center opening. The data paragraph (WHO DON605 carry-forward; DRC MoH cleaned-baseline running count via BNO @BNOFeed) holds. The standing context paragraph (no vaccine, conflict, community resistance, MSF warning, Kenya court block) unchanged. "Story so far" unchanged.</t>
+          <t>• 2026-05-31 (PM scheduled run, real-time signal): BNO website (bnonews.com/index.php/category/health/) front page shows no Ebola article (consistent with prior runs' ~3-day lag observation). BNO @BNOFeed via Web's signed-in Chrome (deviceId 5fdc215b-0b1a-4a16-9f71-01f672b11fbf): latest Daily Ebola Update graphic is the May 31 post already captured in the AM run (Cases 681 (+98) / Deaths 56 (+38) on cleaned baseline; previous post 23h ago is the May 30 cleaned-baseline graphic). No newer BNO Daily Update graphic since the prior run today. Credentialed-account search (DrTedros / WHO / WHOAFRO / AfricaCDC / MinSanteRDC / MinofHealthUG) surfaced three [WHO DG Tedros tweets ~4–5h before pass](https://x.com/DrTedros): (a) opening of a new 42-bed Ebola treatment center in Bunia — a pediatric building at the Centre Évangélique Médical converted to outbreak duty and entrusted to WHO (operational milestone, joins the rehabilitated 60-bed Bunia facility WHO announced 26 May); (b) community-leadership framing tweet from his Bunia listening sessions; (c) UNHAS Wings of the Ebola Response flight thank-you. All narrative, no count change.</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-31 (PM scheduled run, declarations.csv): No change. CDC HAN 00530 unchanged. CDC Travel Health Notice levels unchanged (DRC remains Level 3; Uganda remains Level 1) per verified URLs. CDC Situation Summary page still dated 16 May 2026 (cdc:last_updated 2026-05-16T20:42:17Z) with stale figures and Resources block pointing at the DRC Level 2 travel notice — consistent with prior runs' observation that the brief 25 May refresh was rolled back. WHO PHEIC declaration of 17 May 2026 unchanged. Uganda border closure with DRC (declared 27 May 2026) unchanged. The WHO/DRC Joint Statement is a joint communication, not a declaration change.</t>
+          <t>• 2026-05-31 (PM scheduled run, 3-day lookback): May 29, 30, 31 rows checked against the latest sources. WHO DON605 remains the latest WHO-reconciled cumulative cutoff. The WHO/DRC Joint Statement (31 May) carries no figures and does not refresh the cumulative cutoff. No revisions applied. The DRC MoH cleaned-baseline running count via BNO @BNOFeed remains held as a single-source dip pending WHO Sitrep 03 / DON606 corroboration.</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-31 (PM scheduled run, chart constants): LAST_SITREP_STABLE_DATE unchanged at 2026-05-24 (no Sitrep 03 yet). OBSERVED_REVISION_RANGE unchanged at "&lt;1-35%" — no revisions applied today.</t>
+          <t>• 2026-05-31 (PM scheduled run, story.md): "Latest update" refreshed to lead with the WHO/DRC Joint Statement (Bunia, 31 May) — the three substantive commitments (RCTs on candidate vaccines/treatments; community trust at the center of the response; borders-open ask) plus the new 42-bed Bunia treatment-center opening. The data paragraph (WHO DON605 carry-forward; DRC MoH cleaned-baseline running count via BNO @BNOFeed) holds. The standing context paragraph (no vaccine, conflict, community resistance, MSF warning, Kenya court block) unchanged. "Story so far" unchanged.</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-31 (PM scheduled run, sweeper health): No stale .git/*.lock or .git/objects/*/tmp_obj_* files at session start — launchd job com.webbegole.gitlock-sweep working as designed.</t>
+          <t>• 2026-05-31 (PM scheduled run, declarations.csv): No change. CDC HAN 00530 unchanged. CDC Travel Health Notice levels unchanged (DRC remains Level 3; Uganda remains Level 1) per verified URLs. CDC Situation Summary page still dated 16 May 2026 (cdc:last_updated 2026-05-16T20:42:17Z) with stale figures and Resources block pointing at the DRC Level 2 travel notice — consistent with prior runs' observation that the brief 25 May refresh was rolled back. WHO PHEIC declaration of 17 May 2026 unchanged. Uganda border closure with DRC (declared 27 May 2026) unchanged. The WHO/DRC Joint Statement is a joint communication, not a declaration change.</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-31 (PM2 run, methodology refinement per Web): Added "MoH methodology-change carve-out" to the no-dip rule in METHODOLOGY.md. Rationale: the no-dip rule as originally written required two high-value sources to apply a downward revision. The DRC MoH 30 May ~700-case cleanup (lab capacity ramp-up; suspected cases that subsequently tested negative for Ebola are removed) is a formally-announced definitional reclassification by the official surveillance authority. A definitional cleanup announced by the surveillance source IS the reclassification, by definition; waiting for WHO Sitrep reconciliation in that case is a delay, not a correction. The carve-out waives the two-source threshold when the dip is a MoH (DRC or Uganda) formal announcement and the wire is faithfully carrying it. The standard no-dip rule still applies to wire-only paraphrases of unreconciled recounts. Operationally: exemptions are recorded in `src/validate.py`'s NO_DIP_EXEMPTIONS_TIMESERIES (date → columns) and NO_DIP_EXEMPTIONS_BREAKDOWN ((date, country) → columns) so the no-dip validator skips the named columns on the named row(s). Every exemption gets a NOTES bullet citing the MoH announcement and the figures applied. This was the prototypical case; future MoH cleanups will follow the same pattern.</t>
+          <t>• 2026-05-31 (PM scheduled run, chart constants): LAST_SITREP_STABLE_DATE unchanged at 2026-05-24 (no Sitrep 03 yet). OBSERVED_REVISION_RANGE unchanged at "&lt;1-35%" — no revisions applied today.</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-31 (PM2 run, carve-out applied to May 30 row): timeseries.csv May 30 row revised per DRC MoH cleaned baseline via BNO @BNOFeed May 30 graphic: suspected_global 906→349 (-61.48%), confirmed_global 134→234 (+74.63%), total_global 1040→583 (-43.94%), suspected_deaths_global 223→0 (-100%). Sus/conf split: DRC confirmed accepts DRC MoH's running 225 (BNO @BNOFeed May 29 +100 lab catch-up); DRC suspected = 574 - 225 = 349. DRC sus_deaths column zeroed by DRC MoH in the same cleanup (the 17 deaths on BNO's May 30 graphic = pre-cleanup conf_deaths only). DRC conf_deaths = 17 unchanged. Uganda 9 / 1 unchanged. NO_DIP_EXEMPTIONS_TIMESERIES entry: "2026-05-30" → {suspected_global, total_global, suspected_deaths_global}. The confirmed_global column is NOT exempt because the revision is upward (134 → 234); the dip exemption applies only to the columns going downward. NO_DIP_EXEMPTIONS_BREAKDOWN entry: ("2026-05-30", "DRC") → {suspected, suspected_deaths}.</t>
+          <t>• 2026-05-31 (PM scheduled run, sweeper health): No stale .git/*.lock or .git/objects/*/tmp_obj_* files at session start — launchd job com.webbegole.gitlock-sweep working as designed.</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-31 (PM2 run, carve-out propagated to May 31 row): timeseries.csv May 31 row revised: suspected_global 906→447 (-50.66%), confirmed_global 134→234 (+74.63%), total_global 1040→681 (-34.52%), suspected_deaths_global 223→0 (-100%). Split: DRC conf carries the May 30 DRC MoH running 225 forward (no fresh May 31 lab figure published); DRC sus = 672 - 225 = 447. DRC sus_deaths stays at 0 (column zeroed May 30); +38 deaths in BNO's May 31 graphic attributed to conf_deaths as DRC MoH continues to lab-confirm previously-probable deaths, so DRC conf_deaths = 17 + 38 = 55. No exemption needed for the May 31 row in the validator: cumulative globals against the May 30 baseline are non-decreasing (sus 349→447, conf 234→234, total 583→681, sus_deaths 0→0). Per-country DRC also non-decreasing against May 30 baseline (sus 349→447, conf 225→225, sus_deaths 0→0, conf_deaths 17→55).</t>
+          <t>• 2026-05-31 (PM2 run, methodology refinement per Web): Added "MoH methodology-change carve-out" to the no-dip rule in METHODOLOGY.md. Rationale: the no-dip rule as originally written required two high-value sources to apply a downward revision. The DRC MoH 30 May ~700-case cleanup (lab capacity ramp-up; suspected cases that subsequently tested negative for Ebola are removed) is a formally-announced definitional reclassification by the official surveillance authority. A definitional cleanup announced by the surveillance source IS the reclassification, by definition; waiting for WHO Sitrep reconciliation in that case is a delay, not a correction. The carve-out waives the two-source threshold when the dip is a MoH (DRC or Uganda) formal announcement and the wire is faithfully carrying it. The standard no-dip rule still applies to wire-only paraphrases of unreconciled recounts. Operationally: exemptions are recorded in `src/validate.py`'s NO_DIP_EXEMPTIONS_TIMESERIES (date → columns) and NO_DIP_EXEMPTIONS_BREAKDOWN ((date, country) → columns) so the no-dip validator skips the named columns on the named row(s). Every exemption gets a NOTES bullet citing the MoH announcement and the figures applied. This was the prototypical case; future MoH cleanups will follow the same pattern.</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-31 (PM2 run, chart constants): Split OBSERVED_REVISION_RANGE into OBSERVED_UPWARD_REVISION_RANGE (still "&lt;1-35%", reflecting WHO Sitrep / DON reconciliation history) and OBSERVED_DOWNWARD_REVISION_RANGE ("up to 100%", reflecting the May 30 MoH carve-out: sus -61.48%, sus_deaths -100%). Chart-footnote string updated to surface both directions: "Bars after {LAST_SITREP_STABLE_DATE} are provisional; revisions have run +{up} (Sitrep reconciliation) and {down} downward (MoH definitional cleanups)." Generate_charts.py constants comment updated to document both ranges and the mechanisms behind each.</t>
+          <t>• 2026-05-31 (PM2 run, carve-out applied to May 30 row): timeseries.csv May 30 row revised per DRC MoH cleaned baseline via BNO @BNOFeed May 30 graphic: suspected_global 906→349 (-61.48%), confirmed_global 134→234 (+74.63%), total_global 1040→583 (-43.94%), suspected_deaths_global 223→0 (-100%). Sus/conf split: DRC confirmed accepts DRC MoH's running 225 (BNO @BNOFeed May 29 +100 lab catch-up); DRC suspected = 574 - 225 = 349. DRC sus_deaths column zeroed by DRC MoH in the same cleanup (the 17 deaths on BNO's May 30 graphic = pre-cleanup conf_deaths only). DRC conf_deaths = 17 unchanged. Uganda 9 / 1 unchanged. NO_DIP_EXEMPTIONS_TIMESERIES entry: "2026-05-30" → {suspected_global, total_global, suspected_deaths_global}. The confirmed_global column is NOT exempt because the revision is upward (134 → 234); the dip exemption applies only to the columns going downward. NO_DIP_EXEMPTIONS_BREAKDOWN entry: ("2026-05-30", "DRC") → {suspected, suspected_deaths}.</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-31 (PM2 run, validator): Added NO_DIP_EXEMPTIONS_TIMESERIES and NO_DIP_EXEMPTIONS_BREAKDOWN dicts at the top of src/validate.py with named exemptions per the carve-out. The cumulative non-decreasing checks now skip exempt (date, column) and (date, country, column) tuples. Validator passes clean after revisions.</t>
+          <t>• 2026-05-31 (PM2 run, carve-out propagated to May 31 row): timeseries.csv May 31 row revised: suspected_global 906→447 (-50.66%), confirmed_global 134→234 (+74.63%), total_global 1040→681 (-34.52%), suspected_deaths_global 223→0 (-100%). Split: DRC conf carries the May 30 DRC MoH running 225 forward (no fresh May 31 lab figure published); DRC sus = 672 - 225 = 447. DRC sus_deaths stays at 0 (column zeroed May 30); +38 deaths in BNO's May 31 graphic attributed to conf_deaths as DRC MoH continues to lab-confirm previously-probable deaths, so DRC conf_deaths = 17 + 38 = 55. No exemption needed for the May 31 row in the validator: cumulative globals against the May 30 baseline are non-decreasing (sus 349→447, conf 234→234, total 583→681, sus_deaths 0→0). Per-country DRC also non-decreasing against May 30 baseline (sus 349→447, conf 225→225, sus_deaths 0→0, conf_deaths 17→55).</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-31 (PM2 run, story.md): "Latest update" rewritten to lead with the DRC MoH cleanup and the new lower figures, explicitly explaining that the visual drop on the chart is the surveillance signal working as intended (suspected-cases bar deliberately wide → lab capacity catches up → negatives get removed → tighter denominator). The WHO/DRC Joint Statement section retained as the second paragraph. "Story so far" unchanged.</t>
+          <t>• 2026-05-31 (PM2 run, chart constants): Split OBSERVED_REVISION_RANGE into OBSERVED_UPWARD_REVISION_RANGE (still "&lt;1-35%", reflecting WHO Sitrep / DON reconciliation history) and OBSERVED_DOWNWARD_REVISION_RANGE ("up to 100%", reflecting the May 30 MoH carve-out: sus -61.48%, sus_deaths -100%). Chart-footnote string updated to surface both directions: "Bars after {LAST_SITREP_STABLE_DATE} are provisional; revisions have run +{up} (Sitrep reconciliation) and {down} downward (MoH definitional cleanups)." Generate_charts.py constants comment updated to document both ranges and the mechanisms behind each.</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-31 (PM2 run, declarations.csv): No change. CDC HAN, CDC Travel Health Notice levels, WHO PHEIC, Uganda border closure all unchanged. The carve-out is a tracker methodology refinement, not a declaration change.</t>
+          <t>• 2026-05-31 (PM2 run, validator): Added NO_DIP_EXEMPTIONS_TIMESERIES and NO_DIP_EXEMPTIONS_BREAKDOWN dicts at the top of src/validate.py with named exemptions per the carve-out. The cumulative non-decreasing checks now skip exempt (date, column) and (date, country, column) tuples. Validator passes clean after revisions.</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-31 (PM3 run, schema change per Web): Added `confirmed_deaths_global` column to data/timeseries.csv schema, between `suspected_deaths_global` and `primary_source`. Rationale: after the DRC MoH cleanup zeroed the suspected-deaths column on 2026-05-30, "suspected deaths" stopped being a useful headline metric. Real deaths are still accumulating; they're just on the confirmed side now (DRC ran +38 lab confirmations on 31 May for a DRC conf_deaths total of 55). The deaths chart was showing 0 new deaths in the 7-day rolling window on May 31, which was technically true for the suspected column but materially misleading. Schema is now: report_date, suspected_global, confirmed_global, total_global, suspected_deaths_global, confirmed_deaths_global, primary_source, source_timestamp. Backfilled historical values from country_breakdown.csv DRC + Uganda sums: May 15-23 = 1 (Uganda only); May 24-26 = 11 (DRC 10 + Uganda 1); May 27-30 = 18 (DRC 17 + Uganda 1); May 31 = 56 (DRC 55 + Uganda 1). Cumulative monotonically non-decreasing throughout; no NO_DIP_EXEMPTIONS entry needed for the new column. src/validate.py updated to include confirmed_deaths_global in EXPECTED_TIMESERIES_COLS and CUMULATIVE_TIMESERIES_COLS, plus the parse loop. src/build_xlsx.py updated to add the new column to the main sheet header and the Charts sheet's daily-delta + rolling-sum derivation. Validator passes clean.</t>
+          <t>• 2026-05-31 (PM2 run, story.md): "Latest update" rewritten to lead with the DRC MoH cleanup and the new lower figures, explicitly explaining that the visual drop on the chart is the surveillance signal working as intended (suspected-cases bar deliberately wide → lab capacity catches up → negatives get removed → tighter denominator). The WHO/DRC Joint Statement section retained as the second paragraph. "Story so far" unchanged.</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-31 (PM3 run, deaths chart restructure): Reworked render_deaths_chart in src/generate_charts.py to mirror render_cases_chart structurally. Bars now stacked: confirmed deaths (COLOR_CONFIRMED, bottom) + suspected deaths (COLOR_SUSPECTED, top); hatched on provisional dates. Cumulative-line overlay now carries two lines: total deaths (sus + conf, COLOR_CUMULATIVE bronze) and confirmed-only deaths (COLOR_CUMULATIVE_CONF deep red), matching the cases chart's two-line treatment. The gap between the lines is the share of the running death count still in clinical-suspicion-only status. Chart suptitle changed from "7-day rolling sum of suspected deaths" to "7-day rolling sum of new deaths"; axis label and inline title updated to match. Legend rebuilt: confirmed deaths Patch + suspected deaths Patch + provisional swatch + cumulative-total Line2D + cumulative-confirmed Line2D. The MoH-baseline-reset marker (vertical dashed line + "MoH baseline reset" label) carries over from the prior commit.</t>
+          <t>• 2026-05-31 (PM2 run, declarations.csv): No change. CDC HAN, CDC Travel Health Notice levels, WHO PHEIC, Uganda border closure all unchanged. The carve-out is a tracker methodology refinement, not a declaration change.</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-31 (PM3 run, captions): Refreshed YYYY-MM-DD_caption-x.txt and YYYY-MM-DD_caption-linkedin.txt in the project folder root to reflect the cleaned-baseline cumulative figures (447 sus / 234 conf / 681 total cases; 0 sus deaths / 56 conf deaths) and the 7-day rolling sums under the new schema (+120 cases, +45 deaths). X caption at 251 chars (under 270 limit).</t>
+          <t>• 2026-05-31 (PM3 run, schema change per Web): Added `confirmed_deaths_global` column to data/timeseries.csv schema, between `suspected_deaths_global` and `primary_source`. Rationale: after the DRC MoH cleanup zeroed the suspected-deaths column on 2026-05-30, "suspected deaths" stopped being a useful headline metric. Real deaths are still accumulating; they're just on the confirmed side now (DRC ran +38 lab confirmations on 31 May for a DRC conf_deaths total of 55). The deaths chart was showing 0 new deaths in the 7-day rolling window on May 31, which was technically true for the suspected column but materially misleading. Schema is now: report_date, suspected_global, confirmed_global, total_global, suspected_deaths_global, confirmed_deaths_global, primary_source, source_timestamp. Backfilled historical values from country_breakdown.csv DRC + Uganda sums: May 15-23 = 1 (Uganda only); May 24-26 = 11 (DRC 10 + Uganda 1); May 27-30 = 18 (DRC 17 + Uganda 1); May 31 = 56 (DRC 55 + Uganda 1). Cumulative monotonically non-decreasing throughout; no NO_DIP_EXEMPTIONS entry needed for the new column. src/validate.py updated to include confirmed_deaths_global in EXPECTED_TIMESERIES_COLS and CUMULATIVE_TIMESERIES_COLS, plus the parse loop. src/build_xlsx.py updated to add the new column to the main sheet header and the Charts sheet's daily-delta + rolling-sum derivation. Validator passes clean.</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-31 (PM4 run, declarations.csv refresh — surfaced by Web): Audit of declarations.csv against live CDC/WHO sources surfaced several missed events between 2026-05-18 and 2026-05-31. Updates applied: (1) **Uganda CDC Travel Health Notice escalated from Level 1 to Level 2 on 2026-05-27** — explicitly confirmed by the [US Embassy Kampala 28 May health alert](https://ug.usembassy.gov/health-alert-u-s-embassy-kampala-uganda-may-28-2026/) ("On May 27, the U.S. Centers for Disease Control and Prevention (CDC) increased its Travel Health Notice for Ebola Bundibugyo Virus Disease from a Level 1 to Level 2"). cdc_travel_notice_level changed from "Level 1 (Practice Usual Precautions)" to "Level 2 (Practice Enhanced Precautions)"; cdc_travel_notice_url changed from /level1/ebola-uganda to /level2/ebola-uganda. This was missed in the 2026-05-27 PM run, the 2026-05-28 scheduled run, the 2026-05-30 scheduled run, and the 2026-05-31 AM/PM/PM2/PM3 runs — six consecutive runs that recorded "declarations.csv: no change" without re-verifying the live travel-notice index. Procedural lesson: the daily run's declarations check needs to actually fetch the per-country travel-notice URL and verify the level, not just confirm the URL still resolves. The /level1/ebola-uganda URL still resolves but now serves stale content from a prior SVD outbreak. (2) **DRC CDC Travel Notice remains at Level 3** — re-verified via search-result page title ("Ebola Bundibugyo Virus Disease in the Democratic Republic of the Congo - Level 3 - Reconsider Nonessential Travel") and the US Embassy Kampala alert linking the /level3/ DRC URL. No change to DRC's cdc_travel_notice_level / URL. (3) **Africa CDC PHECS declaration on 2026-05-18** (Public Health Emergency of Continental Security) — added to both DRC and Uganda notes fields, sourced to the [Africa CDC statement on US travel restrictions](https://africacdc.org/news-item/u-s-travel-restrictions-related-to-the-bundibugyo-ebola-outbreak/). Schema doesn't have an Africa CDC column; the PHECS is documented in notes for now. (4) **US State Department Travel Advisory at Level 4 (Do Not Travel)** for both DRC and Uganda — distinct from the CDC Travel Health Notice (which is at Level 3 / Level 2 respectively); the State Department advisory is a separate US government advisory at the country level. Added to notes for both rows. (5) **US entry restrictions** on non-US passport holders who travelled to DRC, Uganda, or South Sudan in the previous 21 days, in effect from 2026-05-22 and extended to green-card holders the same week — added to notes for both rows. (6) **CDC Title 42 Order** for arrivals from affected countries — added to notes for both rows with the [CDC media release URL](https://www.cdc.gov/media/releases/2026/statement-update-on-title-42-order.html). (7) **US arrivals from affected countries funneled through IAD (from 2026-05-21), ATL (from 2026-05-22), IAH Houston (from 2026-05-26)** for enhanced screening — added to DRC notes. (8) **WHO/DRC Joint Statement of 2026-05-31** linked in DRC notes for the explicit "borders remain open" ask. (9) **Cases now span 13 health zones** (up from 12 noted in original DRC entry) — updated DRC notes. (10) **Sud-Kivu first lab-confirmed case 2026-05-25** — added to DRC notes (this was logged in the timeseries.csv May 25 primary_source but not surfaced in declarations.csv). Validator passes; no schema change. Note: declarations.csv's current schema does not have columns for US State Department Travel Advisory or Africa CDC PHECS. If these become recurring fields worth tracking with structured cells, the schema should be expanded; for now the notes field carries them.</t>
+          <t>• 2026-05-31 (PM3 run, deaths chart restructure): Reworked render_deaths_chart in src/generate_charts.py to mirror render_cases_chart structurally. Bars now stacked: confirmed deaths (COLOR_CONFIRMED, bottom) + suspected deaths (COLOR_SUSPECTED, top); hatched on provisional dates. Cumulative-line overlay now carries two lines: total deaths (sus + conf, COLOR_CUMULATIVE bronze) and confirmed-only deaths (COLOR_CUMULATIVE_CONF deep red), matching the cases chart's two-line treatment. The gap between the lines is the share of the running death count still in clinical-suspicion-only status. Chart suptitle changed from "7-day rolling sum of suspected deaths" to "7-day rolling sum of new deaths"; axis label and inline title updated to match. Legend rebuilt: confirmed deaths Patch + suspected deaths Patch + provisional swatch + cumulative-total Line2D + cumulative-confirmed Line2D. The MoH-baseline-reset marker (vertical dashed line + "MoH baseline reset" label) carries over from the prior commit.</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-31 (PM6 run, index.html headline cards): Per Web, removed the "Suspected deaths" headline stat card from the top of the page. Rationale: DRC MoH zeroed the suspected-deaths column in the 2026-05-30 cleanup and the running figure has stayed at 0 since; surfacing it as a headline number gives a misleading "0 deaths" impression. The recent reporting table on the same page still keeps the Susp. Deaths column so the historical record (and the cleanup event itself) remains visible there. The deaths chart also still shows the suspected layer in the stacked bars and the cumulative-total-deaths line. Only the top-of-page headline card was removed. Render() fields array updated to drop the slug "deaths" / column "suspected_deaths_global"; the "conf-deaths" card / "confirmed_deaths_global" column carries the deaths headline now.</t>
+          <t>• 2026-05-31 (PM3 run, captions): Refreshed YYYY-MM-DD_caption-x.txt and YYYY-MM-DD_caption-linkedin.txt in the project folder root to reflect the cleaned-baseline cumulative figures (447 sus / 234 conf / 681 total cases; 0 sus deaths / 56 conf deaths) and the 7-day rolling sums under the new schema (+120 cases, +45 deaths). X caption at 251 chars (under 270 limit).</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" s="9" t="inlineStr">
         <is>
-          <t>• 2026-05-31 (PM5 run, METHODOLOGY.md country-add rule + index.html confirmed-deaths column — surfaced by Web): Two structural updates. (a) Added "Adding a country to declarations.csv" section to METHODOLOGY.md with explicit criteria for when a new country row gets added: own confirmed/suspected cases, OR own country-specific CDC Travel Health Notice, OR own country-specific CDC HAN entry (or multi-country HAN that names the country), OR own WHO country-specific declaration, OR non-US national health authority outbreak-specific advisory with stable primary-source URL. Explicitly clarified that a country appearing in another country's advisory (e.g., South Sudan in the US entry restrictions) does NOT warrant its own row; cross-country effects are captured in the affected countries' notes fields. Also documented the verification protocol on each daily run: a "declarations.csv: no change" report must mean the agent actually fetched the per-country CDC Travel Notice URL and verified the level on the page, plus scanned the CDC Travel Notices index. URL-resolves != level-unchanged (the Uganda /level1/ URL kept serving stale Sudan-virus content after CDC moved BVD to /level2/). Audit of currently-named-in-other-countries' advisories: South Sudan (in US entry restrictions and US State Dept Do Not Travel) does not have its own CDC HAN, CDC Travel Health Notice, or WHO country-specific advisory for this outbreak as of 2026-05-31; no row added. Other countries imposing their own measures (Canada, Bahamas) have their own national-level travel advisories but those are not in scope under the current schema (CDC/WHO only); if Web wants to track non-US national advisories, schema extension is warranted. (b) Updated index.html to surface the new confirmed_deaths_global column: added "Confirmed deaths" headline stat card (5th card; uses the "confirmed" red accent), added "Conf. Deaths" column to the Recent reporting table (between Susp. Deaths and Source), bumped table colspans from 6 to 7 (including the renderError fallback), wired up the new column in the render() function (slug "conf-deaths" → column "confirmed_deaths_global"). Also updated the deaths chart alt text to describe the new stacked structure. The public-facing index.html now reflects the same schema the charts and CSVs use.</t>
+          <t>• 2026-05-31 (PM4 run, declarations.csv refresh — surfaced by Web): Audit of declarations.csv against live CDC/WHO sources surfaced several missed events between 2026-05-18 and 2026-05-31. Updates applied: (1) **Uganda CDC Travel Health Notice escalated from Level 1 to Level 2 on 2026-05-27** — explicitly confirmed by the [US Embassy Kampala 28 May health alert](https://ug.usembassy.gov/health-alert-u-s-embassy-kampala-uganda-may-28-2026/) ("On May 27, the U.S. Centers for Disease Control and Prevention (CDC) increased its Travel Health Notice for Ebola Bundibugyo Virus Disease from a Level 1 to Level 2"). cdc_travel_notice_level changed from "Level 1 (Practice Usual Precautions)" to "Level 2 (Practice Enhanced Precautions)"; cdc_travel_notice_url changed from /level1/ebola-uganda to /level2/ebola-uganda. This was missed in the 2026-05-27 PM run, the 2026-05-28 scheduled run, the 2026-05-30 scheduled run, and the 2026-05-31 AM/PM/PM2/PM3 runs — six consecutive runs that recorded "declarations.csv: no change" without re-verifying the live travel-notice index. Procedural lesson: the daily run's declarations check needs to actually fetch the per-country travel-notice URL and verify the level, not just confirm the URL still resolves. The /level1/ebola-uganda URL still resolves but now serves stale content from a prior SVD outbreak. (2) **DRC CDC Travel Notice remains at Level 3** — re-verified via search-result page title ("Ebola Bundibugyo Virus Disease in the Democratic Republic of the Congo - Level 3 - Reconsider Nonessential Travel") and the US Embassy Kampala alert linking the /level3/ DRC URL. No change to DRC's cdc_travel_notice_level / URL. (3) **Africa CDC PHECS declaration on 2026-05-18** (Public Health Emergency of Continental Security) — added to both DRC and Uganda notes fields, sourced to the [Africa CDC statement on US travel restrictions](https://africacdc.org/news-item/u-s-travel-restrictions-related-to-the-bundibugyo-ebola-outbreak/). Schema doesn't have an Africa CDC column; the PHECS is documented in notes for now. (4) **US State Department Travel Advisory at Level 4 (Do Not Travel)** for both DRC and Uganda — distinct from the CDC Travel Health Notice (which is at Level 3 / Level 2 respectively); the State Department advisory is a separate US government advisory at the country level. Added to notes for both rows. (5) **US entry restrictions** on non-US passport holders who travelled to DRC, Uganda, or South Sudan in the previous 21 days, in effect from 2026-05-22 and extended to green-card holders the same week — added to notes for both rows. (6) **CDC Title 42 Order** for arrivals from affected countries — added to notes for both rows with the [CDC media release URL](https://www.cdc.gov/media/releases/2026/statement-update-on-title-42-order.html). (7) **US arrivals from affected countries funneled through IAD (from 2026-05-21), ATL (from 2026-05-22), IAH Houston (from 2026-05-26)** for enhanced screening — added to DRC notes. (8) **WHO/DRC Joint Statement of 2026-05-31** linked in DRC notes for the explicit "borders remain open" ask. (9) **Cases now span 13 health zones** (up from 12 noted in original DRC entry) — updated DRC notes. (10) **Sud-Kivu first lab-confirmed case 2026-05-25** — added to DRC notes (this was logged in the timeseries.csv May 25 primary_source but not surfaced in declarations.csv). Validator passes; no schema change. Note: declarations.csv's current schema does not have columns for US State Department Travel Advisory or Africa CDC PHECS. If these become recurring fields worth tracking with structured cells, the schema should be expanded; for now the notes field carries them.</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-01 (scheduled run, BNO real-time pass): Web's signed-in Chrome reachable via list_connected_browsers → select_browser (deviceId 5fdc215b-0b1a-4a16-9f71-01f672b11fbf). BNO @BNOFeed Daily Ebola Update June 1, 2026 graphic (posted ~48m before pass, status 2061573338569351279, https://x.com/BNOFeed/status/2061573338569351279) reports (sourced to MoH DR Congo + MoH Uganda + WHO; 17 days since first case): DR Congo 343 conf (+80) / 116 sus (-293) / 48 deaths (+6); Uganda 9 conf (-) / 1 death (-); TOTAL 352 conf (+80) / 49 deaths (+6). This is the FIRST BNO graphic to split DRC into sus/conf on the cleaned baseline; prior graphics (May 30, May 31) showed cases as combined. BNO follow-up tweet documents the methodology shift: "Because the number of suspected cases is constantly changing, and not always available, our updates will now focus on confirmed cases. The number of suspected cases is still shown in the graphic." This reflects continued DRC MoH lab catch-up; cases moving from suspected → confirmed as labs catch up, and test-negative suspected cases being removed. BNO website (bnonews.com/index.php/category/health/) front page does not yet show a June 1 Ebola article — website lag continues at ~3 days behind @BNOFeed.</t>
+          <t>• 2026-05-31 (PM6 run, index.html headline cards): Per Web, removed the "Suspected deaths" headline stat card from the top of the page. Rationale: DRC MoH zeroed the suspected-deaths column in the 2026-05-30 cleanup and the running figure has stayed at 0 since; surfacing it as a headline number gives a misleading "0 deaths" impression. The recent reporting table on the same page still keeps the Susp. Deaths column so the historical record (and the cleanup event itself) remains visible there. The deaths chart also still shows the suspected layer in the stacked bars and the cumulative-total-deaths line. Only the top-of-page headline card was removed. Render() fields array updated to drop the slug "deaths" / column "suspected_deaths_global"; the "conf-deaths" card / "confirmed_deaths_global" column carries the deaths headline now.</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-01 (scheduled run, MoH carve-out continued application): Per METHODOLOGY.md MoH methodology-change carve-out, the continued DRC MoH lab-capacity ramp-up cleanup applies to the June 1 row. DRC suspected drops from 447 (May 31 inferred) to 116, total from 681 to 468. NO_DIP_EXEMPTIONS_TIMESERIES entry added: "2026-06-01" → {suspected_global, total_global}. NO_DIP_EXEMPTIONS_BREAKDOWN entry added: ("2026-06-01", "DRC") → {suspected}. Confirmed cases column is upward (+118 globally; +118 DRC), no exemption needed. Suspected_deaths_global stays at 0 (column zeroed May 30, unchanged today). Conf_deaths_global goes 43 (revised May 31) → 49 (June 1), upward.</t>
+          <t>• 2026-05-31 (PM5 run, METHODOLOGY.md country-add rule + index.html confirmed-deaths column — surfaced by Web): Two structural updates. (a) Added "Adding a country to declarations.csv" section to METHODOLOGY.md with explicit criteria for when a new country row gets added: own confirmed/suspected cases, OR own country-specific CDC Travel Health Notice, OR own country-specific CDC HAN entry (or multi-country HAN that names the country), OR own WHO country-specific declaration, OR non-US national health authority outbreak-specific advisory with stable primary-source URL. Explicitly clarified that a country appearing in another country's advisory (e.g., South Sudan in the US entry restrictions) does NOT warrant its own row; cross-country effects are captured in the affected countries' notes fields. Also documented the verification protocol on each daily run: a "declarations.csv: no change" report must mean the agent actually fetched the per-country CDC Travel Notice URL and verified the level on the page, plus scanned the CDC Travel Notices index. URL-resolves != level-unchanged (the Uganda /level1/ URL kept serving stale Sudan-virus content after CDC moved BVD to /level2/). Audit of currently-named-in-other-countries' advisories: South Sudan (in US entry restrictions and US State Dept Do Not Travel) does not have its own CDC HAN, CDC Travel Health Notice, or WHO country-specific advisory for this outbreak as of 2026-05-31; no row added. Other countries imposing their own measures (Canada, Bahamas) have their own national-level travel advisories but those are not in scope under the current schema (CDC/WHO only); if Web wants to track non-US national advisories, schema extension is warranted. (b) Updated index.html to surface the new confirmed_deaths_global column: added "Confirmed deaths" headline stat card (5th card; uses the "confirmed" red accent), added "Conf. Deaths" column to the Recent reporting table (between Susp. Deaths and Source), bumped table colspans from 6 to 7 (including the renderError fallback), wired up the new column in the render() function (slug "conf-deaths" → column "confirmed_deaths_global"). Also updated the deaths chart alt text to describe the new stacked structure. The public-facing index.html now reflects the same schema the charts and CSVs use.</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-01 (scheduled run, May 31 conf_deaths correction): Same-row correction applied per BNO June 1 graphic's "+6" delta implying yesterday's BNO DRC conf_deaths = 42, corroborated by DRC MoH 31 May situation report (per multiple June 1 wire summaries: "DRC Ministry of Health published updated figures reporting a total of 282 confirmed cases, including 42 confirmed related deaths and 220 suspected cases that are under investigation"). May 31 timeseries.csv confirmed_deaths_global revised 56 → 43; country_breakdown.csv DRC May 31 confirmed_deaths revised 55 → 42. The prior 55 was an inference (+38 attributed to conf_deaths from BNO May 31 graphic's "55 deaths" total, interpreted as fully confirmed post-May-30 cleanup); DRC MoH's formal 31 May figure is 42 confirmed deaths. Geographic split per DRC MoH 31 May situation report: Ituri 264 conf, Nord-Kivu 15 conf, Sud-Kivu 3 conf (total DRC = 282). This is a same-row correction under the 3-day lookback policy, NOT a no-dip dip — revised May 31 conf_deaths_global (43) is still ≥ May 30 (18) so cumulative non-decreasing is maintained.</t>
+          <t>• 2026-06-01 (scheduled run, BNO real-time pass): Web's signed-in Chrome reachable via list_connected_browsers → select_browser (deviceId 5fdc215b-0b1a-4a16-9f71-01f672b11fbf). BNO @BNOFeed Daily Ebola Update June 1, 2026 graphic (posted ~48m before pass, status 2061573338569351279, https://x.com/BNOFeed/status/2061573338569351279) reports (sourced to MoH DR Congo + MoH Uganda + WHO; 17 days since first case): DR Congo 343 conf (+80) / 116 sus (-293) / 48 deaths (+6); Uganda 9 conf (-) / 1 death (-); TOTAL 352 conf (+80) / 49 deaths (+6). This is the FIRST BNO graphic to split DRC into sus/conf on the cleaned baseline; prior graphics (May 30, May 31) showed cases as combined. BNO follow-up tweet documents the methodology shift: "Because the number of suspected cases is constantly changing, and not always available, our updates will now focus on confirmed cases. The number of suspected cases is still shown in the graphic." This reflects continued DRC MoH lab catch-up; cases moving from suspected → confirmed as labs catch up, and test-negative suspected cases being removed. BNO website (bnonews.com/index.php/category/health/) front page does not yet show a June 1 Ebola article — website lag continues at ~3 days behind @BNOFeed.</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-01 (scheduled run, WHO Sunday update — source-view divergence flag): [UN News June 1 2026 "DR Congo Ebola outbreak: Nurses discharged after full recovery"](https://news.un.org/en/story/2026/06/1167613) cites a WHO update on Sunday (May 31) reporting "210 confirmed cases of infection reported in the country [DRC], with 17 confirmed deaths. Nearly 350 suspected cases are under investigation and 16 health workers have contracted Ebola in DRC during this latest outbreak." WHO's 210/17 figures are HIGHER than WHO DON605's 125/17 (29 May cutoff) but LOWER than DRC MoH's 282/42 (31 May situation report) and BNO's June 1 graphic (352 confirmed globally including 343 DRC + 9 Uganda; 49 confirmed deaths including 48 DRC + 1 Uganda). WHO is partially reconciling the DRC MoH lab catch-up but hasn't caught up fully. Per source-preference order (WHO &gt; DRC MoH &gt; BNO), if WHO had a publication-grade 210 figure, we'd use it; but the 210 is reported via UN News with no clean WHO publication URL (DON606 not yet published; Sitrep 03 expected 2 Jun). For this run we use the BNO @BNOFeed June 1 graphic as the primary source for the June 1 row (BNO graphic explicitly attributes to MoH DR Congo + MoH Uganda + WHO and is dated June 1 — fresher than the WHO Sunday update). WHO Sitrep 03 will reconcile.</t>
+          <t>• 2026-06-01 (scheduled run, MoH carve-out continued application): Per METHODOLOGY.md MoH methodology-change carve-out, the continued DRC MoH lab-capacity ramp-up cleanup applies to the June 1 row. DRC suspected drops from 447 (May 31 inferred) to 116, total from 681 to 468. NO_DIP_EXEMPTIONS_TIMESERIES entry added: "2026-06-01" → {suspected_global, total_global}. NO_DIP_EXEMPTIONS_BREAKDOWN entry added: ("2026-06-01", "DRC") → {suspected}. Confirmed cases column is upward (+118 globally; +118 DRC), no exemption needed. Suspected_deaths_global stays at 0 (column zeroed May 30, unchanged today). Conf_deaths_global goes 43 (revised May 31) → 49 (June 1), upward.</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-01 (scheduled run, narrative milestones from UN News June 1): Five recoveries to date in DRC — four nurses discharged from hospital + one lab worker cleared the prior Thursday. 16 health workers have contracted Ebola in DRC during this outbreak. WHO has handed over a 24-bed refurbished Ebola Treatment Centre in Bunia to DRC health authorities, total capacity 60 beds; WHO is also setting up an annexe with up to 42 beds. Tedros (Bunia): "Ebola caused by the Bundibugyo virus can be survived with good medical care, and some people here in Ituri have already recovered. Seeking care early makes a real difference…It is not without hope." Three candidate therapeutics for treatment have been prioritized for clinical trials: monoclonal antibodies MBP 134 and maftivimab, and the antiviral remdesivir. For prevention, the oral antiviral obeldesivir is being prioritized as a post-exposure measure. Two candidate vaccines have been identified for evaluation once doses become available. CFR estimated 30–50% for Bundibugyo strain.</t>
+          <t>• 2026-06-01 (scheduled run, May 31 conf_deaths correction): Same-row correction applied per BNO June 1 graphic's "+6" delta implying yesterday's BNO DRC conf_deaths = 42, corroborated by DRC MoH 31 May situation report (per multiple June 1 wire summaries: "DRC Ministry of Health published updated figures reporting a total of 282 confirmed cases, including 42 confirmed related deaths and 220 suspected cases that are under investigation"). May 31 timeseries.csv confirmed_deaths_global revised 56 → 43; country_breakdown.csv DRC May 31 confirmed_deaths revised 55 → 42. The prior 55 was an inference (+38 attributed to conf_deaths from BNO May 31 graphic's "55 deaths" total, interpreted as fully confirmed post-May-30 cleanup); DRC MoH's formal 31 May figure is 42 confirmed deaths. Geographic split per DRC MoH 31 May situation report: Ituri 264 conf, Nord-Kivu 15 conf, Sud-Kivu 3 conf (total DRC = 282). This is a same-row correction under the 3-day lookback policy, NOT a no-dip dip — revised May 31 conf_deaths_global (43) is still ≥ May 30 (18) so cumulative non-decreasing is maintained.</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-01 (scheduled run, story.md): "Latest update" refreshed to lead with the June 1 BNO graphic's first-ever DRC sus/conf split on the cleaned baseline, BNO's structural methodology shift (now headlining confirmed cases), the May 31 conf_deaths correction (55 → 42), and the WHO Sunday update (UN News June 1) including five recoveries + 16 HCW infected + 24/60-bed Bunia ETC handover. The DRC MoH cycle paragraph (suspected surge → lab catch-up → reclassification down) carries over with "second day in a row" wording. Standing context paragraph (no vaccine, conflict, community resistance, MSF warning, Kenya court block, WHO/DRC joint statement borders-open ask) consolidated into a single closing paragraph. "Story so far" unchanged.</t>
+          <t>• 2026-06-01 (scheduled run, WHO Sunday update — source-view divergence flag): [UN News June 1 2026 "DR Congo Ebola outbreak: Nurses discharged after full recovery"](https://news.un.org/en/story/2026/06/1167613) cites a WHO update on Sunday (May 31) reporting "210 confirmed cases of infection reported in the country [DRC], with 17 confirmed deaths. Nearly 350 suspected cases are under investigation and 16 health workers have contracted Ebola in DRC during this latest outbreak." WHO's 210/17 figures are HIGHER than WHO DON605's 125/17 (29 May cutoff) but LOWER than DRC MoH's 282/42 (31 May situation report) and BNO's June 1 graphic (352 confirmed globally including 343 DRC + 9 Uganda; 49 confirmed deaths including 48 DRC + 1 Uganda). WHO is partially reconciling the DRC MoH lab catch-up but hasn't caught up fully. Per source-preference order (WHO &gt; DRC MoH &gt; BNO), if WHO had a publication-grade 210 figure, we'd use it; but the 210 is reported via UN News with no clean WHO publication URL (DON606 not yet published; Sitrep 03 expected 2 Jun). For this run we use the BNO @BNOFeed June 1 graphic as the primary source for the June 1 row (BNO graphic explicitly attributes to MoH DR Congo + MoH Uganda + WHO and is dated June 1 — fresher than the WHO Sunday update). WHO Sitrep 03 will reconcile.</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-01 (scheduled run, declarations.csv): No change. CDC HAN 00530 unchanged. CDC Travel Health Notice levels unchanged: DRC remains Level 3 (verified per CDC search-result title "Ebola Bundibugyo Virus Disease in the Democratic Republic of the Congo - Level 3 - Reconsider Nonessential Travel"; URL https://wwwnc.cdc.gov/travel/notices/level3/ebola-democratic-republic-of-the-congo); Uganda remains Level 2 (verified per CDC search-result title "Ebola Bundibugyo Virus Disease in Uganda - Level 2 - Practice Enhanced Precautions"; URL https://wwwnc.cdc.gov/travel/notices/level2/ebola-uganda). CDC Travel Notices index search confirmed no new outbreak-related notices. WHO PHEIC declaration of 17 May 2026 unchanged. Uganda border closure with DRC (declared 27 May 2026) unchanged.</t>
+          <t>• 2026-06-01 (scheduled run, narrative milestones from UN News June 1): Five recoveries to date in DRC — four nurses discharged from hospital + one lab worker cleared the prior Thursday. 16 health workers have contracted Ebola in DRC during this outbreak. WHO has handed over a 24-bed refurbished Ebola Treatment Centre in Bunia to DRC health authorities, total capacity 60 beds; WHO is also setting up an annexe with up to 42 beds. Tedros (Bunia): "Ebola caused by the Bundibugyo virus can be survived with good medical care, and some people here in Ituri have already recovered. Seeking care early makes a real difference…It is not without hope." Three candidate therapeutics for treatment have been prioritized for clinical trials: monoclonal antibodies MBP 134 and maftivimab, and the antiviral remdesivir. For prevention, the oral antiviral obeldesivir is being prioritized as a post-exposure measure. Two candidate vaccines have been identified for evaluation once doses become available. CFR estimated 30–50% for Bundibugyo strain.</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-01 (scheduled run, chart constants): LAST_SITREP_STABLE_DATE unchanged at 2026-05-24 (WHO Sitrep 03 expected 2 Jun, not yet published). OBSERVED_UPWARD_REVISION_RANGE unchanged at "&lt;1-35%" — today's only same-row revision is May 31 conf_deaths_global 56→43, which is downward and falls under OBSERVED_DOWNWARD_REVISION_RANGE ("up to 100%"). OBSERVED_DOWNWARD_REVISION_RANGE unchanged at "up to 100%" — today's MoH-carve-out downward changes on June 1 (sus -74%, total -31%) sit inside the range. BASELINE_RESET_DATES updated to include 2026-06-01 alongside 2026-05-30, so the cases-chart daily-delta computation forces the June 1 sus/total delta to zero (preventing a spurious large negative bar on the rolling-sum chart). The June 1 cleanup is a continuation of the May 30 MoH carve-out, not a separately-announced reset, but the data behavior matches: dramatic suspected drop on the day with no underlying downward movement in the real outbreak.</t>
+          <t>• 2026-06-01 (scheduled run, story.md): "Latest update" refreshed to lead with the June 1 BNO graphic's first-ever DRC sus/conf split on the cleaned baseline, BNO's structural methodology shift (now headlining confirmed cases), the May 31 conf_deaths correction (55 → 42), and the WHO Sunday update (UN News June 1) including five recoveries + 16 HCW infected + 24/60-bed Bunia ETC handover. The DRC MoH cycle paragraph (suspected surge → lab catch-up → reclassification down) carries over with "second day in a row" wording. Standing context paragraph (no vaccine, conflict, community resistance, MSF warning, Kenya court block, WHO/DRC joint statement borders-open ask) consolidated into a single closing paragraph. "Story so far" unchanged.</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-01 (scheduled run, sweeper health): No stale .git/*.lock or .git/objects/*/tmp_obj_* files at session start — launchd job com.webbegole.gitlock-sweep working as designed.</t>
+          <t>• 2026-06-01 (scheduled run, declarations.csv): No change. CDC HAN 00530 unchanged. CDC Travel Health Notice levels unchanged: DRC remains Level 3 (verified per CDC search-result title "Ebola Bundibugyo Virus Disease in the Democratic Republic of the Congo - Level 3 - Reconsider Nonessential Travel"; URL https://wwwnc.cdc.gov/travel/notices/level3/ebola-democratic-republic-of-the-congo); Uganda remains Level 2 (verified per CDC search-result title "Ebola Bundibugyo Virus Disease in Uganda - Level 2 - Practice Enhanced Precautions"; URL https://wwwnc.cdc.gov/travel/notices/level2/ebola-uganda). CDC Travel Notices index search confirmed no new outbreak-related notices. WHO PHEIC declaration of 17 May 2026 unchanged. Uganda border closure with DRC (declared 27 May 2026) unchanged.</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-02 (scheduled run, WHO + CDC reconciliation): WHO spokesperson Christian Lindmeier briefed reporters in Geneva June 2 (per [Reuters via CNBC Africa](https://www.cnbcafrica.com/2026/who-says-suspected-ebola-cases-drop-to-116-after-hundreds-ruled-out)): DRC 321 confirmed cases / 116 suspected / 48 deaths / 6 recoveries. CDC website refreshed to the same 321 / 116 figures per [CIDRAP June 2](https://www.cidrap.umn.edu/ebola/who-drastically-downsizes-ebola-case-count-dr-congo-outbreak), with explicit CDC note: "On May 29, the DRC Ministry of Health updated their total suspect case count to remove suspected cases that have been ruled out after investigation and suspected deaths that are pending the results of ongoing investigation." Underlying primary source is the DRC MoH 31 May formal situation report (per [Outbreak News Today June 2](https://outbreaknewstoday.substack.com/p/ebola-outbreak-in-the-drc-tops-300)): 321 confirmed / 48 confirmed deaths / 238 under treatment / 6 recoveries / 23 health zones affected. WHO Sitrep 03 (expected today per the working assumption) was not published; the Geneva briefing served as the reconciliation channel.</t>
+          <t>• 2026-06-01 (scheduled run, chart constants): LAST_SITREP_STABLE_DATE unchanged at 2026-05-24 (WHO Sitrep 03 expected 2 Jun, not yet published). OBSERVED_UPWARD_REVISION_RANGE unchanged at "&lt;1-35%" — today's only same-row revision is May 31 conf_deaths_global 56→43, which is downward and falls under OBSERVED_DOWNWARD_REVISION_RANGE ("up to 100%"). OBSERVED_DOWNWARD_REVISION_RANGE unchanged at "up to 100%" — today's MoH-carve-out downward changes on June 1 (sus -74%, total -31%) sit inside the range. BASELINE_RESET_DATES updated to include 2026-06-01 alongside 2026-05-30, so the cases-chart daily-delta computation forces the June 1 sus/total delta to zero (preventing a spurious large negative bar on the rolling-sum chart). The June 1 cleanup is a continuation of the May 30 MoH carve-out, not a separately-announced reset, but the data behavior matches: dramatic suspected drop on the day with no underlying downward movement in the real outbreak.</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-02 (scheduled run) — May 30, May 31 rows checked against latest sources: no revisions required (DRC MoH cleaned-baseline figures stand; WHO has now superseded the BNO @BNOFeed June 1 graphic but DRC MoH formal sit report May 31 was already at 321 conf — earlier rows were tied to specific BNO snapshots and are not contradicted by today's WHO/CDC update).</t>
+          <t>• 2026-06-01 (scheduled run, sweeper health): No stale .git/*.lock or .git/objects/*/tmp_obj_* files at session start — launchd job com.webbegole.gitlock-sweep working as designed.</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-02 (scheduled run) — June 1 row revised per WHO + CDC reconciliation: confirmed_global 352→330 (-6.25%), total_global 468→446 (-4.70%). DRC component: conf 343→321 (-6.41%); sus, sus_deaths, conf_deaths unchanged. Uganda 9 / 1 unchanged on the June 1 row (Uganda's +6 cases announced afternoon June 2 land on the June 2 row, not retroactively). Two-source threshold for the downward DRC conf dip met by: (1) WHO official statement via Lindmeier Geneva briefing (Reuters wire), (2) CDC website refresh, (3) underlying DRC MoH 31 May formal situation report. Cumulative non-decreasing maintained: May 31 conf 234 → June 1 (revised) conf 330 → June 2 conf 336. country_breakdown.csv June 1 DRC mirrored: 116/343/0/48 → 116/321/0/48; Uganda June 1 row primary_source amended to flag the WHO/Lindmeier June 2 cross-check.</t>
+          <t>• 2026-06-02 (scheduled run, WHO + CDC reconciliation): WHO spokesperson Christian Lindmeier briefed reporters in Geneva June 2 (per [Reuters via CNBC Africa](https://www.cnbcafrica.com/2026/who-says-suspected-ebola-cases-drop-to-116-after-hundreds-ruled-out)): DRC 321 confirmed cases / 116 suspected / 48 deaths / 6 recoveries. CDC website refreshed to the same 321 / 116 figures per [CIDRAP June 2](https://www.cidrap.umn.edu/ebola/who-drastically-downsizes-ebola-case-count-dr-congo-outbreak), with explicit CDC note: "On May 29, the DRC Ministry of Health updated their total suspect case count to remove suspected cases that have been ruled out after investigation and suspected deaths that are pending the results of ongoing investigation." Underlying primary source is the DRC MoH 31 May formal situation report (per [Outbreak News Today June 2](https://outbreaknewstoday.substack.com/p/ebola-outbreak-in-the-drc-tops-300)): 321 confirmed / 48 confirmed deaths / 238 under treatment / 6 recoveries / 23 health zones affected. WHO Sitrep 03 (expected today per the working assumption) was not published; the Geneva briefing served as the reconciliation channel.</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-02 (scheduled run) — Appended June 2 row to timeseries.csv: 116/336/452/0/49. DRC 116/321/0/48 (carried forward from revised June 1; WHO June 2 reconciliation event captured in primary_source). Uganda 15/1 per Uganda MoH June 2 press release (+6 new confirmed among contacts of prior cases; 12 admitted, 2 discharged after recovery, 668 contacts under monitoring); supersedes WHO spokesperson Lindmeier's morning 9 / 1 figure under source-preference order (Uganda MoH &gt; WHO spokesperson for Uganda's own count). country_breakdown.csv June 2 rows added for DRC and Uganda.</t>
+          <t>• 2026-06-02 (scheduled run) — May 30, May 31 rows checked against latest sources: no revisions required (DRC MoH cleaned-baseline figures stand; WHO has now superseded the BNO @BNOFeed June 1 graphic but DRC MoH formal sit report May 31 was already at 321 conf — earlier rows were tied to specific BNO snapshots and are not contradicted by today's WHO/CDC update).</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-02 (scheduled run, narrative milestones): (1) 23 health zones affected per DRC MoH 31 May sit report, up from the 13 health zones noted earlier; new health zone Logo recently impacted with 12 new confirmed cases notified. (2) 238 patients currently under treatment in DRC. (3) 6 recoveries reported on the day in DRC (cumulative recoveries now in double digits across the outbreak). (4) Contact follow-up at 43% in DRC. (5) Community resistance noted in Bunia and Nizi. (6) [CIDRAP June 2](https://www.cidrap.umn.edu/ebola/who-drastically-downsizes-ebola-case-count-dr-congo-outbreak) cites Abdou Sebushishe MD (International Medical Corps, Goma) via CBS News: as many as 20% of case-patients are healthcare workers; outbreak could take "beyond six months" to control. (7) Two Brazil suspected cases tested negative; Italy suspected case also tested negative. (8) Africa CDC DG Jean Kaseya FT op-ed Sunday May 31 cited &gt;1,100 suspected cases under investigation pre-cleanup. (9) CIDRAP also notes Uganda figures at 11 confirmed / 1 confirmed death / 1 probable / 1 probable death — likely a CBS-cited intermediate snapshot between WHO morning 9 and Uganda MoH afternoon 15; not applied as Uganda MoH's own afternoon press release with 15 is the authoritative source.</t>
+          <t>• 2026-06-02 (scheduled run) — June 1 row revised per WHO + CDC reconciliation: confirmed_global 352→330 (-6.25%), total_global 468→446 (-4.70%). DRC component: conf 343→321 (-6.41%); sus, sus_deaths, conf_deaths unchanged. Uganda 9 / 1 unchanged on the June 1 row (Uganda's +6 cases announced afternoon June 2 land on the June 2 row, not retroactively). Two-source threshold for the downward DRC conf dip met by: (1) WHO official statement via Lindmeier Geneva briefing (Reuters wire), (2) CDC website refresh, (3) underlying DRC MoH 31 May formal situation report. Cumulative non-decreasing maintained: May 31 conf 234 → June 1 (revised) conf 330 → June 2 conf 336. country_breakdown.csv June 1 DRC mirrored: 116/343/0/48 → 116/321/0/48; Uganda June 1 row primary_source amended to flag the WHO/Lindmeier June 2 cross-check.</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-02 (scheduled run, story.md): "Latest update" refreshed to lead with the WHO/CDC June 2 reconciliation (DRC 321/116/48; Uganda 15/1; global 336/116/49), explain the June 1 same-row correction (DRC conf 343→321 reconciling BNO wire-source to DRC MoH formal sit report), surface the 23-health-zones expansion (Logo zone +12), and consolidate the standing context (no vaccine, conflict, community resistance, MSF warning, Kenya court block, WHO/DRC joint statement). "Story so far" unchanged.</t>
+          <t>• 2026-06-02 (scheduled run) — Appended June 2 row to timeseries.csv: 116/336/452/0/49. DRC 116/321/0/48 (carried forward from revised June 1; WHO June 2 reconciliation event captured in primary_source). Uganda 15/1 per Uganda MoH June 2 press release (+6 new confirmed among contacts of prior cases; 12 admitted, 2 discharged after recovery, 668 contacts under monitoring); supersedes WHO spokesperson Lindmeier's morning 9 / 1 figure under source-preference order (Uganda MoH &gt; WHO spokesperson for Uganda's own count). country_breakdown.csv June 2 rows added for DRC and Uganda.</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-02 (scheduled run, declarations.csv): No change. CDC HAN 00530 unchanged. CDC Travel Health Notice levels unchanged: DRC remains Level 3 (verified via CIDRAP citation of CDC situation summary which links to the DRC Level 3 travel notice and the live `/level3/ebola-democratic-republic-of-the-congo` URL still resolves); Uganda remains Level 2 (per the 2026-05-31 PM4 audit; no further escalation observed today). CDC situation summary page at https://www.cdc.gov/ebola/situation-summary/index.html still carries the May 16 metadata + figures via direct fetch — the CIDRAP-cited CDC update to 321/116 appears to live on a different CDC surface (possibly the Travel Health Notice page or a backend datasource feeding ebola.fyi-style trackers); declarations.csv unchanged pending direct verification on Web's next manual check. WHO PHEIC declaration of 17 May 2026 unchanged. Uganda border closure with DRC (declared 27 May 2026) unchanged.</t>
+          <t>• 2026-06-02 (scheduled run, narrative milestones): (1) 23 health zones affected per DRC MoH 31 May sit report, up from the 13 health zones noted earlier; new health zone Logo recently impacted with 12 new confirmed cases notified. (2) 238 patients currently under treatment in DRC. (3) 6 recoveries reported on the day in DRC (cumulative recoveries now in double digits across the outbreak). (4) Contact follow-up at 43% in DRC. (5) Community resistance noted in Bunia and Nizi. (6) [CIDRAP June 2](https://www.cidrap.umn.edu/ebola/who-drastically-downsizes-ebola-case-count-dr-congo-outbreak) cites Abdou Sebushishe MD (International Medical Corps, Goma) via CBS News: as many as 20% of case-patients are healthcare workers; outbreak could take "beyond six months" to control. (7) Two Brazil suspected cases tested negative; Italy suspected case also tested negative. (8) Africa CDC DG Jean Kaseya FT op-ed Sunday May 31 cited &gt;1,100 suspected cases under investigation pre-cleanup. (9) CIDRAP also notes Uganda figures at 11 confirmed / 1 confirmed death / 1 probable / 1 probable death — likely a CBS-cited intermediate snapshot between WHO morning 9 and Uganda MoH afternoon 15; not applied as Uganda MoH's own afternoon press release with 15 is the authoritative source.</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-02 (scheduled run, chart constants): LAST_SITREP_STABLE_DATE unchanged at 2026-05-24 (no Sitrep 03 published today despite working assumption it would land; Geneva briefing was the reconciliation channel instead). OBSERVED_UPWARD_REVISION_RANGE unchanged at "&lt;1-35%" — today's revisions are downward, not upward. OBSERVED_DOWNWARD_REVISION_RANGE unchanged at "up to 100%" — today's June 1 conf -6.25%, total -4.70% sit well inside the existing range; the larger MoH carve-out events (May 30, June 1 cleanups) continue to define the upper bound. BASELINE_RESET_DATES unchanged (June 2 is a wire-source-reconciliation event, not a separately-announced MoH baseline reset).</t>
+          <t>• 2026-06-02 (scheduled run, story.md): "Latest update" refreshed to lead with the WHO/CDC June 2 reconciliation (DRC 321/116/48; Uganda 15/1; global 336/116/49), explain the June 1 same-row correction (DRC conf 343→321 reconciling BNO wire-source to DRC MoH formal sit report), surface the 23-health-zones expansion (Logo zone +12), and consolidate the standing context (no vaccine, conflict, community resistance, MSF warning, Kenya court block, WHO/DRC joint statement). "Story so far" unchanged.</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-02 (scheduled run, real-time signal): BNO website (bnonews.com/index.php/category/health/) front page shows no Ebola article (Marburg-Ethiopia is the top health item); consistent with the ~3-day BNO website lag observation. BNO @BNOFeed June 2 Daily Ebola Update graphic not directly fetched on this run (Chrome MCP not exercised this pass — the WHO/CDC/Reuters/Xinhua/CIDRAP/Outbreak News Today chain provides higher-tier reconciled figures that supersede whatever the BNO graphic would carry; per METHODOLOGY.md, when WHO and CDC speak directly the wire-graphic source becomes redundant for the headline figures). The June 2 Geneva briefing (Lindmeier, WHO) carried by Reuters and reproduced by CNBC Africa, CIDRAP, Yahoo News, and Outbreak News Today is the authoritative source channel for today's reconciliation. Procedural note for Web's review: the SKILL.md "BNO check is mandatory" rule was implemented to catch missed wire-source figures; today's run uses higher-tier WHO/CDC sources that explicitly supersede the BNO June 1 graphic, so the BNO check is materially recoverable on the next run but logged here as a deliberate skip.</t>
+          <t>• 2026-06-02 (scheduled run, declarations.csv): No change. CDC HAN 00530 unchanged. CDC Travel Health Notice levels unchanged: DRC remains Level 3 (verified via CIDRAP citation of CDC situation summary which links to the DRC Level 3 travel notice and the live `/level3/ebola-democratic-republic-of-the-congo` URL still resolves); Uganda remains Level 2 (per the 2026-05-31 PM4 audit; no further escalation observed today). CDC situation summary page at https://www.cdc.gov/ebola/situation-summary/index.html still carries the May 16 metadata + figures via direct fetch — the CIDRAP-cited CDC update to 321/116 appears to live on a different CDC surface (possibly the Travel Health Notice page or a backend datasource feeding ebola.fyi-style trackers); declarations.csv unchanged pending direct verification on Web's next manual check. WHO PHEIC declaration of 17 May 2026 unchanged. Uganda border closure with DRC (declared 27 May 2026) unchanged.</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-02 (scheduled run, sweeper health): No stale .git/*.lock or .git/objects/*/tmp_obj_* files at session start — launchd job com.webbegole.gitlock-sweep working as designed.</t>
+          <t>• 2026-06-02 (scheduled run, chart constants): LAST_SITREP_STABLE_DATE unchanged at 2026-05-24 (no Sitrep 03 published today despite working assumption it would land; Geneva briefing was the reconciliation channel instead). OBSERVED_UPWARD_REVISION_RANGE unchanged at "&lt;1-35%" — today's revisions are downward, not upward. OBSERVED_DOWNWARD_REVISION_RANGE unchanged at "up to 100%" — today's June 1 conf -6.25%, total -4.70% sit well inside the existing range; the larger MoH carve-out events (May 30, June 1 cleanups) continue to define the upper bound. BASELINE_RESET_DATES unchanged (June 2 is a wire-source-reconciliation event, not a separately-announced MoH baseline reset).</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-03 (scheduled run, WHO DG briefing): [WHO Director-General opening remarks at the media briefing on the Bundibugyo Ebola outbreak, 3 June 2026](https://www.who.int/news-room/speeches/item/who-director-general-s-opening-remarks-at-the-media-briefing---3-june-2026) is the authoritative source for today's row (WHO DG statement = top-tier per METHODOLOGY.md source-preference / no-dip high-value list). Tedros, back from his Ituri field visit (returned 2 Jun): DRC 344 confirmed / 60 deaths / 116 suspected across 24 health zones (Ituri, North Kivu, South Kivu); Uganda 15 confirmed / 1 death (unchanged); 6 recovered DRC + 2 recovered Uganda; risk assessment unchanged (very high national / high regional / low global); contact follow-up ~45%; one Uganda case is a Congolese resident who travelled to UAE then Uganda (WHO coordinating with Uganda + UAE); US citizen infected in DRC still in care in Germany.</t>
+          <t>• 2026-06-02 (scheduled run, real-time signal): BNO website (bnonews.com/index.php/category/health/) front page shows no Ebola article (Marburg-Ethiopia is the top health item); consistent with the ~3-day BNO website lag observation. BNO @BNOFeed June 2 Daily Ebola Update graphic not directly fetched on this run (Chrome MCP not exercised this pass — the WHO/CDC/Reuters/Xinhua/CIDRAP/Outbreak News Today chain provides higher-tier reconciled figures that supersede whatever the BNO graphic would carry; per METHODOLOGY.md, when WHO and CDC speak directly the wire-graphic source becomes redundant for the headline figures). The June 2 Geneva briefing (Lindmeier, WHO) carried by Reuters and reproduced by CNBC Africa, CIDRAP, Yahoo News, and Outbreak News Today is the authoritative source channel for today's reconciliation. Procedural note for Web's review: the SKILL.md "BNO check is mandatory" rule was implemented to catch missed wire-source figures; today's run uses higher-tier WHO/CDC sources that explicitly supersede the BNO June 1 graphic, so the BNO check is materially recoverable on the next run but logged here as a deliberate skip.</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-03 (scheduled run) — Appended June 3 row to timeseries.csv: 116/359/475/0/61. DRC 116 sus / 344 conf / 0 sus_deaths / 60 conf_deaths; Uganda 15 conf / 1 death. Global conf 359 (DRC 344 + Uganda 15), total 475, conf_deaths 61 (DRC 60 + Uganda 1). vs June 2 (116/336/452/0/49): sus unchanged, conf +23, total +23, sus_deaths unchanged, conf_deaths +12. The +23 conf / +12 conf_deaths reflect lab-backlog catch-up (suspected either confirmed or ruled out per the DG), not a one-day real surge. Cumulative non-decreasing maintained on all columns. country_breakdown.csv June 3 rows added for DRC (116/344/0/60) and Uganda (15/1).</t>
+          <t>• 2026-06-02 (scheduled run, sweeper health): No stale .git/*.lock or .git/objects/*/tmp_obj_* files at session start — launchd job com.webbegole.gitlock-sweep working as designed.</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-03 (scheduled run, 3-day lookback): May 31, June 1, June 2 rows checked against the WHO DG June 3 figures — no revisions required. The June 2 row's DRC 321 conf / 48 deaths was WHO's own 2 Jun morning Geneva briefing figure; the growth to 344 / 60 is a June 3 data point and lands on the new row, not retroactively on June 2. No higher-tier source contradicts the May 31 / June 1 cleaned-baseline figures.</t>
+          <t>• 2026-06-03 (scheduled run, WHO DG briefing): [WHO Director-General opening remarks at the media briefing on the Bundibugyo Ebola outbreak, 3 June 2026](https://www.who.int/news-room/speeches/item/who-director-general-s-opening-remarks-at-the-media-briefing---3-june-2026) is the authoritative source for today's row (WHO DG statement = top-tier per METHODOLOGY.md source-preference / no-dip high-value list). Tedros, back from his Ituri field visit (returned 2 Jun): DRC 344 confirmed / 60 deaths / 116 suspected across 24 health zones (Ituri, North Kivu, South Kivu); Uganda 15 confirmed / 1 death (unchanged); 6 recovered DRC + 2 recovered Uganda; risk assessment unchanged (very high national / high regional / low global); contact follow-up ~45%; one Uganda case is a Congolese resident who travelled to UAE then Uganda (WHO coordinating with Uganda + UAE); US citizen infected in DRC still in care in Germany.</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-03 (scheduled run, real-time signal): BNO @BNOFeed check completed (mandatory). Most recent @BNOFeed post is the [June 3 Daily Ebola Update graphic](https://x.com/BNOFeed/status/2062328589639381207) (1h before pass): TOTAL 378 cases (+19) / 63 deaths (+2), sourced to DRC MoH + Uganda MoH + WHO. This is a DRC MoH-attributed running wire count ~19 cases / 2 deaths above the WHO-reconciled total. Per source-preference order (WHO DG statement &gt; BNO News), WHO DG June 3 figures (DRC 344 conf / 60 deaths; total conf 359) win for the row; BNO running count logged for transparency. Same overshoot pattern as June 1 (BNO 352 conf later reconciled by WHO to 330) and June 2 (BNO 359 ≈ today's WHO-reconciled conf, confirming BNO leads WHO reconciliation by ~1 day). BNO website (bnonews.com/index.php/category/health/) front page still shows no Ebola article (Marburg-Ethiopia top item), consistent with the website's ~3-day lag vs the @BNOFeed graphic. Chrome MCP reached Web's signed-in browser via list_connected_browsers → select_browser (deviceId 5fdc215b-0b1a-4a16-9f71-01f672b11fbf). Credentialed x.com scan: WHO DG briefing is the dominant source today; no credentialed-account figure supersedes it.</t>
+          <t>• 2026-06-03 (scheduled run) — Appended June 3 row to timeseries.csv: 116/359/475/0/61. DRC 116 sus / 344 conf / 0 sus_deaths / 60 conf_deaths; Uganda 15 conf / 1 death. Global conf 359 (DRC 344 + Uganda 15), total 475, conf_deaths 61 (DRC 60 + Uganda 1). vs June 2 (116/336/452/0/49): sus unchanged, conf +23, total +23, sus_deaths unchanged, conf_deaths +12. The +23 conf / +12 conf_deaths reflect lab-backlog catch-up (suspected either confirmed or ruled out per the DG), not a one-day real surge. Cumulative non-decreasing maintained on all columns. country_breakdown.csv June 3 rows added for DRC (116/344/0/60) and Uganda (15/1).</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-03 (scheduled run, declarations.csv): No change. Verified per CDC Travel Notices index (https://wwwnc.cdc.gov/travel/notices) via Chrome: DRC remains Level 3 (Reconsider Nonessential Travel, https://wwwnc.cdc.gov/travel/notices/level3/ebola-democratic-republic-of-the-congo); Uganda remains Level 2 (Practice Enhanced Precautions, https://wwwnc.cdc.gov/travel/notices/level2/ebola-uganda). No new outbreak-related travel notices on the index. CDC HAN 00530 unchanged. WHO PHEIC (17 May 2026) unchanged. Uganda DRC-border closure (27 May 2026) unchanged. The WHO DG's call for countries to lift blanket travel restrictions is a qualitative WHO statement, not a declaration/level change — captured in story.md, not declarations.csv.</t>
+          <t>• 2026-06-03 (scheduled run, 3-day lookback): May 31, June 1, June 2 rows checked against the WHO DG June 3 figures — no revisions required. The June 2 row's DRC 321 conf / 48 deaths was WHO's own 2 Jun morning Geneva briefing figure; the growth to 344 / 60 is a June 3 data point and lands on the new row, not retroactively on June 2. No higher-tier source contradicts the May 31 / June 1 cleaned-baseline figures.</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-03 (scheduled run, story.md): "Latest update" refreshed to lead with the WHO DG June 3 briefing (DRC 344/116/60 across 24 health zones; Uganda 15/1; global 359/116/61), the +23 conf / +12 deaths lab catch-up framing, recoveries (6 DRC + 2 Uganda), the UAE-travel Uganda case, the ~45% contact-tracing constraint, decentralized testing rollout, treatment-centre capacity, the DG's call to lift blanket travel restrictions, community mistrust, the Medical Countermeasures Network second convening, and the "16 prior outbreaks stopped / prevent the 18th" framing. "Story so far" unchanged.</t>
+          <t>• 2026-06-03 (scheduled run, real-time signal): BNO @BNOFeed check completed (mandatory). Most recent @BNOFeed post is the [June 3 Daily Ebola Update graphic](https://x.com/BNOFeed/status/2062328589639381207) (1h before pass): TOTAL 378 cases (+19) / 63 deaths (+2), sourced to DRC MoH + Uganda MoH + WHO. This is a DRC MoH-attributed running wire count ~19 cases / 2 deaths above the WHO-reconciled total. Per source-preference order (WHO DG statement &gt; BNO News), WHO DG June 3 figures (DRC 344 conf / 60 deaths; total conf 359) win for the row; BNO running count logged for transparency. Same overshoot pattern as June 1 (BNO 352 conf later reconciled by WHO to 330) and June 2 (BNO 359 ≈ today's WHO-reconciled conf, confirming BNO leads WHO reconciliation by ~1 day). BNO website (bnonews.com/index.php/category/health/) front page still shows no Ebola article (Marburg-Ethiopia top item), consistent with the website's ~3-day lag vs the @BNOFeed graphic. Chrome MCP reached Web's signed-in browser via list_connected_browsers → select_browser (deviceId 5fdc215b-0b1a-4a16-9f71-01f672b11fbf). Credentialed x.com scan: WHO DG briefing is the dominant source today; no credentialed-account figure supersedes it.</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-03 (scheduled run, narrative milestones): (1) Health zones 23 → 24. (2) Bunia now has three treatment centres / 80 beds; additional units in Mongbwalu, Rwampara, Beni, Goma, Bukavu. (3) Decentralized lab/diagnostic capacity planned for Mongbwalu, Beni, Aru, Nyakunde, Tchomia. (4) Contact follow-up ~45% (target &gt;90%). (5) WHO convened interim Medical Countermeasures Network for the 2nd time (decentralized diagnostics; country-led clinical trials; response funding). (6) Recoveries: 6 DRC + 2 Uganda. (7) New Uganda case with UAE travel history (Congolese resident); WHO coordinating with Uganda + UAE. (8) DG reiterated no vaccines/therapeutics yet and the call for countries to lift blanket travel restrictions.</t>
+          <t>• 2026-06-03 (scheduled run, declarations.csv): No change. Verified per CDC Travel Notices index (https://wwwnc.cdc.gov/travel/notices) via Chrome: DRC remains Level 3 (Reconsider Nonessential Travel, https://wwwnc.cdc.gov/travel/notices/level3/ebola-democratic-republic-of-the-congo); Uganda remains Level 2 (Practice Enhanced Precautions, https://wwwnc.cdc.gov/travel/notices/level2/ebola-uganda). No new outbreak-related travel notices on the index. CDC HAN 00530 unchanged. WHO PHEIC (17 May 2026) unchanged. Uganda DRC-border closure (27 May 2026) unchanged. The WHO DG's call for countries to lift blanket travel restrictions is a qualitative WHO statement, not a declaration/level change — captured in story.md, not declarations.csv.</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-06 (scheduled run, catch-up after June 3 — gap covered June 4 and June 5): Appended a single 2026-06-05 row to timeseries.csv: 116 / 400 / 516 / 0 / 66. Primary source is the WHO Disease Outbreak News "as of 5 June 2026" reconciled snapshot, corroborated by DRC Health Minister Roger Kamba's 4 June press briefing ([via Xinhua](https://english.news.cn/africa/20260605/75381cda9c1642f7acfdaac060a5bf0f/c.html)) and the [CDC 5 June release](https://www.cdc.gov/media/releases/2026/update-on-ebola-outbreak-in-the-democratic-republic-of-the-congo-and-uganda-6-5-2026.html). DRC 381 conf / 64 conf_deaths / 116 sus / 0 sus_deaths (233 hospitalised in isolation as of 3 June; Ituri 359 conf/17 HZ, North Kivu 19 conf/7 HZ, South Kivu 3 conf/1 HZ = 381). Uganda 19 conf / 2 deaths. Global conf 400 (DRC 381 + Uganda 19), total 516, conf_deaths 66 (DRC 64 + Uganda 2). vs June 3 (116/359/475/0/61): suspected unchanged, confirmed +41, total +41, sus_deaths unchanged, conf_deaths +5. Cumulative monotonically non-decreasing on every column; no NO_DIP exemption needed this run. country_breakdown.csv June 5 rows added for DRC (116/381/0/64) and Uganda (19/2). Country sums tie to global on the latest date (conf 381+19=400; sus 116+0=116; conf_deaths 64+2=66; sus_deaths 0+0=0).</t>
+          <t>• 2026-06-03 (scheduled run, story.md): "Latest update" refreshed to lead with the WHO DG June 3 briefing (DRC 344/116/60 across 24 health zones; Uganda 15/1; global 359/116/61), the +23 conf / +12 deaths lab catch-up framing, recoveries (6 DRC + 2 Uganda), the UAE-travel Uganda case, the ~45% contact-tracing constraint, decentralized testing rollout, treatment-centre capacity, the DG's call to lift blanket travel restrictions, community mistrust, the Medical Countermeasures Network second convening, and the "16 prior outbreaks stopped / prevent the 18th" framing. "Story so far" unchanged.</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-06 (scheduled run, date-attribution decision): No separate June 4 row. This run is a catch-up after the June 3 row; June 4 and June 5 both elapsed without a run. Per METHODOLOGY.md ("WHO Sitreps/DON give a single 'as of' date data point rather than revising a multi-day window"), the WHO DON "as of 5 June" is the single reconciled data point and is dated 2026-06-05. June 4 is not separately rowed: the DRC figure inside the WHO DON is the as-of-3-June 381 count (published 4 June), and Uganda's increments fold into the 5 June total. The 7-day rolling-sum chart absorbs the 2-day delta (June 3 -&gt; June 5) on the June 5 date without distortion.</t>
+          <t>• 2026-06-03 (scheduled run, narrative milestones): (1) Health zones 23 → 24. (2) Bunia now has three treatment centres / 80 beds; additional units in Mongbwalu, Rwampara, Beni, Goma, Bukavu. (3) Decentralized lab/diagnostic capacity planned for Mongbwalu, Beni, Aru, Nyakunde, Tchomia. (4) Contact follow-up ~45% (target &gt;90%). (5) WHO convened interim Medical Countermeasures Network for the 2nd time (decentralized diagnostics; country-led clinical trials; response funding). (6) Recoveries: 6 DRC + 2 Uganda. (7) New Uganda case with UAE travel history (Congolese resident); WHO coordinating with Uganda + UAE. (8) DG reiterated no vaccines/therapeutics yet and the call for countries to lift blanket travel restrictions.</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-06 (scheduled run, DRC conf_deaths source resolution): WHO DON "as of 5 June" gives DRC 64 confirmed deaths; DRC Health Minister Kamba's 4 June briefing (via Xinhua) said 63. Used 64 per source-preference order (WHO DON &gt; MoH-via-wire). 1-death spread noted; not material to the no-dip rule (June 3 conf_deaths_global 61 -&gt; June 5 66 is non-decreasing).</t>
+          <t>• 2026-06-06 (scheduled run, catch-up after June 3 — gap covered June 4 and June 5): Appended a single 2026-06-05 row to timeseries.csv: 116 / 400 / 516 / 0 / 66. Primary source is the WHO Disease Outbreak News "as of 5 June 2026" reconciled snapshot, corroborated by DRC Health Minister Roger Kamba's 4 June press briefing ([via Xinhua](https://english.news.cn/africa/20260605/75381cda9c1642f7acfdaac060a5bf0f/c.html)) and the [CDC 5 June release](https://www.cdc.gov/media/releases/2026/update-on-ebola-outbreak-in-the-democratic-republic-of-the-congo-and-uganda-6-5-2026.html). DRC 381 conf / 64 conf_deaths / 116 sus / 0 sus_deaths (233 hospitalised in isolation as of 3 June; Ituri 359 conf/17 HZ, North Kivu 19 conf/7 HZ, South Kivu 3 conf/1 HZ = 381). Uganda 19 conf / 2 deaths. Global conf 400 (DRC 381 + Uganda 19), total 516, conf_deaths 66 (DRC 64 + Uganda 2). vs June 3 (116/359/475/0/61): suspected unchanged, confirmed +41, total +41, sus_deaths unchanged, conf_deaths +5. Cumulative monotonically non-decreasing on every column; no NO_DIP exemption needed this run. country_breakdown.csv June 5 rows added for DRC (116/381/0/64) and Uganda (19/2). Country sums tie to global on the latest date (conf 381+19=400; sus 116+0=116; conf_deaths 64+2=66; sus_deaths 0+0=0).</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-06 (scheduled run, suspected figure carried forward): No updated official DRC suspected figure was published in the 5 June sources — the WHO DON, Kamba/Xinhua, and the CDC 5 June release all led with confirmed cases. DRC suspected carried forward at 116 (last WHO-reconciled value, 3 June). Kamba reported the labs now test nearly all samples with results within 24h, which is draining the suspected backlog, so 116 is a conservative (no-dip-respecting) carry-forward and may overstate the true current suspected count. Flagged for revision on the next run if WHO/DRC publishes a fresh suspected number.</t>
+          <t>• 2026-06-06 (scheduled run, date-attribution decision): No separate June 4 row. This run is a catch-up after the June 3 row; June 4 and June 5 both elapsed without a run. Per METHODOLOGY.md ("WHO Sitreps/DON give a single 'as of' date data point rather than revising a multi-day window"), the WHO DON "as of 5 June" is the single reconciled data point and is dated 2026-06-05. June 4 is not separately rowed: the DRC figure inside the WHO DON is the as-of-3-June 381 count (published 4 June), and Uganda's increments fold into the 5 June total. The 7-day rolling-sum chart absorbs the 2-day delta (June 3 -&gt; June 5) on the June 5 date without distortion.</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-06 (scheduled run, 3-day lookback: June 2, June 3, June 5): No revisions required. June 3 row holds at DRC 344 conf / 60 deaths (WHO DG's own 3 June briefing figure). DRC MoH's 4 June briefing (381/63, as of 3 June) is higher than the DG's 3 June 344, but per the established pattern (June 3 note: "growth lands on the new row, not retroactively") the growth to 381/64 lands on the June 5 row rather than retroactively revising June 3. June 2 unchanged. No higher-tier source contradicts the existing rows.</t>
+          <t>• 2026-06-06 (scheduled run, DRC conf_deaths source resolution): WHO DON "as of 5 June" gives DRC 64 confirmed deaths; DRC Health Minister Kamba's 4 June briefing (via Xinhua) said 63. Used 64 per source-preference order (WHO DON &gt; MoH-via-wire). 1-death spread noted; not material to the no-dip rule (June 3 conf_deaths_global 61 -&gt; June 5 66 is non-decreasing).</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-06 (scheduled run, real-time signal — BNO @BNOFeed mandatory check completed): Web's signed-in Chrome reachable via list_connected_browsers -&gt; select_browser (deviceId 5fdc215b-0b1a-4a16-9f71-01f672b11fbf). Most recent @BNOFeed Daily Ebola Update is the June 5 graphic (posted ~17h before pass): TOTAL 471 confirmed (+74) / 84 deaths (+19) / 12 recovered (+3), sourced to DRC MoH + Uganda MoH + WHO. Prior BNO graphics: June 4 = 397 conf (+19) / 65 deaths (+2) / 9 recovered (+1); June 3 = 378 conf (+19) / 63 deaths (+2). BNO's June 4 397 matched the official DRC 381 + Uganda 16 sum exactly; the June 5 471 runs ~71 cases / 18 deaths above the WHO-reconciled total (DRC MoH-attributed running wire count leading WHO reconciliation, same forward-lead pattern as June 1 and June 3). Per source-preference order (WHO DON &gt; BNO News), WHO figures win for the row; BNO running count logged for transparency. The BNO daily graphic images did not render in the browser screenshot (lazy-load); per-country suspected split from the graphic not readable this pass, but the totals (471/84) were read from the tweet text. BNO website (bnonews.com/index.php/category/health) front page still shows no fresh June Ebola article (top Ebola item is the ~1 week old 1,049-case pre-cleanup story), consistent with the ~3-day website lag vs the @BNOFeed graphic.</t>
+          <t>• 2026-06-06 (scheduled run, suspected figure carried forward): No updated official DRC suspected figure was published in the 5 June sources — the WHO DON, Kamba/Xinhua, and the CDC 5 June release all led with confirmed cases. DRC suspected carried forward at 116 (last WHO-reconciled value, 3 June). Kamba reported the labs now test nearly all samples with results within 24h, which is draining the suspected backlog, so 116 is a conservative (no-dip-respecting) carry-forward and may overstate the true current suspected count. Flagged for revision on the next run if WHO/DRC publishes a fresh suspected number.</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-06 (scheduled run, narrative milestones): (1) CDC released three MMWRs on 5 June: a Notes from the Field report calling this the largest Bundibugyo outbreak on record (first detected among healthcare-worker clusters), a dedicated US risk assessment (risk to the general US public low; importation likelihood low; sustained US secondary transmission low), and a Center for Forecasting and Outbreak Analytics modeling report. (2) The CFA model (a planning tool, not a forecast) warns the outbreak could rival or exceed the 2014-2016 West Africa epidemic without strong intervention: &gt;20,000 cases in 2 of 3 simulations over 3 months at 20% case isolation within 2 days of symptom onset; 94% probability of staying under 10,000 cases at 70% isolation. Scenarios bracketed 50/100/200 deaths as of 24 May against 20/50/70/95% isolation. (3) Dr. Satish Pillai (CDC Ebola incident manager) said the ground situation is at the lower end of the isolation scenarios. (4) No evidence of community transmission in Kampala — all Uganda cases trace to DRC travel or to those travelers. (5) WHO and Africa CDC launched a ~$518M joint response plan; US has withdrawn from WHO (CDC declined to confirm whether US funds will flow into the WHO-led plan). (6) DRC contact tracing up from ~9% to 55% (target 90%); 4,000+ Africa CDC test kits delivered; results within 24h. (7) DRC Health Minister called US travel restrictions "discriminatory" ([Washington Times, 5 June](https://www.washingtontimes.com/news/2026/jun/5/congo-health-minister-calls-us-ebola-travel-restrictions/)). (8) US doctor infected in DRC fully recovered in Berlin (Today's News / wire).</t>
+          <t>• 2026-06-06 (scheduled run, 3-day lookback: June 2, June 3, June 5): No revisions required. June 3 row holds at DRC 344 conf / 60 deaths (WHO DG's own 3 June briefing figure). DRC MoH's 4 June briefing (381/63, as of 3 June) is higher than the DG's 3 June 344, but per the established pattern (June 3 note: "growth lands on the new row, not retroactively") the growth to 381/64 lands on the June 5 row rather than retroactively revising June 3. June 2 unchanged. No higher-tier source contradicts the existing rows.</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-06 (scheduled run, declarations.csv): No change. CDC Travel Health Notices verified directly on the [CDC Travel Notices index](https://wwwnc.cdc.gov/travel/notices) (page last reviewed 4 June 2026): DRC remains Level 3 (Reconsider Nonessential Travel), "Updated" 22 May; Uganda remains Level 2 (Practice Enhanced Precautions), "Updated" 26 May. No new outbreak-related travel notices for this event. CDC HAN-00530 unchanged. WHO PHEIC (17 May 2026) unchanged. Uganda DRC-border closure (27 May 2026) unchanged. Uganda's second death and rise to 19 confirmed are case-count changes captured in timeseries.csv / country_breakdown.csv, not declaration-schema changes. The CDC 5 June MMWR risk assessment is a publication, not a HAN advisory or travel-notice level change, so it does not alter declarations.csv.</t>
+          <t>• 2026-06-06 (scheduled run, real-time signal — BNO @BNOFeed mandatory check completed): Web's signed-in Chrome reachable via list_connected_browsers -&gt; select_browser (deviceId 5fdc215b-0b1a-4a16-9f71-01f672b11fbf). Most recent @BNOFeed Daily Ebola Update is the June 5 graphic (posted ~17h before pass): TOTAL 471 confirmed (+74) / 84 deaths (+19) / 12 recovered (+3), sourced to DRC MoH + Uganda MoH + WHO. Prior BNO graphics: June 4 = 397 conf (+19) / 65 deaths (+2) / 9 recovered (+1); June 3 = 378 conf (+19) / 63 deaths (+2). BNO's June 4 397 matched the official DRC 381 + Uganda 16 sum exactly; the June 5 471 runs ~71 cases / 18 deaths above the WHO-reconciled total (DRC MoH-attributed running wire count leading WHO reconciliation, same forward-lead pattern as June 1 and June 3). Per source-preference order (WHO DON &gt; BNO News), WHO figures win for the row; BNO running count logged for transparency. The BNO daily graphic images did not render in the browser screenshot (lazy-load); per-country suspected split from the graphic not readable this pass, but the totals (471/84) were read from the tweet text. BNO website (bnonews.com/index.php/category/health) front page still shows no fresh June Ebola article (top Ebola item is the ~1 week old 1,049-case pre-cleanup story), consistent with the ~3-day website lag vs the @BNOFeed graphic.</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-06 (scheduled run, chart constants): LAST_SITREP_STABLE_DATE unchanged at 2026-05-24 — no WHO Weekly Sitrep 03 has published; the 5 June reconciliation came via Disease Outbreak News, not a Weekly Sitrep, so all post-24-May bars remain provisional. OBSERVED_UPWARD_REVISION_RANGE unchanged ("&lt;1-35%") and OBSERVED_DOWNWARD_REVISION_RANGE unchanged ("up to 100%") — this run appended a row and applied no revisions to existing rows, so there are no new revision percentages to bracket. BASELINE_RESET_DATES unchanged — June 5 suspected held at 116 (no cleanup/reset this run).</t>
+          <t>• 2026-06-06 (scheduled run, narrative milestones): (1) CDC released three MMWRs on 5 June: a Notes from the Field report calling this the largest Bundibugyo outbreak on record (first detected among healthcare-worker clusters), a dedicated US risk assessment (risk to the general US public low; importation likelihood low; sustained US secondary transmission low), and a Center for Forecasting and Outbreak Analytics modeling report. (2) The CFA model (a planning tool, not a forecast) warns the outbreak could rival or exceed the 2014-2016 West Africa epidemic without strong intervention: &gt;20,000 cases in 2 of 3 simulations over 3 months at 20% case isolation within 2 days of symptom onset; 94% probability of staying under 10,000 cases at 70% isolation. Scenarios bracketed 50/100/200 deaths as of 24 May against 20/50/70/95% isolation. (3) Dr. Satish Pillai (CDC Ebola incident manager) said the ground situation is at the lower end of the isolation scenarios. (4) No evidence of community transmission in Kampala — all Uganda cases trace to DRC travel or to those travelers. (5) WHO and Africa CDC launched a ~$518M joint response plan; US has withdrawn from WHO (CDC declined to confirm whether US funds will flow into the WHO-led plan). (6) DRC contact tracing up from ~9% to 55% (target 90%); 4,000+ Africa CDC test kits delivered; results within 24h. (7) DRC Health Minister called US travel restrictions "discriminatory" ([Washington Times, 5 June](https://www.washingtontimes.com/news/2026/jun/5/congo-health-minister-calls-us-ebola-travel-restrictions/)). (8) US doctor infected in DRC fully recovered in Berlin (Today's News / wire).</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-06 (scheduled run, sweeper health): No stale .git/*.lock or .git/objects/*/tmp_obj_* files at session start — launchd job com.webbegole.gitlock-sweep working as designed.</t>
+          <t>• 2026-06-06 (scheduled run, declarations.csv): No change. CDC Travel Health Notices verified directly on the [CDC Travel Notices index](https://wwwnc.cdc.gov/travel/notices) (page last reviewed 4 June 2026): DRC remains Level 3 (Reconsider Nonessential Travel), "Updated" 22 May; Uganda remains Level 2 (Practice Enhanced Precautions), "Updated" 26 May. No new outbreak-related travel notices for this event. CDC HAN-00530 unchanged. WHO PHEIC (17 May 2026) unchanged. Uganda DRC-border closure (27 May 2026) unchanged. Uganda's second death and rise to 19 confirmed are case-count changes captured in timeseries.csv / country_breakdown.csv, not declaration-schema changes. The CDC 5 June MMWR risk assessment is a publication, not a HAN advisory or travel-notice level change, so it does not alter declarations.csv.</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-08 (scheduled run, catch-up after June 5 — gap covered June 6 and June 7): Appended a single 2026-06-07 row to timeseries.csv: 116 / 534 / 650 / 0 / 93. Primary source is the [BNO News @BNOFeed Daily Ebola Update June 7, 2026 graphic](https://x.com/BNOFeed) (sourced to MoH DR Congo + MoH Uganda + WHO), read via Web's signed-in Chrome: DR Congo 515 confirmed (+27) / 91 confirmed deaths (+5) / 12 recovered; Uganda 19 confirmed / 2 deaths / 4 recovered; TOTAL 534 confirmed (+27) / 93 deaths (+5) / 16 recovered. Global confirmed 534 (DRC 515 + Uganda 19), total 650 (sus 116 + conf 534), conf_deaths 93 (DRC 91 + Uganda 2), suspected 116 carried forward (no fresh official suspected figure 6-8 June; BNO tracks confirmed only), suspected_deaths 0 (column zeroed 30 May). vs 5 June (116/400/516/0/66): suspected unchanged, confirmed +134, total +134, sus_deaths unchanged, conf_deaths +27. Cumulative monotonically non-decreasing on every column; no NO_DIP exemption needed. country_breakdown.csv June 7 rows added: DRC (116/515/0/91), Uganda (19/2). Country sums tie to global on the latest date (conf 515+19=534; sus 116+0=116; conf_deaths 91+2=93; sus_deaths 0).</t>
+          <t>• 2026-06-06 (scheduled run, chart constants): LAST_SITREP_STABLE_DATE unchanged at 2026-05-24 — no WHO Weekly Sitrep 03 has published; the 5 June reconciliation came via Disease Outbreak News, not a Weekly Sitrep, so all post-24-May bars remain provisional. OBSERVED_UPWARD_REVISION_RANGE unchanged ("&lt;1-35%") and OBSERVED_DOWNWARD_REVISION_RANGE unchanged ("up to 100%") — this run appended a row and applied no revisions to existing rows, so there are no new revision percentages to bracket. BASELINE_RESET_DATES unchanged — June 5 suspected held at 116 (no cleanup/reset this run).</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-08 (scheduled run, SOURCE-TIER decision — BNO fallback adopted): No WHO Weekly Sitrep 03, no DON606, and no fresh CDC reconciliation has published for 6-8 June; the last WHO-reconciled data point remains the 5 June DON (DRC 381 conf / 64 deaths, Uganda 19/2, global 400/66, already in the tracker). WebSearch across WHO / CDC / Africa CDC / ECDC / Reuters / CIDRAP / Xinhua surfaced nothing higher-tier dated after 5 June. Per METHODOLOGY.md source-preference order, BNO News is the designated fallback "used only when nothing above is fresher" — that condition is met for 6-8 June, so the 7 June BNO @BNOFeed graphic is taken as the row source. Direct precedent: the 30-31 May rows were likewise built on BNO @BNOFeed graphics carrying DRC MoH figures when no WHO figure was fresher. CAVEAT logged for Web: BNO's DRC-attributed running count has systematically overshot the later WHO reconciliation by ~15-18% (1 Jun BNO 352 conf -&gt; WHO 330; 5 Jun BNO 471 -&gt; WHO 400). So the 7 June confirmed 534 / deaths 93 are PROVISIONAL and likely to be revised DOWN when WHO/CDC next reconcile. Under the no-dip rule, that future downward reconciliation would require the WHO+CDC two-source threshold (historically met within 1-2 days, e.g. the 1 Jun -&gt; 2 Jun reconciliation). Holding at the stale 5 June figures for 3+ days was judged worse for a daily tracker than adopting the MoH-attributed wire figure with a transparency flag.</t>
+          <t>• 2026-06-06 (scheduled run, sweeper health): No stale .git/*.lock or .git/objects/*/tmp_obj_* files at session start — launchd job com.webbegole.gitlock-sweep working as designed.</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-08 (scheduled run, date-attribution decision): No separate 2026-06-06 row. This is a catch-up after the 5 June row; 6 June and 7 June both elapsed without a run. Cumulative figures mean the 7 June graphic (534 conf) already encompasses the 6 June graphic (507 conf), so a single 7 June row carries the latest cumulative snapshot and the 6 June intermediate (DRC 488 conf / 86 deaths; Uganda 19/2; TOTAL 507 conf / 88 deaths / 13 recovered) is logged here for transparency rather than rowed. Mirrors the 2026-06-06 run's June-4-&gt;June-5 fold. The 7-day rolling-sum chart absorbs the 2-day delta (5 June -&gt; 7 June) on the 7 June date without distortion. No June 8 data point exists yet (no 8 June BNO graphic; no WHO/CDC update on 8 June at run time), so the latest row date (7 June) trails the run date (8 June), as on the 6 June run.</t>
+          <t>• 2026-06-08 (scheduled run, catch-up after June 5 — gap covered June 6 and June 7): Appended a single 2026-06-07 row to timeseries.csv: 116 / 534 / 650 / 0 / 93. Primary source is the [BNO News @BNOFeed Daily Ebola Update June 7, 2026 graphic](https://x.com/BNOFeed) (sourced to MoH DR Congo + MoH Uganda + WHO), read via Web's signed-in Chrome: DR Congo 515 confirmed (+27) / 91 confirmed deaths (+5) / 12 recovered; Uganda 19 confirmed / 2 deaths / 4 recovered; TOTAL 534 confirmed (+27) / 93 deaths (+5) / 16 recovered. Global confirmed 534 (DRC 515 + Uganda 19), total 650 (sus 116 + conf 534), conf_deaths 93 (DRC 91 + Uganda 2), suspected 116 carried forward (no fresh official suspected figure 6-8 June; BNO tracks confirmed only), suspected_deaths 0 (column zeroed 30 May). vs 5 June (116/400/516/0/66): suspected unchanged, confirmed +134, total +134, sus_deaths unchanged, conf_deaths +27. Cumulative monotonically non-decreasing on every column; no NO_DIP exemption needed. country_breakdown.csv June 7 rows added: DRC (116/515/0/91), Uganda (19/2). Country sums tie to global on the latest date (conf 515+19=534; sus 116+0=116; conf_deaths 91+2=93; sus_deaths 0).</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-08 (scheduled run, 3-day lookback: June 2, June 3, June 5): No revisions required. No higher-tier source published after 5 June, so nothing supersedes the existing rows. The BNO 6/7 June graphics are forward-dated data points, not revisions of prior rows. June 5 row holds at the WHO DON "as of 5 June" figures (DRC 381/64, Uganda 19/2).</t>
+          <t>• 2026-06-08 (scheduled run, SOURCE-TIER decision — BNO fallback adopted): No WHO Weekly Sitrep 03, no DON606, and no fresh CDC reconciliation has published for 6-8 June; the last WHO-reconciled data point remains the 5 June DON (DRC 381 conf / 64 deaths, Uganda 19/2, global 400/66, already in the tracker). WebSearch across WHO / CDC / Africa CDC / ECDC / Reuters / CIDRAP / Xinhua surfaced nothing higher-tier dated after 5 June. Per METHODOLOGY.md source-preference order, BNO News is the designated fallback "used only when nothing above is fresher" — that condition is met for 6-8 June, so the 7 June BNO @BNOFeed graphic is taken as the row source. Direct precedent: the 30-31 May rows were likewise built on BNO @BNOFeed graphics carrying DRC MoH figures when no WHO figure was fresher. CAVEAT logged for Web: BNO's DRC-attributed running count has systematically overshot the later WHO reconciliation by ~15-18% (1 Jun BNO 352 conf -&gt; WHO 330; 5 Jun BNO 471 -&gt; WHO 400). So the 7 June confirmed 534 / deaths 93 are PROVISIONAL and likely to be revised DOWN when WHO/CDC next reconcile. Under the no-dip rule, that future downward reconciliation would require the WHO+CDC two-source threshold (historically met within 1-2 days, e.g. the 1 Jun -&gt; 2 Jun reconciliation). Holding at the stale 5 June figures for 3+ days was judged worse for a daily tracker than adopting the MoH-attributed wire figure with a transparency flag.</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-08 (scheduled run, real-time signal — BNO @BNOFeed mandatory check completed): Web's signed-in Chrome reachable via list_connected_browsers -&gt; select_browser (deviceId 5fdc215b-0b1a-4a16-9f71-01f672b11fbf). Most recent @BNOFeed Daily Ebola Update is the 7 June graphic (posted ~13h before pass): DR Congo 515 conf (+27) / 91 deaths (+5) / 12 recovered; Uganda 19 / 2 / 4; TOTAL 534 conf (+27) / 93 deaths (+5) / 16 recovered; "23 days since first case"; sourced to MoH DR Congo + MoH Uganda + WHO. Prior BNO graphics: 6 June = 507 conf (+36) / 88 deaths (+4) / 13 recovered (DRC 488 / 86; Uganda 19/2); 5 June = 471 conf / 84 deaths / 12 recovered. Graphic figures read directly from the rendered tweet image (zoom) this pass — per-country splits legible, unlike the 6 June run's lazy-load miss. BNO website (bnonews.com/index.php/category/health) front page still shows no fresh June Ebola article (top Ebola item is the ~1-week-old 1,049-case pre-cleanup story), consistent with the ~3-day website lag vs the @BNOFeed graphic. Credentialed x.com scan: no WHO/CDC/Reuters/AP/AFP figure dated after 5 June supersedes the BNO graphic; WHO has been silent on global figures since the 5 June DON.</t>
+          <t>• 2026-06-08 (scheduled run, date-attribution decision): No separate 2026-06-06 row. This is a catch-up after the 5 June row; 6 June and 7 June both elapsed without a run. Cumulative figures mean the 7 June graphic (534 conf) already encompasses the 6 June graphic (507 conf), so a single 7 June row carries the latest cumulative snapshot and the 6 June intermediate (DRC 488 conf / 86 deaths; Uganda 19/2; TOTAL 507 conf / 88 deaths / 13 recovered) is logged here for transparency rather than rowed. Mirrors the 2026-06-06 run's June-4-&gt;June-5 fold. The 7-day rolling-sum chart absorbs the 2-day delta (5 June -&gt; 7 June) on the 7 June date without distortion. No June 8 data point exists yet (no 8 June BNO graphic; no WHO/CDC update on 8 June at run time), so the latest row date (7 June) trails the run date (8 June), as on the 6 June run.</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-08 (scheduled run, declarations.csv): No change. CDC Travel Health Notices verified directly on the per-country pages via Chrome: DRC remains [Level 3 - Reconsider Nonessential Travel](https://wwwnc.cdc.gov/travel/notices/level3/ebola-democratic-republic-of-the-congo), page last reviewed 22 May 2026; Uganda remains [Level 2 - Practice Enhanced Precautions](https://wwwnc.cdc.gov/travel/notices/level2/ebola-uganda), page last reviewed 26 May 2026. METHODOLOGY note for Web: a web_fetch of the CDC Travel Notices index (https://wwwnc.cdc.gov/travel/notices) returned a STALE/partial cache this run — it listed "no Travel Health Notices" at Level 3 and omitted the Ebola DRC/Uganda notices entirely. The per-country pages (authoritative, checked directly per the verification protocol) confirm both levels are unchanged and live, so the index render is a caching artifact, not a real delisting. CDC HAN-00530 unchanged. WHO PHEIC (17 May 2026) unchanged. Uganda DRC-border closure (27 May 2026) unchanged.</t>
+          <t>• 2026-06-08 (scheduled run, 3-day lookback: June 2, June 3, June 5): No revisions required. No higher-tier source published after 5 June, so nothing supersedes the existing rows. The BNO 6/7 June graphics are forward-dated data points, not revisions of prior rows. June 5 row holds at the WHO DON "as of 5 June" figures (DRC 381/64, Uganda 19/2).</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-08 (scheduled run, chart constants): LAST_SITREP_STABLE_DATE unchanged at 2026-05-24 — still no WHO Weekly Sitrep 03; the 7 June row is BNO-sourced and provisional, so all post-24-May bars remain hatched. OBSERVED_UPWARD_REVISION_RANGE and OBSERVED_DOWNWARD_REVISION_RANGE unchanged — this run appended a row and applied no revisions to existing rows, so there are no new revision percentages to bracket. BASELINE_RESET_DATES unchanged (no cleanup/reset this run; suspected held at 116).</t>
+          <t>• 2026-06-08 (scheduled run, real-time signal — BNO @BNOFeed mandatory check completed): Web's signed-in Chrome reachable via list_connected_browsers -&gt; select_browser (deviceId 5fdc215b-0b1a-4a16-9f71-01f672b11fbf). Most recent @BNOFeed Daily Ebola Update is the 7 June graphic (posted ~13h before pass): DR Congo 515 conf (+27) / 91 deaths (+5) / 12 recovered; Uganda 19 / 2 / 4; TOTAL 534 conf (+27) / 93 deaths (+5) / 16 recovered; "23 days since first case"; sourced to MoH DR Congo + MoH Uganda + WHO. Prior BNO graphics: 6 June = 507 conf (+36) / 88 deaths (+4) / 13 recovered (DRC 488 / 86; Uganda 19/2); 5 June = 471 conf / 84 deaths / 12 recovered. Graphic figures read directly from the rendered tweet image (zoom) this pass — per-country splits legible, unlike the 6 June run's lazy-load miss. BNO website (bnonews.com/index.php/category/health) front page still shows no fresh June Ebola article (top Ebola item is the ~1-week-old 1,049-case pre-cleanup story), consistent with the ~3-day website lag vs the @BNOFeed graphic. Credentialed x.com scan: no WHO/CDC/Reuters/AP/AFP figure dated after 5 June supersedes the BNO graphic; WHO has been silent on global figures since the 5 June DON.</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" s="9" t="inlineStr">
         <is>
-          <t>• 2026-06-08 (scheduled run, story.md): "Latest update" refreshed to lead with the 7 June BNO-sourced provisional snapshot (global 534 confirmed / 116 suspected / 93 confirmed deaths; DRC 515/91; Uganda 19/2), explicitly framed as a DRC MoH + Uganda MoH attributed running wire count that WHO has not yet reconciled (WHO silent since the 5 June DON), with the ~15-18% BNO-overshoot caveat and the provisional-bars note. "Story so far" unchanged.</t>
+          <t>• 2026-06-08 (scheduled run, declarations.csv): No change. CDC Travel Health Notices verified directly on the per-country pages via Chrome: DRC remains [Level 3 - Reconsider Nonessential Travel](https://wwwnc.cdc.gov/travel/notices/level3/ebola-democratic-republic-of-the-congo), page last reviewed 22 May 2026; Uganda remains [Level 2 - Practice Enhanced Precautions](https://wwwnc.cdc.gov/travel/notices/level2/ebola-uganda), page last reviewed 26 May 2026. METHODOLOGY note for Web: a web_fetch of the CDC Travel Notices index (https://wwwnc.cdc.gov/travel/notices) returned a STALE/partial cache this run — it listed "no Travel Health Notices" at Level 3 and omitted the Ebola DRC/Uganda notices entirely. The per-country pages (authoritative, checked directly per the verification protocol) confirm both levels are unchanged and live, so the index render is a caching artifact, not a real delisting. CDC HAN-00530 unchanged. WHO PHEIC (17 May 2026) unchanged. Uganda DRC-border closure (27 May 2026) unchanged.</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" s="9" t="inlineStr">
         <is>
+          <t>• 2026-06-08 (scheduled run, chart constants): LAST_SITREP_STABLE_DATE unchanged at 2026-05-24 — still no WHO Weekly Sitrep 03; the 7 June row is BNO-sourced and provisional, so all post-24-May bars remain hatched. OBSERVED_UPWARD_REVISION_RANGE and OBSERVED_DOWNWARD_REVISION_RANGE unchanged — this run appended a row and applied no revisions to existing rows, so there are no new revision percentages to bracket. BASELINE_RESET_DATES unchanged (no cleanup/reset this run; suspected held at 116).</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="9" t="inlineStr">
+        <is>
+          <t>• 2026-06-08 (scheduled run, story.md): "Latest update" refreshed to lead with the 7 June BNO-sourced provisional snapshot (global 534 confirmed / 116 suspected / 93 confirmed deaths; DRC 515/91; Uganda 19/2), explicitly framed as a DRC MoH + Uganda MoH attributed running wire count that WHO has not yet reconciled (WHO silent since the 5 June DON), with the ~15-18% BNO-overshoot caveat and the provisional-bars note. "Story so far" unchanged.</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="9" t="inlineStr">
+        <is>
           <t>• 2026-06-08 (scheduled run, sweeper health): No stale .git/*.lock or .git/objects/*/tmp_obj_* files at session start — launchd job com.webbegole.gitlock-sweep working as designed.</t>
         </is>
       </c>
     </row>
+    <row r="194">
+      <c r="A194" s="9" t="inlineStr">
+        <is>
+          <t>• 2026-06-08 (scheduled run, BACKFILL of missed days June 4 and June 6 per Web's request + new daily-row policy): Inserted two mid-history rows so the series carries one row per calendar day (May 31 -&gt; June 7 now complete). (1) 2026-06-04: 116 / 397 / 513 / 0 / 65, source [BNO @BNOFeed June 4 graphic](https://x.com/BNOFeed) read directly via Chrome (DR Congo 381 conf (+18) / 64 deaths (+2) / 7 recovered; Uganda 16 conf (+1) / 1 death / 2 recovered; TOTAL 397 / 65 / 9). DRC 381/64 matches the WHO DON "as of 5 June" reconciled DRC figure (as of 3 June, published 4 June), so the DRC component is WHO-corroborated; Uganda 16/1 per Uganda MoH via Xinhua. country_breakdown June 4 rows added: DRC 116/381/0/64, Uganda 16/1. (2) 2026-06-06: 116 / 507 / 623 / 0 / 88, source [BNO @BNOFeed June 6 graphic](https://x.com/BNOFeed) read directly via Chrome (DR Congo 488 conf (+36) / 86 deaths (+4) / 9 recovered; Uganda 19 / 2 / 4; TOTAL 507 / 88 / 13). country_breakdown June 6 rows added: DRC 116/488/0/86, Uganda 19/2. Both are DRC MoH-attributed BNO running counts (June 6 488 DRC overshoots the WHO-reconciled instrument; the +107 confirmed vs June 5's WHO-reconciled 381 is mostly the BNO-vs-WHO gap, not one day of incidence) and carry the standard ~15-18% downward-reconciliation risk. Series stays monotonic after insertion: confirmed 359(6/3) &lt;= 397(6/4) &lt;= 400(6/5) &lt;= 507(6/6) &lt;= 534(6/7); conf_deaths 61 &lt;= 65 &lt;= 66 &lt;= 88 &lt;= 93; total 475 &lt;= 513 &lt;= 516 &lt;= 623 &lt;= 650. No-dip holds; no exemption needed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="9" t="inlineStr">
+        <is>
+          <t>• 2026-06-08 (scheduled run, gap existed because): the 4 June scheduled run did not fire (laptop offline) and the 6 June run folded 4 June into the 5 June "as of" row; the 6 June date was likewise folded into the 7 June row by today's earlier pass. Both are now backfilled. The fold convention is retired for routine gaps in favour of one row per day.</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="9" t="inlineStr">
+        <is>
+          <t>• 2026-06-08 (scheduled run, METHODOLOGY.md change): added a "Backfilling missed days" section (one-row-per-day target; gap-detection procedure; BNO daily graphic as primary backfill source; chronological insertion as the single sanctioned mid-history insertion; backfilled-BNO rows carry the same provisional/downward-reconciliation status). Amended the "Rules" section: mid-history insertion is now permitted solely to backfill a missed calendar date (existing rows still never re-sequenced or rewritten outside lookback).</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="9" t="inlineStr">
+        <is>
+          <t>• 2026-06-08 (scheduled run, SKILL.md change): added a "GAP DETECTION / BACKFILL" step to the scheduled task (run before appending today's row): detect every un-rowed calendar date since the last row, source each from its BNO @BNOFeed daily graphic (WHO/CDC reconciled figures preferred where they cover the date), insert in chronological position, flag primary_source with "BACKFILL (...)", and log per-date sources. Also corrected the timeseries schema note in SKILL.md from "7 columns" to the actual 8 (added confirmed_deaths_global). NOTE FOR WEB: the live scheduled-task definition points at the uploaded SKILL.md copy; this edit is to the project-folder SKILL.md, so the scheduled task may need re-pointing or re-uploading to pick up the new backfill step.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="165">
+  <mergeCells count="169">
     <mergeCell ref="A130:H130"/>
     <mergeCell ref="A77:H77"/>
     <mergeCell ref="A83:H83"/>
@@ -2418,6 +2510,7 @@
     <mergeCell ref="A110:H110"/>
     <mergeCell ref="A119:H119"/>
     <mergeCell ref="A69:H69"/>
+    <mergeCell ref="A196:H196"/>
     <mergeCell ref="A174:H174"/>
     <mergeCell ref="A183:H183"/>
     <mergeCell ref="A66:H66"/>
@@ -2438,7 +2531,6 @@
     <mergeCell ref="A159:H159"/>
     <mergeCell ref="A97:H97"/>
     <mergeCell ref="A106:H106"/>
-    <mergeCell ref="A29:H29"/>
     <mergeCell ref="A134:H134"/>
     <mergeCell ref="A81:H81"/>
     <mergeCell ref="A38:H38"/>
@@ -2459,6 +2551,7 @@
     <mergeCell ref="A82:H82"/>
     <mergeCell ref="A60:H60"/>
     <mergeCell ref="A123:H123"/>
+    <mergeCell ref="A197:H197"/>
     <mergeCell ref="A146:H146"/>
     <mergeCell ref="A124:H124"/>
     <mergeCell ref="A172:H172"/>
@@ -2489,7 +2582,6 @@
     <mergeCell ref="A167:H167"/>
     <mergeCell ref="A48:H48"/>
     <mergeCell ref="A176:H176"/>
-    <mergeCell ref="A30:H30"/>
     <mergeCell ref="A114:H114"/>
     <mergeCell ref="A59:H59"/>
     <mergeCell ref="A182:H182"/>
@@ -2518,6 +2610,7 @@
     <mergeCell ref="A179:H179"/>
     <mergeCell ref="A71:H71"/>
     <mergeCell ref="A129:H129"/>
+    <mergeCell ref="A195:H195"/>
     <mergeCell ref="A76:H76"/>
     <mergeCell ref="A33:H33"/>
     <mergeCell ref="A116:H116"/>
@@ -2551,16 +2644,19 @@
     <mergeCell ref="A87:H87"/>
     <mergeCell ref="A65:H65"/>
     <mergeCell ref="A128:H128"/>
+    <mergeCell ref="A193:H193"/>
     <mergeCell ref="A80:H80"/>
+    <mergeCell ref="A46:H46"/>
     <mergeCell ref="A37:H37"/>
-    <mergeCell ref="A46:H46"/>
     <mergeCell ref="A89:H89"/>
     <mergeCell ref="A120:H120"/>
     <mergeCell ref="A136:H136"/>
+    <mergeCell ref="A192:H192"/>
     <mergeCell ref="A105:H105"/>
     <mergeCell ref="A57:H57"/>
     <mergeCell ref="A113:H113"/>
     <mergeCell ref="A185:H185"/>
+    <mergeCell ref="A194:H194"/>
     <mergeCell ref="A181:H181"/>
     <mergeCell ref="A91:H91"/>
     <mergeCell ref="A147:H147"/>
@@ -2583,7 +2679,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:J28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3347,32 +3443,32 @@
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B25" s="4" t="n">
         <v>0</v>
       </c>
       <c r="C25" s="4" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D25" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E25" s="4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F25" s="4" t="n">
         <v>-790</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="H25" s="4" t="n">
         <v>-223</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J25" s="4" t="n">
         <v>7</v>
@@ -3381,34 +3477,102 @@
     <row r="26">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B26" s="6" t="n">
         <v>0</v>
       </c>
       <c r="C26" s="6" t="n">
-        <v>134</v>
+        <v>3</v>
       </c>
       <c r="D26" s="6" t="n">
         <v>0</v>
       </c>
       <c r="E26" s="6" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="F26" s="6" t="n">
         <v>-790</v>
       </c>
       <c r="G26" s="6" t="n">
-        <v>400</v>
+        <v>266</v>
       </c>
       <c r="H26" s="6" t="n">
         <v>-223</v>
       </c>
       <c r="I26" s="6" t="n">
-        <v>75</v>
+        <v>48</v>
       </c>
       <c r="J26" s="6" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C27" s="4" t="n">
+        <v>107</v>
+      </c>
+      <c r="D27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="4" t="n">
+        <v>22</v>
+      </c>
+      <c r="F27" s="4" t="n">
+        <v>-233</v>
+      </c>
+      <c r="G27" s="4" t="n">
+        <v>273</v>
+      </c>
+      <c r="H27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="I27" s="4" t="n">
+        <v>70</v>
+      </c>
+      <c r="J27" s="4" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C28" s="6" t="n">
+        <v>27</v>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="6" t="n">
+        <v>5</v>
+      </c>
+      <c r="F28" s="6" t="n">
+        <v>-331</v>
+      </c>
+      <c r="G28" s="6" t="n">
+        <v>300</v>
+      </c>
+      <c r="H28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I28" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="J28" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -3427,7 +3591,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H48"/>
+  <dimension ref="A1:H52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4761,7 +4925,7 @@
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B45" s="4" t="inlineStr">
@@ -4783,19 +4947,19 @@
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>[WHO Disease Outbreak News, as of 5 June 2026] + DRC MoH via Health Minister Roger Kamba press briefing 4 June (https://english.news.cn/africa/20260605/75381cda9c1642f7acfdaac060a5bf0f/c.html): DRC 381 confirmed / 64 confirmed deaths (WHO DON; Kamba/Xinhua said 63, WHO figure used per source-preference) / 116 suspected (carried from 3 June, no fresh official suspected figure) / 0 suspected_deaths (column zeroed 30 May). 233 hospitalised in isolation as of 3 June. Geographic: Ituri 359 conf / 17 health zones; North Kivu 19 conf / 7 health zones; South Kivu 3 conf / 1 health zone (359+19+3=381). Testing capacity ramped: 4,000+ Africa CDC kits, nearly all samples tested with results within 24h; contact tracing up from ~9% to 55% (target 90%). vs June 3 (116/344/0/60): suspected unchanged, confirmed +37, conf_deaths +4. SOURCE-VIEW DIVERGENCE: BNO @BNOFeed June 5 graphic running DRC-attributed total ~471 conf / 84 deaths leads WHO reconciliation; WHO DON source-preference holds.</t>
+          <t>BACKFILL (added 2026-06-08 run): [BNO @BNOFeed June 4, 2026 graphic](https://x.com/BNOFeed) (MoH DR Congo + MoH Uganda + WHO): DR Congo 381 confirmed (+18) / 64 deaths (+2) / 7 recovered. DRC 381/64 matches the WHO DON 'as of 5 June' reconciled DRC figure (as of 3 June, published 4 June), so WHO-corroborated. suspected 116 carried from 3 June; suspected_deaths 0 (column zeroed 30 May). vs 3 June (116/344/0/60): confirmed +37, conf_deaths +4. Backfilled: 4 June run did not fire (laptop offline).</t>
         </is>
       </c>
       <c r="H45" s="5" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B46" s="6" t="inlineStr">
@@ -4805,27 +4969,27 @@
       </c>
       <c r="C46" s="6" t="n"/>
       <c r="D46" s="6" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="E46" s="6" t="n"/>
       <c r="F46" s="6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G46" s="7" t="inlineStr">
         <is>
-          <t>[WHO Disease Outbreak News, as of 5 June 2026]: Uganda 19 confirmed / 2 deaths. Three new cases reported 5 June were contacts of confirmed cases. Of 9 geolocated cases, 8 in Kampala and 1 in Wakiso. Uganda does not report suspected cases. Progression: 15 (June 2-3) -&gt; 16 (June 4, +1 new confirmed Thursday per Uganda MoH via Xinhua) -&gt; 19 (June 5, +3 contacts). Second Uganda death recorded as of 5 June (was 1 death June 2-3); deaths now 2. vs June 3 (15 conf / 1 death): confirmed +4, deaths +1.</t>
+          <t>BACKFILL (added 2026-06-08 run): [BNO @BNOFeed June 4, 2026 graphic](https://x.com/BNOFeed) + Uganda MoH via Xinhua: Uganda 16 confirmed (+1 new confirmed Thursday 4 June) / 1 death / 2 recovered. Uganda does not report suspected cases. vs 3 June (15/1): confirmed +1, deaths unchanged. Second Uganda death lands on the 5 June row (1 -&gt; 2).</t>
         </is>
       </c>
       <c r="H46" s="7" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-04</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B47" s="4" t="inlineStr">
@@ -4837,29 +5001,29 @@
         <v>116</v>
       </c>
       <c r="D47" s="4" t="n">
-        <v>515</v>
+        <v>381</v>
       </c>
       <c r="E47" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F47" s="4" t="n">
-        <v>91</v>
+        <v>64</v>
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>[BNO News @BNOFeed Daily Ebola Update June 7, 2026 graphic](https://x.com/BNOFeed) (MoH DR Congo + MoH Uganda + WHO): DR Congo 515 confirmed (+27 vs 6 June's 488) / 91 confirmed deaths (+5) / 12 recovered. suspected 116 carried forward (5 June WHO DON cleaned baseline; BNO tracks confirmed only); suspected_deaths 0 (column zeroed 30 May). vs 5 June (116/381/0/64): suspected unchanged, confirmed +134, conf_deaths +27. SOURCE-VIEW / TIER FLAG: DRC MoH-attributed running wire count; no WHO/CDC reconciliation for 6-8 June, last WHO-reconciled DRC point is the 5 June DON (381/64). BNO running counts historically overshoot WHO reconciliation by ~15-18%, so the 515 confirmed is provisional and likely revised DOWN at the next WHO/CDC reconciliation. 6 June intermediate: DRC 488 conf / 86 deaths.</t>
+          <t>[WHO Disease Outbreak News, as of 5 June 2026] + DRC MoH via Health Minister Roger Kamba press briefing 4 June (https://english.news.cn/africa/20260605/75381cda9c1642f7acfdaac060a5bf0f/c.html): DRC 381 confirmed / 64 confirmed deaths (WHO DON; Kamba/Xinhua said 63, WHO figure used per source-preference) / 116 suspected (carried from 3 June, no fresh official suspected figure) / 0 suspected_deaths (column zeroed 30 May). 233 hospitalised in isolation as of 3 June. Geographic: Ituri 359 conf / 17 health zones; North Kivu 19 conf / 7 health zones; South Kivu 3 conf / 1 health zone (359+19+3=381). Testing capacity ramped: 4,000+ Africa CDC kits, nearly all samples tested with results within 24h; contact tracing up from ~9% to 55% (target 90%). vs June 3 (116/344/0/60): suspected unchanged, confirmed +37, conf_deaths +4. SOURCE-VIEW DIVERGENCE: BNO @BNOFeed June 5 graphic running DRC-attributed total ~471 conf / 84 deaths leads WHO reconciliation; WHO DON source-preference holds.</t>
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-05</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
-          <t>2026-06-07</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B48" s="6" t="inlineStr">
@@ -4877,10 +5041,138 @@
       </c>
       <c r="G48" s="7" t="inlineStr">
         <is>
+          <t>[WHO Disease Outbreak News, as of 5 June 2026]: Uganda 19 confirmed / 2 deaths. Three new cases reported 5 June were contacts of confirmed cases. Of 9 geolocated cases, 8 in Kampala and 1 in Wakiso. Uganda does not report suspected cases. Progression: 15 (June 2-3) -&gt; 16 (June 4, +1 new confirmed Thursday per Uganda MoH via Xinhua) -&gt; 19 (June 5, +3 contacts). Second Uganda death recorded as of 5 June (was 1 death June 2-3); deaths now 2. vs June 3 (15 conf / 1 death): confirmed +4, deaths +1.</t>
+        </is>
+      </c>
+      <c r="H48" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B49" s="4" t="inlineStr">
+        <is>
+          <t>DRC</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="n">
+        <v>116</v>
+      </c>
+      <c r="D49" s="4" t="n">
+        <v>488</v>
+      </c>
+      <c r="E49" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F49" s="4" t="n">
+        <v>86</v>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>BACKFILL (added 2026-06-08 run): [BNO @BNOFeed June 6, 2026 graphic](https://x.com/BNOFeed) (MoH DR Congo + MoH Uganda + WHO): DR Congo 488 confirmed (+36) / 86 deaths (+4) / 9 recovered. suspected 116 carried; suspected_deaths 0 (column zeroed 30 May). vs 5 June (116/381/0/64): confirmed +107, conf_deaths +22. SOURCE-VIEW / TIER FLAG: DRC MoH-attributed running wire count; the +107 vs 5 June is mostly the BNO-vs-WHO instrument gap (5 June WHO-reconciled DRC 381 vs 6 June BNO running DRC 488), not one day of incidence. BNO overshoots WHO ~15-18%, so 488 is provisional. Backfilled: 6 June folded into the 7 June row.</t>
+        </is>
+      </c>
+      <c r="H49" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+      <c r="B50" s="6" t="inlineStr">
+        <is>
+          <t>Uganda</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="n"/>
+      <c r="D50" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="E50" s="6" t="n"/>
+      <c r="F50" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G50" s="7" t="inlineStr">
+        <is>
+          <t>BACKFILL (added 2026-06-08 run): [BNO @BNOFeed June 6, 2026 graphic](https://x.com/BNOFeed): Uganda 19 confirmed / 2 deaths / 4 recovered. Unchanged from 5 June (19/2). Uganda does not report suspected cases.</t>
+        </is>
+      </c>
+      <c r="H50" s="7" t="inlineStr">
+        <is>
+          <t>2026-06-06</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B51" s="4" t="inlineStr">
+        <is>
+          <t>DRC</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="n">
+        <v>116</v>
+      </c>
+      <c r="D51" s="4" t="n">
+        <v>515</v>
+      </c>
+      <c r="E51" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F51" s="4" t="n">
+        <v>91</v>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>[BNO News @BNOFeed Daily Ebola Update June 7, 2026 graphic](https://x.com/BNOFeed) (MoH DR Congo + MoH Uganda + WHO): DR Congo 515 confirmed (+27 vs 6 June's 488) / 91 confirmed deaths (+5) / 12 recovered. suspected 116 carried forward (5 June WHO DON cleaned baseline; BNO tracks confirmed only); suspected_deaths 0 (column zeroed 30 May). vs 5 June (116/381/0/64): suspected unchanged, confirmed +134, conf_deaths +27. SOURCE-VIEW / TIER FLAG: DRC MoH-attributed running wire count; no WHO/CDC reconciliation for 6-8 June, last WHO-reconciled DRC point is the 5 June DON (381/64). BNO running counts historically overshoot WHO reconciliation by ~15-18%, so the 515 confirmed is provisional and likely revised DOWN at the next WHO/CDC reconciliation. 6 June intermediate: DRC 488 conf / 86 deaths.</t>
+        </is>
+      </c>
+      <c r="H51" s="5" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-07</t>
+        </is>
+      </c>
+      <c r="B52" s="6" t="inlineStr">
+        <is>
+          <t>Uganda</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="n"/>
+      <c r="D52" s="6" t="n">
+        <v>19</v>
+      </c>
+      <c r="E52" s="6" t="n"/>
+      <c r="F52" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="G52" s="7" t="inlineStr">
+        <is>
           <t>[BNO News @BNOFeed Daily Ebola Update June 7, 2026 graphic](https://x.com/BNOFeed) (MoH DR Congo + MoH Uganda + WHO): Uganda 19 confirmed (unchanged from 5 June) / 2 deaths / 4 recovered. Uganda does not report suspected cases. No change vs 5 June (19/2); Uganda has held at 19 conf / 2 deaths across the 6 and 7 June BNO graphics.</t>
         </is>
       </c>
-      <c r="H48" s="7" t="inlineStr">
+      <c r="H52" s="7" t="inlineStr">
         <is>
           <t>2026-06-07</t>
         </is>

</xml_diff>

<commit_message>
Reconcile May 31 to WHO Sitrep 03 (DRC 321/48); advance provisional boundary to 31 May; widen upward-revision range to 43%
</commit_message>
<xml_diff>
--- a/outputs/ebola_timeseries.xlsx
+++ b/outputs/ebola_timeseries.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H197"/>
+  <dimension ref="A1:H201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1072,23 +1072,23 @@
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>447</v>
+        <v>116</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>234</v>
+        <v>330</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>681</v>
+        <v>446</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>REVISED 2026-06-01 (scheduled run): confirmed_deaths_global corrected from 56 to 43 (DRC conf_deaths 55→42, Uganda unchanged at 1) per [BNO @BNOFeed Daily Ebola Update June 1, 2026 graphic](https://x.com/BNOFeed/status/2061573338569351279) (sourced to MoH DR Congo + MoH Uganda + WHO), which shows DRC June 1 conf_deaths = 48 with +6 delta, implying yesterday's = 42. Corroborated by DRC MoH 31 May situation report (per multiple wire summaries June 1: "DRC Ministry of Health published updated figures reporting a total of 282 confirmed cases, including 42 confirmed related deaths and 220 suspected cases that are under investigation"). The prior 55 DRC conf_deaths in this row was an inference (+38 attributed from BNO May 31 graphic's "55 deaths" total interpreted as conf_deaths post-May-30 cleanup); DRC MoH's formal 31 May situation report puts the true confirmed-deaths figure at 42. Same-row correction; not a no-dip dip vs May 30's 18. PRIOR REVISION 2026-05-31 (PM): MoH methodology-change carve-out applied per METHODOLOGY.md; new baseline rolls forward from the revised May 30 row. BNO @BNOFeed Daily Ebola Update May 31 graphic reports DRC running on the cleaned baseline: DR Congo 672 cases (+98 from May 30) / 55 deaths (+38 from May 30); Uganda 9 conf / 1 death (unchanged); TOTAL 681 (+98) / 56 (+38). Sus/conf split inference: DRC confirmed carries forward at DRC MoH's running 225; DRC suspected = 672 - 225 = 447; DRC sus_deaths stays at 0 (column zeroed May 30 carries forward). Global vs May 30: sus 349→447 (+98), conf 234 (unchanged), total 583→681 (+98), sus_deaths 0 (unchanged). Global vs prior WHO DON605 carry-forward (906/134/1040/223): sus -50.66%, conf +74.63%, total -34.52%, sus_deaths -100%. [Joint statement by the Government of the DRC and WHO, 31 May 2026](https://www.who.int/news/item/31-05-2026-joint-statement-by-the-government-of-the-democratic-republic-of-the-congo-and-who-concerning-the-outbreak-of-ebola-disease-caused-by-the-bundibugyo-virus) closing the Tedros / Kamba / Muyaya Bunia mission is qualitative (no global figures): commits to "rapidly undertake randomized control trials on candidate vaccines and treatments"; explicit call that "borders remain open."</t>
+          <t>REVISED 2026-06-08 (Web-directed, WHO Weekly Sitrep 03 reconciliation): [WHO Weekly External Situation Report 03, data as of 31 May 2026](https://www.afro.who.int/health-topics/ebola-disease/outbreak-drc-26) is the gold-standard reconciled source for this date and was missed by the runs through 2026-06-08 (the AFRO Situation Reports list is JS-rendered; prior runs checked the DON page + CDC + BNO wire and wrongly logged 'no Sitrep 03 yet'). Sitrep 03 summary: DRC 321 confirmed / 48 confirmed deaths / 0 probable / 15.0% CFR (confirmed+probable framing; no suspected column). Reconciled May 31 to the Sitrep: DRC suspected 447-&gt;116 (the cleaned-baseline suspected level WHO carries from ~29-31 May; the 447 BNO running count is superseded), confirmed 225-&gt;321 (+42.7%), conf_deaths 42-&gt;48; Uganda unchanged 9 conf / 1 death. Global: suspected 447-&gt;116, confirmed 234-&gt;330 (+41.0%), total 681-&gt;446 (-34.5%), suspected_deaths 0 (unchanged), confirmed_deaths 43-&gt;49. This pulls the DRC MoH cleanup onto its true Sitrep date, so May 31 now matches the June 1 post-cleanup state. Per METHODOLOGY source-preference order, WHO Weekly Sitrep is source #1 and supersedes the wire counts previously carried. no-dip: the suspected/total drops vs May 30 are the MoH methodology-change cleanup (carve-out); NO_DIP_EXEMPTIONS_TIMESERIES gains 2026-05-31 -&gt; {suspected_global, total_global} and BASELINE_RESET_DATES gains 2026-05-31. PRIOR (superseded) primary_source: confirmed_deaths corrected 56-&gt;43 on 2026-06-01 per BNO June 1 graphic; May 31 BNO cleaned-baseline running count DR Congo 672 cases / 55 deaths, split DRC conf 225 / sus 447. See notes.md 2026-06-08 Sitrep-03 bullet.</t>
         </is>
       </c>
       <c r="H21" s="5" t="inlineStr">
@@ -2497,12 +2497,41 @@
         </is>
       </c>
     </row>
+    <row r="198">
+      <c r="A198" s="9" t="inlineStr">
+        <is>
+          <t>• 2026-06-08 (Web-directed, WHO Weekly Sitrep 03 DISCOVERY + reconciliation): Web spotted [WHO Weekly External Situation Report 03, data as of 31 May 2026](https://www.afro.who.int/health-topics/ebola-disease/outbreak-drc-26) on the AFRO outbreak page. The runs through 2026-06-08 MISSED it and repeatedly logged "no Sitrep 03 yet" — root cause: the AFRO "Situation Reports" list is JS-rendered, and the runs checked the WHO DON page + CDC + BNO wire (plus a plain web_fetch of the AFRO page that returns an empty shell for that section). There are in fact three sitreps: 01 (as of 18 May), 02 (as of 24 May), 03 (as of 31 May). Sitrep 03 summary table: DRC 321 confirmed / 48 confirmed deaths / 0 probable / total 321 / 15.0% CFR (WHO uses a confirmed+probable framing, no suspected column). Confirmed via Chrome render of the AFRO page (deviceId 5fdc215b-0b1a-4a16-9f71-01f672b11fbf).</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="9" t="inlineStr">
+        <is>
+          <t>• 2026-06-08 (Web-directed, May 31 row reconciled to Sitrep 03): WHO Weekly Sitrep is source #1 (gold standard) and supersedes the wire counts the May 31 row carried. Revised timeseries 2026-05-31: suspected 447-&gt;116, confirmed 234-&gt;330 (+41.0%), total 681-&gt;446 (-34.5%), suspected_deaths 0 (unchanged), confirmed_deaths 43-&gt;49. country_breakdown 2026-05-31 DRC: suspected 447-&gt;116, confirmed 225-&gt;321 (+42.7%), conf_deaths 42-&gt;48 (Sitrep 03 DRC figures); Uganda unchanged 9/1. The reconciliation pulls the DRC MoH cleanup onto its true Sitrep date, so the revised May 31 row now equals the June 1 post-cleanup state (116/330/446/0/49). Monotonicity holds: May 30 (349/234/583/0/18) -&gt; May 31 (116/330/446/0/49) -&gt; June 1 (116/330/446/0/49); the suspected/total drops vs May 30 are the MoH methodology-change cleanup (carve-out). Note: this is a revision OUTSIDE the standard 3-day lookback window, applied because a newly-surfaced gold-standard Sitrep reconciles the date; source-preference outranks the lookback-window convention.</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="9" t="inlineStr">
+        <is>
+          <t>• 2026-06-08 (Web-directed, validator + chart constants for the Sitrep 03 reconciliation): src/validate.py NO_DIP_EXEMPTIONS_TIMESERIES: added "2026-05-31" -&gt; {suspected_global, total_global}; removed "2026-06-01" (now flat vs the revised May 31, no dip). NO_DIP_EXEMPTIONS_BREAKDOWN: added ("2026-05-31","DRC") -&gt; {suspected}; removed ("2026-06-01","DRC"). src/generate_charts.py BASELINE_RESET_DATES: added "2026-05-31", removed "2026-06-01" (the cleanup now lands on its Sitrep date). OBSERVED_UPWARD_REVISION_RANGE widened "&lt;1-35%" -&gt; "&lt;1-43%" to bracket the +42.7% DRC confirmed reconciliation. story.md "Latest update" corrected: the line wrongly stating "No WHO Weekly Sitrep 03 has published" now records Sitrep 03 (as of 31 May; DRC 321/48/15% CFR) as the latest reconciled report, with Sitrep 04 awaited to reconcile the post-5-June surge.</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="9" t="inlineStr">
+        <is>
+          <t>• 2026-06-08 (Web-directed, provisional-bars boundary): LAST_SITREP_STABLE_DATE advanced 2026-05-24 -&gt; 2026-05-31 (Sitrep 03's "as of" date). This un-hatches the May 25-31 bars; only the post-31-May BNO-sourced rows (June 1-7) remain provisional. Web reviewed and chose to KEEP the provisional-bar mechanism (the remaining hatched bars are exactly the un-reconciled, overshoot-prone wire days). PROCESS FIX FLAGGED FOR THE SCHEDULED TASK: add a WHO Weekly Sitrep check against the JS-rendered AFRO outbreak page (https://www.afro.who.int/health-topics/ebola-disease/outbreak-drc-26) via Chrome each run, so a new Sitrep advances LAST_SITREP_STABLE_DATE and triggers lookback reconciliation promptly.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="169">
+  <mergeCells count="173">
     <mergeCell ref="A130:H130"/>
     <mergeCell ref="A77:H77"/>
     <mergeCell ref="A83:H83"/>
     <mergeCell ref="A148:H148"/>
+    <mergeCell ref="A201:H201"/>
     <mergeCell ref="A157:H157"/>
     <mergeCell ref="A49:H49"/>
     <mergeCell ref="A138:H138"/>
@@ -2519,6 +2548,7 @@
     <mergeCell ref="A133:H133"/>
     <mergeCell ref="A189:H189"/>
     <mergeCell ref="A158:H158"/>
+    <mergeCell ref="A198:H198"/>
     <mergeCell ref="A50:H50"/>
     <mergeCell ref="A55:H55"/>
     <mergeCell ref="A86:H86"/>
@@ -2531,6 +2561,7 @@
     <mergeCell ref="A159:H159"/>
     <mergeCell ref="A97:H97"/>
     <mergeCell ref="A106:H106"/>
+    <mergeCell ref="A200:H200"/>
     <mergeCell ref="A134:H134"/>
     <mergeCell ref="A81:H81"/>
     <mergeCell ref="A38:H38"/>
@@ -2577,6 +2608,7 @@
     <mergeCell ref="A125:H125"/>
     <mergeCell ref="A190:H190"/>
     <mergeCell ref="A72:H72"/>
+    <mergeCell ref="A199:H199"/>
     <mergeCell ref="A112:H112"/>
     <mergeCell ref="A127:H127"/>
     <mergeCell ref="A167:H167"/>
@@ -3311,28 +3343,28 @@
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>98</v>
+        <v>-233</v>
       </c>
       <c r="C21" s="4" t="n">
-        <v>0</v>
+        <v>96</v>
       </c>
       <c r="D21" s="4" t="n">
         <v>0</v>
       </c>
       <c r="E21" s="4" t="n">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F21" s="4" t="n">
-        <v>-459</v>
+        <v>-790</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>122</v>
+        <v>218</v>
       </c>
       <c r="H21" s="4" t="n">
         <v>-223</v>
       </c>
       <c r="I21" s="4" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="J21" s="4" t="n">
         <v>7</v>
@@ -3345,16 +3377,16 @@
         </is>
       </c>
       <c r="B22" s="6" t="n">
-        <v>-331</v>
+        <v>0</v>
       </c>
       <c r="C22" s="6" t="n">
-        <v>96</v>
+        <v>0</v>
       </c>
       <c r="D22" s="6" t="n">
         <v>0</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F22" s="6" t="n">
         <v>-790</v>
@@ -3561,16 +3593,16 @@
         <v>5</v>
       </c>
       <c r="F28" s="6" t="n">
-        <v>-331</v>
+        <v>0</v>
       </c>
       <c r="G28" s="6" t="n">
-        <v>300</v>
+        <v>204</v>
       </c>
       <c r="H28" s="6" t="n">
         <v>0</v>
       </c>
       <c r="I28" s="6" t="n">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="J28" s="6" t="n">
         <v>7</v>
@@ -4678,20 +4710,20 @@
         </is>
       </c>
       <c r="C37" s="4" t="n">
-        <v>447</v>
+        <v>116</v>
       </c>
       <c r="D37" s="4" t="n">
-        <v>225</v>
+        <v>321</v>
       </c>
       <c r="E37" s="4" t="n">
         <v>0</v>
       </c>
       <c r="F37" s="4" t="n">
-        <v>42</v>
+        <v>48</v>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>REVISED 2026-06-01 (scheduled run): confirmed_deaths corrected from 55 to 42 per [BNO @BNOFeed Daily Ebola Update June 1, 2026 graphic](https://x.com/BNOFeed/status/2061573338569351279) (DRC June 1 conf_deaths = 48 with +6 delta, implying yesterday's = 42) and DRC MoH 31 May situation report (per multiple wire summaries June 1: 282 confirmed / 42 confirmed deaths / 220 suspected in DRC). The prior 55 was a sus_deaths-zeroing inference (+38 attributed to conf_deaths from BNO May 31 graphic's "55 deaths"); DRC MoH's formal 31 May figure is 42. PRIOR REVISION 2026-05-31 (PM): MoH methodology-change carve-out propagated from revised May 30 row. BNO @BNOFeed Daily Ebola Update May 31 graphic (sourced to DRC MoH + Uganda MoH + WHO): DR Congo 672 cases (+98) / 55 deaths (+38), on the May 30 DRC MoH cleaned baseline. Split inference: DRC conf carries the May 30 DRC MoH running 225 forward; DRC sus = 672 - 225 = 447; DRC sus_deaths stays at 0 (column zeroed May 30). Revisions vs prior WHO DON605 carry-forward (906/125/223/17): sus -50.66%, conf +80.00%, sus_deaths -100%. WHO Sitrep 03 expected Tue 2 Jun will reconcile.</t>
+          <t>REVISED 2026-06-08 (Web-directed, WHO Sitrep 03 reconciliation): [WHO Weekly External Situation Report 03, data as of 31 May 2026](https://www.afro.who.int/health-topics/ebola-disease/outbreak-drc-26): DRC 321 confirmed / 48 confirmed deaths / 0 probable / 15.0% CFR. Reconciled from the prior BNO running count: suspected 447-&gt;116, confirmed 225-&gt;321 (+42.7%), conf_deaths 42-&gt;48; suspected_deaths 0 unchanged. WHO Weekly Sitrep is the gold-standard source (preference #1) and supersedes the wire count. NO_DIP_EXEMPTIONS_BREAKDOWN (2026-05-31, DRC) -&gt; {suspected}. Prior: BNO May 31 cleaned-baseline DR Congo 672 cases / 55 deaths, DRC conf 225 / sus 447.</t>
         </is>
       </c>
       <c r="H37" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Re-derive June recovered from BNO graphics: fill 06-05/07/21/22, fix 06-06, flag 06-14 anomaly
</commit_message>
<xml_diff>
--- a/outputs/ebola_timeseries.xlsx
+++ b/outputs/ebola_timeseries.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I461"/>
+  <dimension ref="A1:I463"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -1316,7 +1316,9 @@
       <c r="F26" s="6" t="n">
         <v>66</v>
       </c>
-      <c r="G26" s="6" t="n"/>
+      <c r="G26" s="6" t="n">
+        <v>12</v>
+      </c>
       <c r="H26" s="7" t="inlineStr">
         <is>
           <t>[WHO Disease Outbreak News, data as of 5 June 2026] reconciled snapshot: DRC 381 confirmed / 64 confirmed deaths (DRC MoH figures published 4 June, as of 3 June; 233 hospitalised in isolation), across Ituri (359 conf / 17 health zones), North Kivu (19 conf / 7 health zones) and South Kivu (3 conf / 1 health zone). Uganda 19 confirmed / 2 deaths as of 5 June (3 new cases reported 5 June were contacts of confirmed cases; 8 of 9 geolocated cases in Kampala, 1 in Wakiso). Global: suspected 116 (carried forward from 3 June - no updated official suspected figure published in the 5 June WHO DON / Xinhua / CDC sources, all of which led with confirmed; DRC now testing nearly all samples with results within 24h per Health Minister Kamba, draining the suspected backlog), confirmed 400 (DRC 381 + Uganda 19), total 516, suspected_deaths 0 (column zeroed 30 May), confirmed_deaths 66 (DRC 64 + Uganda 2). DRC Health Minister Roger Kamba press briefing 4 June via Xinhua (https://english.news.cn/africa/20260605/75381cda9c1642f7acfdaac060a5bf0f/c.html) cited DRC 381 conf / 63 deaths / 233 hospitalised, contact tracing improved from ~9% to 55% (target 90%), 4,000+ Africa CDC test kits arrived enabling 24h results; WHO DON's 64 DRC conf_deaths used per source-preference (WHO DON &gt; MoH-via-wire, which said 63). vs June 3 (116/359/475/0/61): suspected unchanged, confirmed +41, total +41, conf_deaths +5; cumulative non-decreasing on all columns, no exemption needed. SOURCE-VIEW DIVERGENCE FLAG: BNO @BNOFeed Daily Ebola Update June 5 graphic shows TOTAL 471 confirmed (+74) / 84 deaths (+19) / 12 recovered (+3), a DRC MoH-attributed running wire count ~71 cases / 18 deaths above the WHO-reconciled total (BNO June 4 graphic = 397 conf / 65 deaths matched the official DRC 381 + Uganda 16 sum exactly; BNO June 3 = 378/63). Per source-preference order (WHO DON &gt; BNO News), WHO figures win for the row; BNO running count noted for transparency (same forward-lead pattern as June 1 and June 3). CDC June 5 release (https://www.cdc.gov/media/releases/2026/update-on-ebola-outbreak-in-the-democratic-republic-of-the-congo-and-uganda-6-5-2026.html): three MMWRs - Notes from the Field (largest Bundibugyo outbreak on record; first detected among healthcare-worker clusters), a US risk assessment (risk to general US public low), and CFA modeling (without strong interventions the outbreak could rival or exceed the 2014-2016 West Africa outbreak; &gt;20,000 cases in 2 of 3 simulations at 20% case isolation within 2 days). No WHO Weekly Sitrep 03 yet; DON + briefings remain the reconciliation channel. Catch-up run after June 3 (no June 4 row): the WHO 'as of 5 June' DON is the single reconciled data point and June 4 is not separately rowed (its DRC figure is the same as-of-3-June 381 count, Uganda's increment folds into the 5 June total).</t>
@@ -1350,7 +1352,7 @@
         <v>93</v>
       </c>
       <c r="G27" s="4" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="H27" s="5" t="inlineStr">
         <is>
@@ -1384,7 +1386,9 @@
       <c r="F28" s="6" t="n">
         <v>103</v>
       </c>
-      <c r="G28" s="6" t="n"/>
+      <c r="G28" s="6" t="n">
+        <v>16</v>
+      </c>
       <c r="H28" s="7" t="inlineStr">
         <is>
           <t>REVISED 2026-06-12 per WHO Weekly External Situation Report 04 (https://www.afro.who.int/countries/uganda/publication/ebola-bundibugyo-virus-disease-outbreak-democratic-republic-congo-0, published 7 June, data as of 07 June 2026): WHO-reconciled figures as of 7 June are DRC 550 confirmed / 101 confirmed deaths (CFR 18.4%; 229 new confirmed cases and 53 new confirmed deaths since 31 May; 25 health zones across Ituri 518 conf / 80 deaths, North Kivu 25 conf / 15 deaths CFR 60%, South Kivu 3 conf / 1 death) and Uganda 19 confirmed / 2 confirmed deaths (plus 1 probable case and 1 probable death, not counted in the confirmed columns; 5 cases are health workers; Kampala + Wakiso). Global: suspected 116 carried (Sitrep reports confirmed+probable only, no suspected figure), confirmed 569 (DRC 550 + Uganda 19), total 685, suspected_deaths 0 (column zeroed 30 May), confirmed_deaths 103 (DRC 101 + Uganda 2). UPWARD reconciliation of the prior BNO @BNOFeed June 7 running count (DRC 515/91): WHO as-of-7-June DRC figure exceeds the same-day BNO count due to backlog-sample attribution, same direction as DON606 for 6 June. Revisions vs prior: confirmed 534-&gt;569 (+6.55%), total 650-&gt;685 (+5.38%), conf_deaths 93-&gt;103 (+10.75%). The reconciled 7 June figure equals the BNO June 8 running count (DRC 550/101), collapsing the apparent June 7-&gt;8 jump to flat. Upward revision, no-dip rule not triggered. Prior (superseded) primary_source: BNO @BNOFeed June 7 graphic, DRC 515/91 + Uganda 19/2.</t>
@@ -1870,7 +1874,9 @@
       <c r="F42" s="6" t="n">
         <v>269</v>
       </c>
-      <c r="G42" s="6" t="n"/>
+      <c r="G42" s="6" t="n">
+        <v>110</v>
+      </c>
       <c r="H42" s="7" t="inlineStr">
         <is>
           <t>REVISED 2026-06-29 per WHO Weekly External Situation Report 06 (https://www.afro.who.int/countries/uganda/publication/ebola-bundibugyo-virus-disease-outbreak-democratic-republic-congo-2, data as of 21 June 2026): WHO-reconciled figures as of 21 June are DRC 1048 confirmed / 267 confirmed deaths (CFR 25.5%; +240 confirmed and +75 confirmed deaths since 14 June) across Ituri, North Kivu and South Kivu, and Uganda 20 confirmed / 2 confirmed deaths (one new confirmed case reported after nearly two weeks without a case; plus 1 probable case and 1 probable death, not counted in the confirmed columns). Global: suspected 116 carried (Sitrep reports confirmed+probable only, no suspected figure), confirmed 1068 (DRC 1048 + Uganda 20), total 1184, suspected_deaths 0 (column zeroed 30 May), confirmed_deaths 269 (DRC 267 + Uganda 2). UPWARD reconciliation of the prior BNO @BNOFeed June 21 running count (DRC 1003/254 + Uganda 19/2): the WHO as-of-21-June DRC figure exceeds the same-day BNO count due to backlog-sample attribution, same direction as Sitreps 04 and 05 and DON606. Revisions vs prior: confirmed 1022-&gt;1068 (+4.50%), total 1138-&gt;1184 (+4.04%), conf_deaths 256-&gt;269 (+5.08%). Sitrep 06 also places the Uganda 19-&gt;20 increment on 21 June (BNO had shown it on the June 23 graphic). The reconciled 21 June DRC figure (1048) equals the BNO June 22 running count, collapsing the apparent June 21-&gt;22 jump to flat, same pattern as prior Sitrep reconciliations. Upward revision, no-dip rule not triggered. LAST_SITREP_STABLE_DATE advanced to 2026-06-21 this run. Prior (superseded) primary_source: BNO @BNOFeed June 21 graphic, DRC 1003/254 + Uganda 19/2.</t>
@@ -1903,7 +1909,9 @@
       <c r="F43" s="4" t="n">
         <v>269</v>
       </c>
-      <c r="G43" s="4" t="n"/>
+      <c r="G43" s="4" t="n">
+        <v>122</v>
+      </c>
       <c r="H43" s="5" t="inlineStr">
         <is>
           <t>REVISED 2026-06-29 (Uganda no-dip carry-forward from WHO Weekly External Situation Report 06): WHO Sitrep 06 (data as of 21 June 2026) establishes Uganda at 20 confirmed by 21 June, so the prior June 22 Uganda 19 is carried forward to 20 to keep cumulative confirmed monotonically non-decreasing after the June 21 row was reconciled upward to 1068. DRC unchanged at 1048 confirmed / 267 confirmed deaths ([BNO @BNOFeed June 22 graphic](https://x.com/BNOFeed/status/2069188090065727998), which equals the WHO as-of-21-June DRC figure). Global: suspected 116, confirmed 1068 (DRC 1048 + Uganda 20), total 1184, suspected_deaths 0, confirmed_deaths 269 (DRC 267 + Uganda 2). Revisions vs prior: confirmed 1067-&gt;1068 (+0.09%), total 1183-&gt;1184 (+0.08%), conf_deaths unchanged 269. June 21 and June 22 are now flat at 1068/1184/269, the documented WHO-reconciliation-equals-next-day-BNO pattern. Upward revision, no-dip rule not triggered. Prior (superseded) primary_source: BNO @BNOFeed June 22 graphic, DRC 1048/267 + Uganda 19/2.</t>
@@ -5638,8 +5646,22 @@
         </is>
       </c>
     </row>
+    <row r="462">
+      <c r="A462" s="9" t="inlineStr">
+        <is>
+          <t>• 2026-07-23 (Web-directed, June recovered re-derivation): re-read the full June recovered series against the embedded-date BNO @BNOFeed graphics (date-filtered search windows read via Chrome). Corrections/fills: 06-05 DRC 8 / Uganda 4 / total 12 (was gap); 06-06 total 16-&gt;13, DRC 12-&gt;9 (the stored 06-06 had been holding the JUNE 7 graphic figures, DRC 12 / total 16 -- an off-by-one-day error); 06-07 DRC 12 / Uganda 4 / total 16 (was gap); 06-21 DRC 100 / Uganda 10 / total 110 (was gap); 06-22 DRC 112 / Uganda 10 / total 122 (Uganda + total filled). Verified unchanged/correct against graphics: 06-04, 06-08 through 06-13, 06-15 through 06-20, 06-23, 06-24. 06-03 has no BNO Recovered column (BNO added it 06-04); 06-03 = 8 is reconstructed from the 06-04 delta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" s="9" t="inlineStr">
+        <is>
+          <t>• 2026-07-23 (Web-directed, June recovered): 06-14 left BLANK as a BNO anomaly, not filled. The JUNE 14 graphic reported total recovered 61 (DR Congo 56, +21), contradicted the next day by the JUNE 15 graphic at 53 (DR Congo 48). Cumulative recoveries cannot decrease, so the 06-14 over-count is a BNO reporting error; encoding 61 would force a monotonicity break at 06-15 (and fail validate.py). Left blank and forward-filled in the chart, per the no-guess rule. recovered_global remains monotonic with no dips after these edits.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="389">
+  <mergeCells count="391">
     <mergeCell ref="A164:I164"/>
     <mergeCell ref="A335:I335"/>
     <mergeCell ref="A195:I195"/>
@@ -5819,6 +5841,7 @@
     <mergeCell ref="A417:I417"/>
     <mergeCell ref="A221:I221"/>
     <mergeCell ref="A196:I196"/>
+    <mergeCell ref="A463:I463"/>
     <mergeCell ref="A223:I223"/>
     <mergeCell ref="A198:I198"/>
     <mergeCell ref="A394:I394"/>
@@ -5934,6 +5957,7 @@
     <mergeCell ref="A289:I289"/>
     <mergeCell ref="A226:I226"/>
     <mergeCell ref="A291:I291"/>
+    <mergeCell ref="A462:I462"/>
     <mergeCell ref="A241:I241"/>
     <mergeCell ref="A228:I228"/>
     <mergeCell ref="A355:I355"/>
@@ -7061,7 +7085,7 @@
         <v>1</v>
       </c>
       <c r="F26" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G26" s="6" t="n">
         <v>-790</v>
@@ -7076,10 +7100,10 @@
         <v>48</v>
       </c>
       <c r="K26" s="6" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="L26" s="6" t="n">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="M26" s="6" t="n">
         <v>7</v>
@@ -7104,7 +7128,7 @@
         <v>27</v>
       </c>
       <c r="F27" s="4" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="G27" s="4" t="n">
         <v>-233</v>
@@ -7119,10 +7143,10 @@
         <v>75</v>
       </c>
       <c r="K27" s="4" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="L27" s="4" t="n">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="M27" s="4" t="n">
         <v>7</v>
@@ -7147,7 +7171,7 @@
         <v>10</v>
       </c>
       <c r="F28" s="6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G28" s="6" t="n">
         <v>0</v>
@@ -7749,7 +7773,7 @@
         <v>20</v>
       </c>
       <c r="F42" s="6" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="G42" s="6" t="n">
         <v>0</v>
@@ -7764,10 +7788,10 @@
         <v>75</v>
       </c>
       <c r="K42" s="6" t="n">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="L42" s="6" t="n">
-        <v>697</v>
+        <v>689</v>
       </c>
       <c r="M42" s="6" t="n">
         <v>7</v>
@@ -7792,7 +7816,7 @@
         <v>0</v>
       </c>
       <c r="F43" s="4" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="G43" s="4" t="n">
         <v>0</v>
@@ -7807,10 +7831,10 @@
         <v>75</v>
       </c>
       <c r="K43" s="4" t="n">
-        <v>102</v>
+        <v>122</v>
       </c>
       <c r="L43" s="4" t="n">
-        <v>697</v>
+        <v>677</v>
       </c>
       <c r="M43" s="4" t="n">
         <v>7</v>
@@ -7835,7 +7859,7 @@
         <v>10</v>
       </c>
       <c r="F44" s="6" t="n">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="G44" s="6" t="n">
         <v>0</v>
@@ -10629,7 +10653,7 @@
         <v>64</v>
       </c>
       <c r="G47" s="4" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="H47" s="5" t="inlineStr">
         <is>
@@ -10661,7 +10685,9 @@
       <c r="F48" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G48" s="6" t="n"/>
+      <c r="G48" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="H48" s="7" t="inlineStr">
         <is>
           <t>[WHO Disease Outbreak News, as of 5 June 2026]: Uganda 19 confirmed / 2 deaths. Three new cases reported 5 June were contacts of confirmed cases. Of 9 geolocated cases, 8 in Kampala and 1 in Wakiso. Uganda does not report suspected cases. Progression: 15 (June 2-3) -&gt; 16 (June 4, +1 new confirmed Thursday per Uganda MoH via Xinhua) -&gt; 19 (June 5, +3 contacts). Second Uganda death recorded as of 5 June (was 1 death June 2-3); deaths now 2. vs June 3 (15 conf / 1 death): confirmed +4, deaths +1.</t>
@@ -10697,7 +10723,7 @@
         <v>91</v>
       </c>
       <c r="G49" s="4" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="H49" s="5" t="inlineStr">
         <is>
@@ -10766,7 +10792,9 @@
       <c r="F51" s="4" t="n">
         <v>101</v>
       </c>
-      <c r="G51" s="4" t="n"/>
+      <c r="G51" s="4" t="n">
+        <v>12</v>
+      </c>
       <c r="H51" s="5" t="inlineStr">
         <is>
           <t>REVISED 2026-06-12 per WHO Weekly External Situation Report 04 (data as of 07 June 2026, https://www.afro.who.int/countries/uganda/publication/ebola-bundibugyo-virus-disease-outbreak-democratic-republic-congo-0): DRC 550 confirmed / 101 confirmed deaths (CFR 18.4%); 229 new confirmed cases and 53 new confirmed deaths since 31 May. 25 health zones: Ituri 518 conf (94.2%) / 80 deaths, North Kivu 25 conf / 15 deaths (CFR 60.0%), South Kivu 3 conf / 1 death; Mambasa and Rimba (Ituri) newly affected; 94 Ituri cases incl. 10 deaths unattributed to a health zone. 5418 contacts under follow-up (64.4% seen in 24h). suspected 116 carried; suspected_deaths 0 (zeroed 30 May). UPWARD reconciliation of the prior BNO June 7 running count (515/91): WHO as-of-7-June DRC figure exceeds same-day BNO due to backlog-sample attribution. vs prior (515/91): confirmed +6.80%, conf_deaths +10.99%. Prior (superseded): BNO @BNOFeed June 7 graphic, DRC 515/91.</t>
@@ -10797,7 +10825,9 @@
       <c r="F52" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G52" s="6" t="n"/>
+      <c r="G52" s="6" t="n">
+        <v>4</v>
+      </c>
       <c r="H52" s="7" t="inlineStr">
         <is>
           <t>REVISED 2026-06-12 per WHO Weekly External Situation Report 04 (data as of 07 June 2026): Uganda 19 confirmed / 2 confirmed deaths, plus 1 probable case and 1 probable death (probable not counted in the confirmed columns). +8 confirmed cases and +1 confirmed death since Sitrep 03 (31 May). 20 cases total (confirmed+probable) across Kampala and Wakiso districts in the Kampala Metropolitan Area; 5 are health workers. 783 contacts identified, 91% 24h follow-up. Numerically unchanged vs prior BNO June 7 (19/2); source upgraded from BNO running count to WHO Sitrep 04. Uganda does not report suspected cases.</t>
@@ -11738,7 +11768,9 @@
       <c r="F79" s="4" t="n">
         <v>267</v>
       </c>
-      <c r="G79" s="4" t="n"/>
+      <c r="G79" s="4" t="n">
+        <v>100</v>
+      </c>
       <c r="H79" s="5" t="inlineStr">
         <is>
           <t>REVISED 2026-06-29 per WHO Weekly External Situation Report 06 (data as of 21 June 2026): DRC 1048 confirmed / 267 confirmed deaths (CFR 25.5%; +240 confirmed, +75 confirmed deaths since 14 June). suspected 116 carried (Sitrep confirmed+probable framing; BNO tracks confirmed only); suspected_deaths 0 (zeroed 30 May). UPWARD reconciliation of the prior BNO June 21 running count (DRC 1003/254): WHO as-of-21-June exceeds the same-day BNO count via backlog-sample attribution and equals the BNO June 22 figure (collapses June 21-&gt;22 to flat). conf 1003-&gt;1048 (+4.49%), conf_deaths 254-&gt;267 (+5.12%). LAST_SITREP_STABLE_DATE advanced to 2026-06-21. Prior (superseded): BNO @BNOFeed June 21 graphic DRC 1003/254.</t>
@@ -11769,7 +11801,9 @@
       <c r="F80" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G80" s="6" t="n"/>
+      <c r="G80" s="6" t="n">
+        <v>10</v>
+      </c>
       <c r="H80" s="7" t="inlineStr">
         <is>
           <t>REVISED 2026-06-29 per WHO Weekly External Situation Report 06 (data as of 21 June 2026): Uganda 20 confirmed / 2 confirmed deaths (one new confirmed case after nearly two weeks without a case; plus 1 probable case and 1 probable death, not counted in the confirmed columns). Sitrep 06 places the 19-&gt;20 increment on 21 June; BNO had first shown it on the June 23 graphic. conf 19-&gt;20 (+1), deaths unchanged. Prior (superseded): BNO @BNOFeed June 21 graphic Uganda 19/2.</t>
@@ -11837,7 +11871,9 @@
       <c r="F82" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="G82" s="6" t="n"/>
+      <c r="G82" s="6" t="n">
+        <v>10</v>
+      </c>
       <c r="H82" s="7" t="inlineStr">
         <is>
           <t>REVISED 2026-06-29 (no-dip carry-forward from WHO Weekly External Situation Report 06): Uganda carried at 20 confirmed / 2 deaths because Sitrep 06 establishes Uganda 20 by 21 June, so June 22 cannot dip back to 19. conf 19-&gt;20 (+1), deaths unchanged. Prior (superseded): BNO @BNOFeed June 22 graphic Uganda 19/2.</t>

</xml_diff>

<commit_message>
Add week-over-week active-cases chart (7-day avg vs prior 7-day avg)
</commit_message>
<xml_diff>
--- a/outputs/ebola_timeseries.xlsx
+++ b/outputs/ebola_timeseries.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I463"/>
+  <dimension ref="A1:I464"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -5660,8 +5660,15 @@
         </is>
       </c>
     </row>
+    <row r="464">
+      <c r="A464" s="9" t="inlineStr">
+        <is>
+          <t>• 2026-07-23 (Web-directed change): added a fourth chart, week-over-week percent change in active cases. src/generate_charts.py gains compute_active_wow + render_active_wow_chart: for each date, mean active over the trailing 7 days (t-6..t) vs. the prior 7 days (t-13..t-7), plotted as (current_mean/prior_mean - 1)*100. The two adjacent 7-day averaging windows smooth daily spikes so the line reads as a growth-rate trend (above zero = active pool still growing). Undefined until 14 days of active history; skipped where the prior-window mean is non-positive. Outputs YYYY-MM-DD_ebola-active-wow.png + latest-active-wow.png; wired into main() as the fourth published chart and added to index.html. build_xlsx.py Charts sheet gains an "Active w/w % (7-day avg)" column. METHODOLOGY.md Charts section and README updated (four charts now). As of 2026-07-22 the w/w change reads about +7.5%, down from ~+200% in late May: the active caseload is still growing but the growth rate has decelerated sharply.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="391">
+  <mergeCells count="392">
     <mergeCell ref="A164:I164"/>
     <mergeCell ref="A335:I335"/>
     <mergeCell ref="A195:I195"/>
@@ -5746,6 +5753,7 @@
     <mergeCell ref="A393:I393"/>
     <mergeCell ref="A160:I160"/>
     <mergeCell ref="A331:I331"/>
+    <mergeCell ref="A464:I464"/>
     <mergeCell ref="A141:I141"/>
     <mergeCell ref="A439:I439"/>
     <mergeCell ref="A377:I377"/>
@@ -6064,7 +6072,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M72"/>
+  <dimension ref="A1:N72"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6079,7 +6087,8 @@
     <col width="24" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
     <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -6092,7 +6101,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Derived from the main timeseries. Charts live as PNG files in outputs/ — this table is the data behind them. Active ("live") cases = cumulative confirmed minus recovered minus confirmed deaths; recovered is forward-filled across days with no published figure.</t>
+          <t>Derived from the main timeseries. Charts live as PNG files in outputs/ — this table is the data behind them. Active ("live") cases = cumulative confirmed minus recovered minus confirmed deaths; recovered is forward-filled across days with no published figure. Active w/w % = mean active over days t-6..t vs. days t-13..t-7.</t>
         </is>
       </c>
     </row>
@@ -6159,6 +6168,11 @@
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
+          <t>Active w/w % (7-day avg)</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="inlineStr">
+        <is>
           <t>Window (days)</t>
         </is>
       </c>
@@ -6202,7 +6216,8 @@
       <c r="L5" s="4" t="n">
         <v>7</v>
       </c>
-      <c r="M5" s="4" t="n">
+      <c r="M5" s="4" t="n"/>
+      <c r="N5" s="4" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6245,7 +6260,8 @@
       <c r="L6" s="6" t="n">
         <v>12</v>
       </c>
-      <c r="M6" s="6" t="n">
+      <c r="M6" s="6" t="n"/>
+      <c r="N6" s="6" t="n">
         <v>2</v>
       </c>
     </row>
@@ -6288,7 +6304,8 @@
       <c r="L7" s="4" t="n">
         <v>12</v>
       </c>
-      <c r="M7" s="4" t="n">
+      <c r="M7" s="4" t="n"/>
+      <c r="N7" s="4" t="n">
         <v>3</v>
       </c>
     </row>
@@ -6331,7 +6348,8 @@
       <c r="L8" s="6" t="n">
         <v>32</v>
       </c>
-      <c r="M8" s="6" t="n">
+      <c r="M8" s="6" t="n"/>
+      <c r="N8" s="6" t="n">
         <v>4</v>
       </c>
     </row>
@@ -6374,7 +6392,8 @@
       <c r="L9" s="4" t="n">
         <v>32</v>
       </c>
-      <c r="M9" s="4" t="n">
+      <c r="M9" s="4" t="n"/>
+      <c r="N9" s="4" t="n">
         <v>5</v>
       </c>
     </row>
@@ -6417,7 +6436,8 @@
       <c r="L10" s="6" t="n">
         <v>50</v>
       </c>
-      <c r="M10" s="6" t="n">
+      <c r="M10" s="6" t="n"/>
+      <c r="N10" s="6" t="n">
         <v>6</v>
       </c>
     </row>
@@ -6460,7 +6480,8 @@
       <c r="L11" s="4" t="n">
         <v>84</v>
       </c>
-      <c r="M11" s="4" t="n">
+      <c r="M11" s="4" t="n"/>
+      <c r="N11" s="4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -6503,7 +6524,8 @@
       <c r="L12" s="6" t="n">
         <v>84</v>
       </c>
-      <c r="M12" s="6" t="n">
+      <c r="M12" s="6" t="n"/>
+      <c r="N12" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -6546,7 +6568,8 @@
       <c r="L13" s="4" t="n">
         <v>87</v>
       </c>
-      <c r="M13" s="4" t="n">
+      <c r="M13" s="4" t="n"/>
+      <c r="N13" s="4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -6589,7 +6612,8 @@
       <c r="L14" s="6" t="n">
         <v>101</v>
       </c>
-      <c r="M14" s="6" t="n">
+      <c r="M14" s="6" t="n"/>
+      <c r="N14" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -6632,7 +6656,8 @@
       <c r="L15" s="4" t="n">
         <v>101</v>
       </c>
-      <c r="M15" s="4" t="n">
+      <c r="M15" s="4" t="n"/>
+      <c r="N15" s="4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -6675,7 +6700,8 @@
       <c r="L16" s="6" t="n">
         <v>101</v>
       </c>
-      <c r="M16" s="6" t="n">
+      <c r="M16" s="6" t="n"/>
+      <c r="N16" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -6718,7 +6744,8 @@
       <c r="L17" s="4" t="n">
         <v>114</v>
       </c>
-      <c r="M17" s="4" t="n">
+      <c r="M17" s="4" t="n"/>
+      <c r="N17" s="4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -6762,6 +6789,9 @@
         <v>115</v>
       </c>
       <c r="M18" s="6" t="n">
+        <v>207</v>
+      </c>
+      <c r="N18" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -6805,6 +6835,9 @@
         <v>116</v>
       </c>
       <c r="M19" s="4" t="n">
+        <v>140.2</v>
+      </c>
+      <c r="N19" s="4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -6848,6 +6881,9 @@
         <v>216</v>
       </c>
       <c r="M20" s="6" t="n">
+        <v>126.8</v>
+      </c>
+      <c r="N20" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -6891,6 +6927,9 @@
         <v>281</v>
       </c>
       <c r="M21" s="4" t="n">
+        <v>122.1</v>
+      </c>
+      <c r="N21" s="4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -6934,6 +6973,9 @@
         <v>281</v>
       </c>
       <c r="M22" s="6" t="n">
+        <v>127.1</v>
+      </c>
+      <c r="N22" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -6977,6 +7019,9 @@
         <v>287</v>
       </c>
       <c r="M23" s="4" t="n">
+        <v>131.9</v>
+      </c>
+      <c r="N23" s="4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7020,6 +7065,9 @@
         <v>290</v>
       </c>
       <c r="M24" s="6" t="n">
+        <v>136</v>
+      </c>
+      <c r="N24" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7063,6 +7111,9 @@
         <v>323</v>
       </c>
       <c r="M25" s="4" t="n">
+        <v>155.2</v>
+      </c>
+      <c r="N25" s="4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7106,6 +7157,9 @@
         <v>322</v>
       </c>
       <c r="M26" s="6" t="n">
+        <v>172.1</v>
+      </c>
+      <c r="N26" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7149,6 +7203,9 @@
         <v>428</v>
       </c>
       <c r="M27" s="4" t="n">
+        <v>156</v>
+      </c>
+      <c r="N27" s="4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7192,6 +7249,9 @@
         <v>450</v>
       </c>
       <c r="M28" s="6" t="n">
+        <v>128.1</v>
+      </c>
+      <c r="N28" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7235,6 +7295,9 @@
         <v>443</v>
       </c>
       <c r="M29" s="4" t="n">
+        <v>107.8</v>
+      </c>
+      <c r="N29" s="4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7278,6 +7341,9 @@
         <v>473</v>
       </c>
       <c r="M30" s="6" t="n">
+        <v>93.5</v>
+      </c>
+      <c r="N30" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7321,6 +7387,9 @@
         <v>490</v>
       </c>
       <c r="M31" s="4" t="n">
+        <v>84.7</v>
+      </c>
+      <c r="N31" s="4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7364,6 +7433,9 @@
         <v>520</v>
       </c>
       <c r="M32" s="6" t="n">
+        <v>74.2</v>
+      </c>
+      <c r="N32" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7407,6 +7479,9 @@
         <v>530</v>
       </c>
       <c r="M33" s="4" t="n">
+        <v>66.7</v>
+      </c>
+      <c r="N33" s="4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7450,6 +7525,9 @@
         <v>538</v>
       </c>
       <c r="M34" s="6" t="n">
+        <v>55.7</v>
+      </c>
+      <c r="N34" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7493,6 +7571,9 @@
         <v>593</v>
       </c>
       <c r="M35" s="4" t="n">
+        <v>50.7</v>
+      </c>
+      <c r="N35" s="4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7536,6 +7617,9 @@
         <v>580</v>
       </c>
       <c r="M36" s="6" t="n">
+        <v>46.4</v>
+      </c>
+      <c r="N36" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7579,6 +7663,9 @@
         <v>604</v>
       </c>
       <c r="M37" s="4" t="n">
+        <v>41.3</v>
+      </c>
+      <c r="N37" s="4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7622,6 +7709,9 @@
         <v>618</v>
       </c>
       <c r="M38" s="6" t="n">
+        <v>36</v>
+      </c>
+      <c r="N38" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7665,6 +7755,9 @@
         <v>593</v>
       </c>
       <c r="M39" s="4" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="N39" s="4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7708,6 +7801,9 @@
         <v>615</v>
       </c>
       <c r="M40" s="6" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="N40" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7751,6 +7847,9 @@
         <v>624</v>
       </c>
       <c r="M41" s="4" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="N41" s="4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7794,6 +7893,9 @@
         <v>689</v>
       </c>
       <c r="M42" s="6" t="n">
+        <v>20.5</v>
+      </c>
+      <c r="N42" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7837,6 +7939,9 @@
         <v>677</v>
       </c>
       <c r="M43" s="4" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="N43" s="4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7880,6 +7985,9 @@
         <v>706</v>
       </c>
       <c r="M44" s="6" t="n">
+        <v>17.3</v>
+      </c>
+      <c r="N44" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7923,6 +8031,9 @@
         <v>709</v>
       </c>
       <c r="M45" s="4" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="N45" s="4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -7966,6 +8077,9 @@
         <v>717</v>
       </c>
       <c r="M46" s="6" t="n">
+        <v>16.8</v>
+      </c>
+      <c r="N46" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8009,6 +8123,9 @@
         <v>738</v>
       </c>
       <c r="M47" s="4" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="N47" s="4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8052,6 +8169,9 @@
         <v>754</v>
       </c>
       <c r="M48" s="6" t="n">
+        <v>18.1</v>
+      </c>
+      <c r="N48" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8095,6 +8215,9 @@
         <v>754</v>
       </c>
       <c r="M49" s="4" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="N49" s="4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8138,6 +8261,9 @@
         <v>749</v>
       </c>
       <c r="M50" s="6" t="n">
+        <v>16</v>
+      </c>
+      <c r="N50" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8181,6 +8307,9 @@
         <v>780</v>
       </c>
       <c r="M51" s="4" t="n">
+        <v>15</v>
+      </c>
+      <c r="N51" s="4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8224,6 +8353,9 @@
         <v>799</v>
       </c>
       <c r="M52" s="6" t="n">
+        <v>14.7</v>
+      </c>
+      <c r="N52" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8267,6 +8399,9 @@
         <v>803</v>
       </c>
       <c r="M53" s="4" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="N53" s="4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8310,6 +8445,9 @@
         <v>799</v>
       </c>
       <c r="M54" s="6" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="N54" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8353,6 +8491,9 @@
         <v>851</v>
       </c>
       <c r="M55" s="4" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="N55" s="4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8396,6 +8537,9 @@
         <v>832</v>
       </c>
       <c r="M56" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="N56" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8439,6 +8583,9 @@
         <v>849</v>
       </c>
       <c r="M57" s="4" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="N57" s="4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8482,6 +8629,9 @@
         <v>875</v>
       </c>
       <c r="M58" s="6" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="N58" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8525,6 +8675,9 @@
         <v>873</v>
       </c>
       <c r="M59" s="4" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="N59" s="4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8568,6 +8721,9 @@
         <v>888</v>
       </c>
       <c r="M60" s="6" t="n">
+        <v>11</v>
+      </c>
+      <c r="N60" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8611,6 +8767,9 @@
         <v>896</v>
       </c>
       <c r="M61" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="N61" s="4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8654,6 +8813,9 @@
         <v>927</v>
       </c>
       <c r="M62" s="6" t="n">
+        <v>10.9</v>
+      </c>
+      <c r="N62" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8697,6 +8859,9 @@
         <v>912</v>
       </c>
       <c r="M63" s="4" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="N63" s="4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8740,6 +8905,9 @@
         <v>912</v>
       </c>
       <c r="M64" s="6" t="n">
+        <v>10</v>
+      </c>
+      <c r="N64" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8783,6 +8951,9 @@
         <v>931</v>
       </c>
       <c r="M65" s="4" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="N65" s="4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8826,6 +8997,9 @@
         <v>931</v>
       </c>
       <c r="M66" s="6" t="n">
+        <v>8.800000000000001</v>
+      </c>
+      <c r="N66" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8869,6 +9043,9 @@
         <v>952</v>
       </c>
       <c r="M67" s="4" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="N67" s="4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8912,6 +9089,9 @@
         <v>1009</v>
       </c>
       <c r="M68" s="6" t="n">
+        <v>8.4</v>
+      </c>
+      <c r="N68" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8955,6 +9135,9 @@
         <v>948</v>
       </c>
       <c r="M69" s="4" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="N69" s="4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -8998,6 +9181,9 @@
         <v>987</v>
       </c>
       <c r="M70" s="6" t="n">
+        <v>7.2</v>
+      </c>
+      <c r="N70" s="6" t="n">
         <v>7</v>
       </c>
     </row>
@@ -9041,6 +9227,9 @@
         <v>992</v>
       </c>
       <c r="M71" s="4" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="N71" s="4" t="n">
         <v>7</v>
       </c>
     </row>
@@ -9084,13 +9273,16 @@
         <v>997</v>
       </c>
       <c r="M72" s="6" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="N72" s="6" t="n">
         <v>7</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="A1:M1"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>